<commit_message>
Update model outputs 2026-06-09 21:21:49
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -86,64 +86,103 @@
     <t xml:space="preserve">rain_total_adj</t>
   </si>
   <si>
+    <t xml:space="preserve">19:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">western bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marvel Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interstate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GMHBA Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SameCityDiffGround</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">west coast eagles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optus Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neutral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adelaide Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ninja Stadium</t>
+  </si>
+  <si>
     <t xml:space="preserve">15:15</t>
   </si>
   <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
     <t xml:space="preserve">st kilda</t>
   </si>
   <si>
-    <t xml:space="preserve">SCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Rain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Interstate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather Adjusted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neutral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SameCitySameGround</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marvel Stadium</t>
+    <t xml:space="preserve">greater western sydney</t>
   </si>
 </sst>
 </file>
@@ -482,7 +521,7 @@
     <col min="1" max="1" width="5.7099999026863" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="5.7099999026863" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="16.7099996885961" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="14.7099997275216" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="22.7099995718197" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="16.7099996885961" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="14.7099997275216" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="13.7099997469844" hidden="0" customWidth="1"/>
@@ -581,7 +620,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>24</v>
@@ -604,23 +643,19 @@
       <c r="H2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="3" t="n">
-        <v>-30.5</v>
-      </c>
-      <c r="J2" s="3" t="n">
-        <v>185.5</v>
-      </c>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
       <c r="K2" s="3" t="n">
-        <v>-31.8</v>
+        <v>-9.82</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>182.64</v>
+        <v>182.04</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>25.42</v>
+        <v>4.05</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>173.51</v>
+        <v>174.17</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>30</v>
@@ -629,25 +664,25 @@
         <v>5.3</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>-6.37</v>
+        <v>3.81</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>-5.75</v>
+        <v>-4.79</v>
       </c>
       <c r="T2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U2" s="3" t="n">
-        <v>2.13</v>
+        <v>-1.42</v>
       </c>
       <c r="V2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W2" s="3" t="n">
-        <v>9.14</v>
+        <v>7.87</v>
       </c>
       <c r="X2" s="3" t="n">
         <v>0</v>
@@ -655,7 +690,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46180</v>
+        <v>46184</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>24</v>
@@ -667,7 +702,7 @@
         <v>26</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.57</v>
+        <v>0</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>27</v>
@@ -678,23 +713,19 @@
       <c r="H3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I3" s="3" t="n">
-        <v>-30.5</v>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>185.5</v>
-      </c>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
       <c r="K3" s="3" t="n">
-        <v>-31.86</v>
+        <v>-9.82</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>182.15</v>
+        <v>182.04</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>25.42</v>
+        <v>4.05</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>173.51</v>
+        <v>174.17</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>30</v>
@@ -703,33 +734,33 @@
         <v>5.3</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>-6.37</v>
+        <v>3.81</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S3" s="3" t="n">
-        <v>-5.75</v>
+        <v>-4.79</v>
       </c>
       <c r="T3" s="3" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="U3" s="3" t="n">
-        <v>2.13</v>
+        <v>-1.42</v>
       </c>
       <c r="V3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W3" s="3" t="n">
-        <v>9.14</v>
+        <v>7.87</v>
       </c>
       <c r="X3" s="3" t="n">
-        <v>-0.49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46180</v>
+        <v>46185</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>32</v>
@@ -752,50 +783,46 @@
       <c r="H4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I4" s="3" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>172.5</v>
-      </c>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
       <c r="K4" s="3" t="n">
-        <v>24.08</v>
+        <v>-24.18</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>176.97</v>
+        <v>189.83</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>-20.42</v>
+        <v>16.33</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>167.84</v>
+        <v>181.96</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>-12.56</v>
+        <v>4.42</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>-5.75</v>
+        <v>-4.79</v>
       </c>
       <c r="T4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>1.86</v>
+        <v>13.95</v>
       </c>
       <c r="V4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W4" s="3" t="n">
-        <v>9.14</v>
+        <v>7.87</v>
       </c>
       <c r="X4" s="3" t="n">
         <v>0</v>
@@ -803,7 +830,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46180</v>
+        <v>46185</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>32</v>
@@ -815,7 +842,7 @@
         <v>34</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>35</v>
@@ -826,61 +853,57 @@
       <c r="H5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I5" s="3" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>172.5</v>
-      </c>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
       <c r="K5" s="3" t="n">
-        <v>24.07</v>
+        <v>-24.18</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>176.89</v>
+        <v>189.83</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>-20.42</v>
+        <v>16.33</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>167.84</v>
+        <v>181.96</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>-12.56</v>
+        <v>4.42</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>-5.75</v>
+        <v>-4.79</v>
       </c>
       <c r="T5" s="3" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="U5" s="3" t="n">
-        <v>1.86</v>
+        <v>13.95</v>
       </c>
       <c r="V5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W5" s="3" t="n">
-        <v>9.14</v>
+        <v>7.87</v>
       </c>
       <c r="X5" s="3" t="n">
-        <v>-0.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46181</v>
+        <v>46186</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>37</v>
@@ -892,7 +915,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>28</v>
@@ -900,50 +923,46 @@
       <c r="H6" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>180.5</v>
-      </c>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
       <c r="K6" s="3" t="n">
-        <v>-14.25</v>
+        <v>-29.22</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>178.98</v>
+        <v>184.92</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>8.5</v>
+        <v>27.68</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>169.85</v>
+        <v>177.04</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>0.92</v>
+        <v>-7.6</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>-5.75</v>
+        <v>-4.79</v>
       </c>
       <c r="T6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>-2.12</v>
+        <v>1.11</v>
       </c>
       <c r="V6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W6" s="3" t="n">
-        <v>9.14</v>
+        <v>7.87</v>
       </c>
       <c r="X6" s="3" t="n">
         <v>0</v>
@@ -951,10 +970,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46181</v>
+        <v>46186</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>37</v>
@@ -966,7 +985,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>28</v>
@@ -974,50 +993,46 @@
       <c r="H7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I7" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J7" s="3" t="n">
-        <v>180.5</v>
-      </c>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
       <c r="K7" s="3" t="n">
-        <v>-14.25</v>
+        <v>-29.22</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>178.98</v>
+        <v>184.92</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>8.5</v>
+        <v>27.68</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>169.85</v>
+        <v>177.04</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>0.92</v>
+        <v>-7.6</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>-5.75</v>
+        <v>-4.79</v>
       </c>
       <c r="T7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U7" s="3" t="n">
-        <v>-2.12</v>
+        <v>1.11</v>
       </c>
       <c r="V7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W7" s="3" t="n">
-        <v>9.14</v>
+        <v>7.87</v>
       </c>
       <c r="X7" s="3" t="n">
         <v>0</v>
@@ -1025,22 +1040,22 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46184</v>
+        <v>46186</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>28</v>
@@ -1051,43 +1066,43 @@
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3" t="n">
-        <v>-4.43</v>
+        <v>-16.36</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>185.02</v>
+        <v>191.16</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>3.8</v>
+        <v>11.29</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>175.88</v>
+        <v>183.29</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>5.3</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>-11.63</v>
+        <v>0.21</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S8" s="3" t="n">
-        <v>-5.75</v>
+        <v>-4.79</v>
       </c>
       <c r="T8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U8" s="3" t="n">
-        <v>4.13</v>
+        <v>9.13</v>
       </c>
       <c r="V8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W8" s="3" t="n">
-        <v>9.14</v>
+        <v>7.87</v>
       </c>
       <c r="X8" s="3" t="n">
         <v>0</v>
@@ -1095,22 +1110,22 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46184</v>
+        <v>46186</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>28</v>
@@ -1121,45 +1136,465 @@
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3" t="n">
-        <v>-4.43</v>
+        <v>-16.36</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>185.02</v>
+        <v>191.16</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>3.8</v>
+        <v>11.29</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>175.88</v>
+        <v>183.29</v>
       </c>
       <c r="O9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="3" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="R9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="3" t="n">
+        <v>-4.79</v>
+      </c>
+      <c r="T9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="3" t="n">
+        <v>9.13</v>
+      </c>
+      <c r="V9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="3" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="X9" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>177.69</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>-16.83</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>169.82</v>
+      </c>
+      <c r="O10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="P9" s="3" t="n">
+      <c r="P10" s="3" t="n">
         <v>5.3</v>
       </c>
-      <c r="Q9" s="3" t="n">
-        <v>-11.63</v>
-      </c>
-      <c r="R9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" s="3" t="n">
-        <v>-5.75</v>
-      </c>
-      <c r="T9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U9" s="3" t="n">
-        <v>4.13</v>
-      </c>
-      <c r="V9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W9" s="3" t="n">
-        <v>9.14</v>
-      </c>
-      <c r="X9" s="3" t="n">
+      <c r="Q10" s="3" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="3" t="n">
+        <v>-4.79</v>
+      </c>
+      <c r="T10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="3" t="n">
+        <v>-0.97</v>
+      </c>
+      <c r="V10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" s="3" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="X10" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>177.69</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>-16.83</v>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>169.82</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="3" t="n">
+        <v>-4.79</v>
+      </c>
+      <c r="T11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="3" t="n">
+        <v>-0.97</v>
+      </c>
+      <c r="V11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" s="3" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="X11" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>183.57</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>-42.33</v>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>175.69</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="P12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="3" t="n">
+        <v>-2.33</v>
+      </c>
+      <c r="R12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="3" t="n">
+        <v>-4.79</v>
+      </c>
+      <c r="T12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="3" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="V12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" s="3" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="X12" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>183.57</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>-42.33</v>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>175.69</v>
+      </c>
+      <c r="O13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="P13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="3" t="n">
+        <v>-2.33</v>
+      </c>
+      <c r="R13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="3" t="n">
+        <v>-4.79</v>
+      </c>
+      <c r="T13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="3" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="V13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" s="3" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="X13" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>183.74</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>-3.14</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>175.86</v>
+      </c>
+      <c r="O14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P14" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="Q14" s="3" t="n">
+        <v>-4.71</v>
+      </c>
+      <c r="R14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="3" t="n">
+        <v>-4.79</v>
+      </c>
+      <c r="T14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="3" t="n">
+        <v>-2.69</v>
+      </c>
+      <c r="V14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" s="3" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="X14" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>183.74</v>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>-3.14</v>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>175.86</v>
+      </c>
+      <c r="O15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P15" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="Q15" s="3" t="n">
+        <v>-4.71</v>
+      </c>
+      <c r="R15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="3" t="n">
+        <v>-4.79</v>
+      </c>
+      <c r="T15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="3" t="n">
+        <v>-2.69</v>
+      </c>
+      <c r="V15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" s="3" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="X15" s="3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-06-10 21:00:43
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -643,8 +643,12 @@
       <c r="H2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
+      <c r="I2" s="3" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>180.5</v>
+      </c>
       <c r="K2" s="3" t="n">
         <v>-9.82</v>
       </c>
@@ -713,8 +717,12 @@
       <c r="H3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
+      <c r="I3" s="3" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>180.5</v>
+      </c>
       <c r="K3" s="3" t="n">
         <v>-9.82</v>
       </c>
@@ -783,8 +791,12 @@
       <c r="H4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="I4" s="3" t="n">
+        <v>-24.5</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>178.5</v>
+      </c>
       <c r="K4" s="3" t="n">
         <v>-24.18</v>
       </c>
@@ -853,8 +865,12 @@
       <c r="H5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
+      <c r="I5" s="3" t="n">
+        <v>-24.5</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>178.5</v>
+      </c>
       <c r="K5" s="3" t="n">
         <v>-24.18</v>
       </c>
@@ -923,8 +939,12 @@
       <c r="H6" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
+      <c r="I6" s="3" t="n">
+        <v>-29.5</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>163.5</v>
+      </c>
       <c r="K6" s="3" t="n">
         <v>-29.22</v>
       </c>
@@ -982,7 +1002,7 @@
         <v>38</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>39</v>
@@ -993,13 +1013,17 @@
       <c r="H7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
+      <c r="I7" s="3" t="n">
+        <v>-29.5</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>163.5</v>
+      </c>
       <c r="K7" s="3" t="n">
-        <v>-29.22</v>
+        <v>-29.67</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>184.92</v>
+        <v>181.62</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>27.68</v>
@@ -1023,7 +1047,7 @@
         <v>-4.79</v>
       </c>
       <c r="T7" s="3" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="U7" s="3" t="n">
         <v>1.11</v>
@@ -1035,7 +1059,7 @@
         <v>7.87</v>
       </c>
       <c r="X7" s="3" t="n">
-        <v>0</v>
+        <v>-3.3</v>
       </c>
     </row>
     <row r="8">
@@ -1063,8 +1087,12 @@
       <c r="H8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
+      <c r="I8" s="3" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>165.5</v>
+      </c>
       <c r="K8" s="3" t="n">
         <v>-16.36</v>
       </c>
@@ -1122,7 +1150,7 @@
         <v>43</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>44</v>
@@ -1133,13 +1161,17 @@
       <c r="H9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
+      <c r="I9" s="3" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>165.5</v>
+      </c>
       <c r="K9" s="3" t="n">
-        <v>-16.36</v>
+        <v>-16.49</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>191.16</v>
+        <v>190.21</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>11.29</v>
@@ -1163,7 +1195,7 @@
         <v>-4.79</v>
       </c>
       <c r="T9" s="3" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="U9" s="3" t="n">
         <v>9.13</v>
@@ -1175,7 +1207,7 @@
         <v>7.87</v>
       </c>
       <c r="X9" s="3" t="n">
-        <v>0</v>
+        <v>-0.95</v>
       </c>
     </row>
     <row r="10">
@@ -1203,8 +1235,12 @@
       <c r="H10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
+      <c r="I10" s="3" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>165.5</v>
+      </c>
       <c r="K10" s="3" t="n">
         <v>9.92</v>
       </c>
@@ -1262,7 +1298,7 @@
         <v>48</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0</v>
+        <v>7.98</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>49</v>
@@ -1273,13 +1309,17 @@
       <c r="H11" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
+      <c r="I11" s="3" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>165.5</v>
+      </c>
       <c r="K11" s="3" t="n">
-        <v>9.92</v>
+        <v>8.98</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>177.69</v>
+        <v>170.77</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>-16.83</v>
@@ -1303,7 +1343,7 @@
         <v>-4.79</v>
       </c>
       <c r="T11" s="3" t="n">
-        <v>0</v>
+        <v>0.94</v>
       </c>
       <c r="U11" s="3" t="n">
         <v>-0.97</v>
@@ -1315,7 +1355,7 @@
         <v>7.87</v>
       </c>
       <c r="X11" s="3" t="n">
-        <v>0</v>
+        <v>-6.92</v>
       </c>
     </row>
     <row r="12">
@@ -1343,8 +1383,12 @@
       <c r="H12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
+      <c r="I12" s="3" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>180.5</v>
+      </c>
       <c r="K12" s="3" t="n">
         <v>41.67</v>
       </c>
@@ -1413,8 +1457,12 @@
       <c r="H13" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
+      <c r="I13" s="3" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>180.5</v>
+      </c>
       <c r="K13" s="3" t="n">
         <v>41.67</v>
       </c>
@@ -1483,8 +1531,12 @@
       <c r="H14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
+      <c r="I14" s="3" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>183.5</v>
+      </c>
       <c r="K14" s="3" t="n">
         <v>2.4</v>
       </c>
@@ -1553,8 +1605,12 @@
       <c r="H15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
+      <c r="I15" s="3" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>183.5</v>
+      </c>
       <c r="K15" s="3" t="n">
         <v>2.4</v>
       </c>

</xml_diff>

<commit_message>
Update model outputs 2026-06-14 14:31:48
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t xml:space="preserve">match_id</t>
   </si>
@@ -147,18 +147,6 @@
   </si>
   <si>
     <t xml:space="preserve">Adelaide Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8158</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GMHBA Stadium</t>
   </si>
   <si>
     <t xml:space="preserve">8159</t>
@@ -1150,7 +1138,7 @@
         <v>45</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46185.8194444444</v>
+        <v>46187.5486111111</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>46</v>
@@ -1162,10 +1150,10 @@
         <v>48</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-24.5</v>
+        <v>44.5</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>178.5</v>
+        <v>180.5</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>32</v>
@@ -1174,22 +1162,22 @@
         <v>33</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>-29.9196469288881</v>
+        <v>49.1684920047241</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>196.648734890519</v>
+        <v>175.811951858388</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>5.3</v>
+        <v>0</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>2.20965616457988</v>
+        <v>-3.208535792235</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>11.3964591020741</v>
+        <v>-1.15557392553532</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>183.447627881306</v>
+        <v>162.610844849175</v>
       </c>
       <c r="P8" s="2" t="n">
         <v>170.092592592593</v>
@@ -1207,10 +1195,10 @@
         <v>11.0828460038987</v>
       </c>
       <c r="U8" s="2" t="n">
-        <v>-26.9361928485913</v>
+        <v>52.1519460850209</v>
       </c>
       <c r="V8" s="2" t="n">
-        <v>194.530473885205</v>
+        <v>173.693690853074</v>
       </c>
       <c r="W8" s="2" t="n">
         <v>-2.98345408029678</v>
@@ -1236,7 +1224,7 @@
         <v>45</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>46185.8194444444</v>
+        <v>46187.5486111111</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>46</v>
@@ -1248,10 +1236,10 @@
         <v>48</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-24.5</v>
+        <v>44.5</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>178.5</v>
+        <v>180.5</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>32</v>
@@ -1260,22 +1248,22 @@
         <v>36</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>-29.9196469288881</v>
+        <v>49.1684920047241</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>196.648734890519</v>
+        <v>175.811951858388</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>5.3</v>
+        <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>2.20965616457988</v>
+        <v>-3.208535792235</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>11.3964591020741</v>
+        <v>-1.15557392553532</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>183.447627881306</v>
+        <v>162.610844849175</v>
       </c>
       <c r="P9" s="2" t="n">
         <v>170.092592592593</v>
@@ -1293,10 +1281,10 @@
         <v>11.0828460038987</v>
       </c>
       <c r="U9" s="2" t="n">
-        <v>-26.9361928485913</v>
+        <v>52.1519460850209</v>
       </c>
       <c r="V9" s="2" t="n">
-        <v>194.530473885205</v>
+        <v>173.693690853074</v>
       </c>
       <c r="W9" s="2" t="n">
         <v>-2.98345408029678</v>
@@ -1322,7 +1310,7 @@
         <v>49</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>46187.5486111111</v>
+        <v>46187.6354166667</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>50</v>
@@ -1334,10 +1322,10 @@
         <v>52</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>44.5</v>
+        <v>-3.5</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>180.5</v>
+        <v>183.5</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>32</v>
@@ -1346,22 +1334,22 @@
         <v>33</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>49.1684920047241</v>
+        <v>13.7788535449639</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>175.811951858388</v>
+        <v>184.855020654059</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>-3.208535792235</v>
+        <v>-6.32898274776335</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>-1.15557392553532</v>
+        <v>0.774206135844196</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>162.610844849175</v>
+        <v>171.653913644846</v>
       </c>
       <c r="P10" s="2" t="n">
         <v>170.092592592593</v>
@@ -1379,10 +1367,10 @@
         <v>11.0828460038987</v>
       </c>
       <c r="U10" s="2" t="n">
-        <v>52.1519460850209</v>
+        <v>16.7623076252607</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>173.693690853074</v>
+        <v>182.736759648745</v>
       </c>
       <c r="W10" s="2" t="n">
         <v>-2.98345408029678</v>
@@ -1408,7 +1396,7 @@
         <v>49</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>46187.5486111111</v>
+        <v>46187.6354166667</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>50</v>
@@ -1420,10 +1408,10 @@
         <v>52</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>44.5</v>
+        <v>-3.5</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>180.5</v>
+        <v>183.5</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>32</v>
@@ -1432,22 +1420,22 @@
         <v>36</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>49.1684920047241</v>
+        <v>13.7788535449639</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>175.811951858388</v>
+        <v>184.855020654059</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>-3.208535792235</v>
+        <v>-6.32898274776335</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-1.15557392553532</v>
+        <v>0.774206135844196</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>162.610844849175</v>
+        <v>171.653913644846</v>
       </c>
       <c r="P11" s="2" t="n">
         <v>170.092592592593</v>
@@ -1465,10 +1453,10 @@
         <v>11.0828460038987</v>
       </c>
       <c r="U11" s="2" t="n">
-        <v>52.1519460850209</v>
+        <v>16.7623076252607</v>
       </c>
       <c r="V11" s="2" t="n">
-        <v>173.693690853074</v>
+        <v>182.736759648745</v>
       </c>
       <c r="W11" s="2" t="n">
         <v>-2.98345408029678</v>
@@ -1486,178 +1474,6 @@
         <v>34</v>
       </c>
       <c r="AB11" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>46187.6354166667</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>183.5</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v>13.7788535449639</v>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>184.855020654059</v>
-      </c>
-      <c r="L12" s="2" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>-6.32898274776335</v>
-      </c>
-      <c r="N12" s="2" t="n">
-        <v>0.774206135844196</v>
-      </c>
-      <c r="O12" s="2" t="n">
-        <v>171.653913644846</v>
-      </c>
-      <c r="P12" s="2" t="n">
-        <v>170.092592592593</v>
-      </c>
-      <c r="Q12" s="2" t="n">
-        <v>181.175438596491</v>
-      </c>
-      <c r="R12" s="2" t="n">
-        <v>114</v>
-      </c>
-      <c r="S12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" s="2" t="n">
-        <v>11.0828460038987</v>
-      </c>
-      <c r="U12" s="2" t="n">
-        <v>16.7623076252607</v>
-      </c>
-      <c r="V12" s="2" t="n">
-        <v>182.736759648745</v>
-      </c>
-      <c r="W12" s="2" t="n">
-        <v>-2.98345408029678</v>
-      </c>
-      <c r="X12" s="2" t="n">
-        <v>2.11826100531454</v>
-      </c>
-      <c r="Y12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z12" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA12" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AB12" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>46187.6354166667</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>183.5</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>13.7788535449639</v>
-      </c>
-      <c r="K13" s="2" t="n">
-        <v>184.855020654059</v>
-      </c>
-      <c r="L13" s="2" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>-6.32898274776335</v>
-      </c>
-      <c r="N13" s="2" t="n">
-        <v>0.774206135844196</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>171.653913644846</v>
-      </c>
-      <c r="P13" s="2" t="n">
-        <v>170.092592592593</v>
-      </c>
-      <c r="Q13" s="2" t="n">
-        <v>181.175438596491</v>
-      </c>
-      <c r="R13" s="2" t="n">
-        <v>114</v>
-      </c>
-      <c r="S13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T13" s="2" t="n">
-        <v>11.0828460038987</v>
-      </c>
-      <c r="U13" s="2" t="n">
-        <v>16.7623076252607</v>
-      </c>
-      <c r="V13" s="2" t="n">
-        <v>182.736759648745</v>
-      </c>
-      <c r="W13" s="2" t="n">
-        <v>-2.98345408029678</v>
-      </c>
-      <c r="X13" s="2" t="n">
-        <v>2.11826100531454</v>
-      </c>
-      <c r="Y13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z13" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AB13" s="2" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-06-20 11:02:58
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t xml:space="preserve">match_id</t>
   </si>
@@ -98,67 +98,130 @@
     <t xml:space="preserve">gate_reason</t>
   </si>
   <si>
-    <t xml:space="preserve">8160</t>
+    <t xml:space="preserve">8161</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hawthorn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People First Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">currentpar_plus_ssm_anchor_overlay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">none</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8162</t>
+  </si>
+  <si>
+    <t xml:space="preserve">greater western sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENGIE Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8163</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collingwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8164</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adelaide Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8165</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8166</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">western bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marvel Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8167</t>
+  </si>
+  <si>
+    <t xml:space="preserve">west coast eagles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8168</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gabba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8169</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8171</t>
   </si>
   <si>
     <t xml:space="preserve">fremantle</t>
   </si>
   <si>
-    <t xml:space="preserve">geelong cats</t>
-  </si>
-  <si>
     <t xml:space="preserve">Optus Stadium</t>
   </si>
   <si>
-    <t xml:space="preserve">currentpar_plus_ssm_anchor_overlay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Rain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">none</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather Adjusted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8161</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People First Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8162</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENGIE Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8164</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adelaide Oval</t>
+    <t xml:space="preserve">8172</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8174</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8179</t>
   </si>
 </sst>
 </file>
@@ -492,7 +555,7 @@
     <col min="1" max="1" width="8.70999984429807" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="16.7099996885961" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="22.7099995718197" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="12.7099997664471" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="22.7099995718197" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="20.7099996107452" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="8.70999984429807" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="9.70999982483533" hidden="0" customWidth="1"/>
@@ -610,7 +673,7 @@
         <v>28</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46191.7569444444</v>
+        <v>46192.8194444444</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>29</v>
@@ -622,10 +685,10 @@
         <v>31</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-13.5</v>
+        <v>3.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>174.5</v>
+        <v>183.5</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>32</v>
@@ -634,49 +697,49 @@
         <v>33</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>7.29001852759259</v>
+        <v>2.60988018208875</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>195.167957645186</v>
+        <v>187.84211661561</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>10.5</v>
+        <v>5.3</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0.435903126798202</v>
+        <v>-2.16343632766445</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>8.56503532967531</v>
+        <v>11.6320895566329</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>181.966850635973</v>
+        <v>175.397969781431</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>170.092592592593</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>181.175438596491</v>
+        <v>180.888429752066</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>11.0828460038987</v>
+        <v>10.7958371594735</v>
       </c>
       <c r="U2" s="2" t="n">
-        <v>10.2734726078894</v>
+        <v>5.35455592652194</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>193.049696639872</v>
+        <v>186.193806940905</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>-2.98345408029678</v>
+        <v>-2.74467574443319</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>2.11826100531454</v>
+        <v>1.64830967470505</v>
       </c>
       <c r="Y2" s="2" t="b">
         <v>1</v>
@@ -696,7 +759,7 @@
         <v>28</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46191.7569444444</v>
+        <v>46192.8194444444</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>29</v>
@@ -708,10 +771,10 @@
         <v>31</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-13.5</v>
+        <v>3.5</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>174.5</v>
+        <v>183.5</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>32</v>
@@ -720,49 +783,49 @@
         <v>36</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>7.29001852759259</v>
+        <v>2.60988018208875</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>195.167957645186</v>
+        <v>187.84211661561</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>10.5</v>
+        <v>5.3</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>0.435903126798202</v>
+        <v>-2.16343632766445</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>8.56503532967531</v>
+        <v>11.6320895566329</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>181.966850635973</v>
+        <v>175.397969781431</v>
       </c>
       <c r="P3" s="2" t="n">
         <v>170.092592592593</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>181.175438596491</v>
+        <v>180.888429752066</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="S3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T3" s="2" t="n">
-        <v>11.0828460038987</v>
+        <v>10.7958371594735</v>
       </c>
       <c r="U3" s="2" t="n">
-        <v>10.2734726078894</v>
+        <v>5.35455592652194</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>193.049696639872</v>
+        <v>186.193806940905</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-2.98345408029678</v>
+        <v>-2.74467574443319</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>2.11826100531454</v>
+        <v>1.64830967470505</v>
       </c>
       <c r="Y3" s="2" t="b">
         <v>1</v>
@@ -782,7 +845,7 @@
         <v>37</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46192.8194444444</v>
+        <v>46193.6770833333</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>38</v>
@@ -794,10 +857,10 @@
         <v>40</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>3.5</v>
+        <v>-15.5</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>183.5</v>
+        <v>186.5</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>32</v>
@@ -806,49 +869,49 @@
         <v>33</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>2.29371611060022</v>
+        <v>-35.1986683494074</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>189.116404493941</v>
+        <v>179.442608625445</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>5.3</v>
+        <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>-7.17746763928998</v>
+        <v>3.28998994021156</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>11.1881191775315</v>
+        <v>3.95953087825907</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>175.915297484728</v>
+        <v>166.998461791267</v>
       </c>
       <c r="P4" s="2" t="n">
         <v>170.092592592593</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>181.175438596491</v>
+        <v>180.888429752066</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T4" s="2" t="n">
-        <v>11.0828460038987</v>
+        <v>10.7958371594735</v>
       </c>
       <c r="U4" s="2" t="n">
-        <v>5.277170190897</v>
+        <v>-32.4539926049742</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>186.998143488627</v>
+        <v>177.79429895074</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-2.98345408029678</v>
+        <v>-2.74467574443319</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>2.11826100531454</v>
+        <v>1.64830967470505</v>
       </c>
       <c r="Y4" s="2" t="b">
         <v>1</v>
@@ -868,7 +931,7 @@
         <v>37</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46192.8194444444</v>
+        <v>46193.6770833333</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>38</v>
@@ -880,10 +943,10 @@
         <v>40</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>3.5</v>
+        <v>-15.5</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>183.5</v>
+        <v>186.5</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>32</v>
@@ -892,49 +955,49 @@
         <v>36</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>2.29371611060022</v>
+        <v>-35.1986683494074</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>189.116404493941</v>
+        <v>179.442608625445</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>5.3</v>
+        <v>0</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>-7.17746763928998</v>
+        <v>3.28998994021156</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>11.1881191775315</v>
+        <v>3.95953087825907</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>175.915297484728</v>
+        <v>166.998461791267</v>
       </c>
       <c r="P5" s="2" t="n">
         <v>170.092592592593</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>181.175438596491</v>
+        <v>180.888429752066</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="S5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>11.0828460038987</v>
+        <v>10.7958371594735</v>
       </c>
       <c r="U5" s="2" t="n">
-        <v>5.277170190897</v>
+        <v>-32.4539926049742</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>186.998143488627</v>
+        <v>177.79429895074</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>-2.98345408029678</v>
+        <v>-2.74467574443319</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>2.11826100531454</v>
+        <v>1.64830967470505</v>
       </c>
       <c r="Y5" s="2" t="b">
         <v>1</v>
@@ -954,7 +1017,7 @@
         <v>41</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46193.6770833333</v>
+        <v>46193.8159722222</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>42</v>
@@ -966,10 +1029,10 @@
         <v>44</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-15.5</v>
+        <v>-13.5</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>186.5</v>
+        <v>162.5</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>32</v>
@@ -978,49 +1041,49 @@
         <v>33</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>-34.7951449878185</v>
+        <v>-40.8964839597481</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>180.461618110719</v>
+        <v>179.839527083544</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>1.84141863787485</v>
+        <v>-4.57832925276927</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.851144943866416</v>
+        <v>4.26089144560802</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>167.260511101505</v>
+        <v>167.395380249365</v>
       </c>
       <c r="P6" s="2" t="n">
         <v>170.092592592593</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>181.175438596491</v>
+        <v>180.888429752066</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T6" s="2" t="n">
-        <v>11.0828460038987</v>
+        <v>10.7958371594735</v>
       </c>
       <c r="U6" s="2" t="n">
-        <v>-31.8116909075217</v>
+        <v>-38.1518082153149</v>
       </c>
       <c r="V6" s="2" t="n">
-        <v>178.343357105404</v>
+        <v>178.191217408838</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>-2.98345408029678</v>
+        <v>-2.74467574443319</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>2.11826100531454</v>
+        <v>1.64830967470505</v>
       </c>
       <c r="Y6" s="2" t="b">
         <v>1</v>
@@ -1040,7 +1103,7 @@
         <v>41</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46193.6770833333</v>
+        <v>46193.8159722222</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>42</v>
@@ -1052,10 +1115,10 @@
         <v>44</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-15.5</v>
+        <v>-13.5</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>186.5</v>
+        <v>162.5</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>32</v>
@@ -1064,49 +1127,49 @@
         <v>36</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>-34.7951449878185</v>
+        <v>-42.097619228361</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>180.461618110719</v>
+        <v>171.180435696368</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>1.84141863787485</v>
+        <v>-4.57832925276927</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.851144943866416</v>
+        <v>4.26089144560802</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>167.260511101505</v>
+        <v>167.395380249365</v>
       </c>
       <c r="P7" s="2" t="n">
         <v>170.092592592593</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>181.175438596491</v>
+        <v>180.888429752066</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="S7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T7" s="2" t="n">
-        <v>11.0828460038987</v>
+        <v>10.7958371594735</v>
       </c>
       <c r="U7" s="2" t="n">
-        <v>-31.8116909075217</v>
+        <v>-39.3529434839278</v>
       </c>
       <c r="V7" s="2" t="n">
-        <v>178.343357105404</v>
+        <v>169.532126021663</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>-2.98345408029678</v>
+        <v>-2.74467574443319</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>2.11826100531454</v>
+        <v>1.64830967470505</v>
       </c>
       <c r="Y7" s="2" t="b">
         <v>1</v>
@@ -1150,49 +1213,49 @@
         <v>33</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>-12.8489788859035</v>
+        <v>-18.6499224628315</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>184.54929064637</v>
+        <v>184.96606065125</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>5.3</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>13.4766955129781</v>
+        <v>27.5779354340673</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.0282377066911863</v>
+        <v>2.71872947941213</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>171.348183637157</v>
+        <v>172.521913817071</v>
       </c>
       <c r="P8" s="2" t="n">
         <v>170.092592592593</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>181.175438596491</v>
+        <v>180.888429752066</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T8" s="2" t="n">
-        <v>11.0828460038987</v>
+        <v>10.7958371594735</v>
       </c>
       <c r="U8" s="2" t="n">
-        <v>-9.86552480560674</v>
+        <v>-15.9052467183983</v>
       </c>
       <c r="V8" s="2" t="n">
-        <v>182.431029641056</v>
+        <v>183.317750976545</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>-2.98345408029678</v>
+        <v>-2.74467574443319</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>2.11826100531454</v>
+        <v>1.64830967470505</v>
       </c>
       <c r="Y8" s="2" t="b">
         <v>1</v>
@@ -1236,49 +1299,49 @@
         <v>36</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>-12.8788652762867</v>
+        <v>-18.6806445695369</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>184.32429239832</v>
+        <v>184.744582241182</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>5.3</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>13.4766955129781</v>
+        <v>27.5779354340673</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.0282377066911863</v>
+        <v>2.71872947941213</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>171.348183637157</v>
+        <v>172.521913817071</v>
       </c>
       <c r="P9" s="2" t="n">
         <v>170.092592592593</v>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>181.175438596491</v>
+        <v>180.888429752066</v>
       </c>
       <c r="R9" s="2" t="n">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="S9" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T9" s="2" t="n">
-        <v>11.0828460038987</v>
+        <v>10.7958371594735</v>
       </c>
       <c r="U9" s="2" t="n">
-        <v>-9.89541119598991</v>
+        <v>-15.9359688251037</v>
       </c>
       <c r="V9" s="2" t="n">
-        <v>182.206031393006</v>
+        <v>183.096272566477</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>-2.98345408029678</v>
+        <v>-2.74467574443319</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>2.11826100531454</v>
+        <v>1.64830967470505</v>
       </c>
       <c r="Y9" s="2" t="b">
         <v>1</v>
@@ -1290,6 +1353,1498 @@
         <v>34</v>
       </c>
       <c r="AB9" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>46194.5486111111</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>175.5</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>6.2697041959618</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>160.319349992236</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>-19.1993792143622</v>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>5.1240647366032</v>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>147.875203158057</v>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R10" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T10" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U10" s="2" t="n">
+        <v>9.01437994039498</v>
+      </c>
+      <c r="V10" s="2" t="n">
+        <v>158.671040317531</v>
+      </c>
+      <c r="W10" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X10" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z10" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB10" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>46194.5486111111</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>175.5</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>6.22609862515407</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>160.004993539236</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>-19.1993792143622</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>5.1240647366032</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>147.875203158057</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>8.97077436958726</v>
+      </c>
+      <c r="V11" s="2" t="n">
+        <v>158.356683864531</v>
+      </c>
+      <c r="W11" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X11" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB11" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>46194.6354166667</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>183.5</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>22.3528030626646</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>190.209295605875</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>17.7828000269583</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>-0.0695770530873006</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>177.765148771696</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>25.0974788070978</v>
+      </c>
+      <c r="V12" s="2" t="n">
+        <v>188.56098593117</v>
+      </c>
+      <c r="W12" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X12" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB12" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>46194.6354166667</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>183.5</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>22.3528030626646</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>190.209295605875</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>17.7828000269583</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>-0.0695770530873006</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>177.765148771696</v>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U13" s="2" t="n">
+        <v>25.0974788070978</v>
+      </c>
+      <c r="V13" s="2" t="n">
+        <v>188.56098593117</v>
+      </c>
+      <c r="W13" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X13" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z13" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB13" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>-34.6818443427192</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>162.919724266771</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>8.5018643137553</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>5.34615993575184</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>150.475577432592</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>-31.937168598286</v>
+      </c>
+      <c r="V14" s="2" t="n">
+        <v>161.271414592066</v>
+      </c>
+      <c r="W14" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X14" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z14" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB14" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>-34.6818443427192</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>162.919724266771</v>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>8.5018643137553</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>5.34615993575184</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>150.475577432592</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R15" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U15" s="2" t="n">
+        <v>-31.937168598286</v>
+      </c>
+      <c r="V15" s="2" t="n">
+        <v>161.271414592066</v>
+      </c>
+      <c r="W15" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X15" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB15" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>-17.3693977274073</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>191.245757893949</v>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>8.48046940678483</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>-4.27445438652347</v>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>178.80161105977</v>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q16" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R16" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U16" s="2" t="n">
+        <v>-14.6247219829741</v>
+      </c>
+      <c r="V16" s="2" t="n">
+        <v>189.597448219244</v>
+      </c>
+      <c r="W16" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X16" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB16" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>-17.4011108698129</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>191.01713501904</v>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>8.48046940678483</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>-4.27445438652347</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>178.80161105977</v>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T17" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U17" s="2" t="n">
+        <v>-14.6564351253797</v>
+      </c>
+      <c r="V17" s="2" t="n">
+        <v>189.368825344335</v>
+      </c>
+      <c r="W17" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X17" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z17" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB17" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>-14.1822009530384</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>161.12936041668</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>9.57586564484396</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>10.2430615447799</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>148.685213582502</v>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R18" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U18" s="2" t="n">
+        <v>-11.4375252086052</v>
+      </c>
+      <c r="V18" s="2" t="n">
+        <v>159.481050741975</v>
+      </c>
+      <c r="W18" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X18" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z18" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB18" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>-14.1822009530384</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>161.12936041668</v>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>9.57586564484396</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>10.2430615447799</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>148.685213582502</v>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q19" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R19" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T19" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U19" s="2" t="n">
+        <v>-11.4375252086052</v>
+      </c>
+      <c r="V19" s="2" t="n">
+        <v>159.481050741975</v>
+      </c>
+      <c r="W19" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X19" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z19" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB19" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>-12.8598318181085</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>185.793158116571</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>0.847757042828832</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>12.5848649842145</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>173.349011282392</v>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R20" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T20" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U20" s="2" t="n">
+        <v>-10.1151560736753</v>
+      </c>
+      <c r="V20" s="2" t="n">
+        <v>184.144848441866</v>
+      </c>
+      <c r="W20" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X20" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z20" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB20" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>-13.7398715198644</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>179.448873337848</v>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>0.847757042828832</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>12.5848649842145</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>173.349011282392</v>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R21" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T21" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U21" s="2" t="n">
+        <v>-10.9951957754312</v>
+      </c>
+      <c r="V21" s="2" t="n">
+        <v>177.800563663143</v>
+      </c>
+      <c r="W21" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X21" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z21" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB21" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>-15.8519399231266</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>188.688326525247</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>4.80372068975229</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>5.13370381971959</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>176.244179691068</v>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q22" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R22" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T22" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U22" s="2" t="n">
+        <v>-13.1072641786934</v>
+      </c>
+      <c r="V22" s="2" t="n">
+        <v>187.040016850542</v>
+      </c>
+      <c r="W22" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X22" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z22" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB22" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>-15.8519399231266</v>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>188.688326525247</v>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>4.80372068975229</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>5.13370381971959</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>176.244179691068</v>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R23" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T23" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U23" s="2" t="n">
+        <v>-13.1072641786934</v>
+      </c>
+      <c r="V23" s="2" t="n">
+        <v>187.040016850542</v>
+      </c>
+      <c r="W23" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X23" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z23" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA23" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB23" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>-62.6226675257317</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>173.653008744033</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>4.72800698522382</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>-3.30814541375864</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>161.208861909854</v>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q24" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R24" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T24" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U24" s="2" t="n">
+        <v>-59.8779917812985</v>
+      </c>
+      <c r="V24" s="2" t="n">
+        <v>172.004699069328</v>
+      </c>
+      <c r="W24" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X24" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z24" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB24" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>-62.6226675257317</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>173.653008744033</v>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>4.72800698522382</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>-3.30814541375864</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>161.208861909854</v>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R25" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T25" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U25" s="2" t="n">
+        <v>-59.8779917812985</v>
+      </c>
+      <c r="V25" s="2" t="n">
+        <v>172.004699069328</v>
+      </c>
+      <c r="W25" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X25" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z25" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA25" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB25" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>23.2007058610751</v>
+      </c>
+      <c r="K26" s="2" t="n">
+        <v>177.86313972598</v>
+      </c>
+      <c r="L26" s="2" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>-17.7324666109276</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>12.4189136978695</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>165.418992891802</v>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R26" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T26" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U26" s="2" t="n">
+        <v>25.9453816055083</v>
+      </c>
+      <c r="V26" s="2" t="n">
+        <v>176.214830051275</v>
+      </c>
+      <c r="W26" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X26" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z26" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA26" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB26" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>46195.5</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>23.2007058610751</v>
+      </c>
+      <c r="K27" s="2" t="n">
+        <v>177.86313972598</v>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>-17.7324666109276</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>12.4189136978695</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>165.418992891802</v>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>170.092592592593</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>180.888429752066</v>
+      </c>
+      <c r="R27" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T27" s="2" t="n">
+        <v>10.7958371594735</v>
+      </c>
+      <c r="U27" s="2" t="n">
+        <v>25.9453816055083</v>
+      </c>
+      <c r="V27" s="2" t="n">
+        <v>176.214830051275</v>
+      </c>
+      <c r="W27" s="2" t="n">
+        <v>-2.74467574443319</v>
+      </c>
+      <c r="X27" s="2" t="n">
+        <v>1.64830967470505</v>
+      </c>
+      <c r="Y27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB27" s="2" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-06-30 21:14:31
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -89,100 +89,130 @@
     <t xml:space="preserve">19:30</t>
   </si>
   <si>
+    <t xml:space="preserve">geelong cats</t>
+  </si>
+  <si>
     <t xml:space="preserve">brisbane lions</t>
   </si>
   <si>
+    <t xml:space="preserve">GMHBA Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interstate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">west coast eagles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optus Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:40</t>
+  </si>
+  <si>
     <t xml:space="preserve">sydney swans</t>
   </si>
   <si>
-    <t xml:space="preserve">Gabba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Rain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Interstate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather Adjusted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:40</t>
+    <t xml:space="preserve">western bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:15</t>
   </si>
   <si>
     <t xml:space="preserve">hawthorn</t>
   </si>
   <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UTAS Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neutral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:35</t>
+  </si>
+  <si>
     <t xml:space="preserve">greater western sydney</t>
   </si>
   <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corroboree Group Oval Manuka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collingwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People First Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
     <t xml:space="preserve">MCG</t>
   </si>
   <si>
-    <t xml:space="preserve">13:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">west coast eagles</t>
+    <t xml:space="preserve">SameCitySameGround</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
   </si>
   <si>
     <t xml:space="preserve">Marvel Stadium</t>
   </si>
   <si>
-    <t xml:space="preserve">Neutral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SameCitySameGround</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:05</t>
+    <t xml:space="preserve">16:10</t>
   </si>
   <si>
     <t xml:space="preserve">port adelaide</t>
   </si>
   <si>
-    <t xml:space="preserve">adelaide crows</t>
+    <t xml:space="preserve">north melbourne</t>
   </si>
   <si>
     <t xml:space="preserve">Adelaide Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optus Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
   </si>
 </sst>
 </file>
@@ -520,10 +550,10 @@
   <cols>
     <col min="1" max="1" width="5.7099999026863" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="5.7099999026863" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="15.7099997080589" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="22.7099995718197" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="22.7099995718197" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="16.7099996885961" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="16.7099996885961" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="14.7099997275216" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="28.7099994550433" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="13.7099997469844" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="16.7099996885961" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="17.7099996691334" hidden="0" customWidth="1"/>
@@ -620,7 +650,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46198</v>
+        <v>46205</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>24</v>
@@ -644,22 +674,22 @@
         <v>29</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-1.5</v>
+        <v>-14.5</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>185.5</v>
+        <v>172.5</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-11.13</v>
+        <v>-13.97</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>183.02</v>
+        <v>185.4</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>-0.63</v>
+        <v>12.41</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>186.59</v>
+        <v>189.52</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>30</v>
@@ -668,25 +698,25 @@
         <v>5.3</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>10.02</v>
+        <v>0.27</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U2" s="3" t="n">
-        <v>-3.96</v>
+        <v>8.14</v>
       </c>
       <c r="V2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W2" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X2" s="3" t="n">
         <v>0</v>
@@ -694,7 +724,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46198</v>
+        <v>46205</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>24</v>
@@ -706,7 +736,7 @@
         <v>26</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>27</v>
@@ -718,22 +748,22 @@
         <v>31</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>-1.5</v>
+        <v>-14.5</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>185.5</v>
+        <v>172.5</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>-11.13</v>
+        <v>-14.46</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>183.02</v>
+        <v>182.04</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>-0.63</v>
+        <v>12.41</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>186.59</v>
+        <v>189.52</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>30</v>
@@ -742,33 +772,33 @@
         <v>5.3</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>10.02</v>
+        <v>0.27</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S3" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T3" s="3" t="n">
-        <v>0</v>
+        <v>0.49</v>
       </c>
       <c r="U3" s="3" t="n">
-        <v>-3.96</v>
+        <v>8.14</v>
       </c>
       <c r="V3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W3" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X3" s="3" t="n">
-        <v>0</v>
+        <v>-3.36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46199</v>
+        <v>46206</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>32</v>
@@ -792,49 +822,49 @@
         <v>29</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>-21.5</v>
+        <v>30.5</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>173.5</v>
+        <v>172.5</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>-18.12</v>
+        <v>29.92</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>174.07</v>
+        <v>163.9</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>11.63</v>
+        <v>-31.21</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>177.64</v>
+        <v>168.02</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>5.3</v>
+        <v>10.5</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>6.65</v>
+        <v>-7.83</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>3.03</v>
+        <v>2.21</v>
       </c>
       <c r="V4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W4" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X4" s="3" t="n">
         <v>0</v>
@@ -842,7 +872,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46199</v>
+        <v>46206</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>32</v>
@@ -866,49 +896,49 @@
         <v>31</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-21.5</v>
+        <v>30.5</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>173.5</v>
+        <v>172.5</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>-18.12</v>
+        <v>29.92</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>174.07</v>
+        <v>163.9</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>11.63</v>
+        <v>-31.21</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>177.64</v>
+        <v>168.02</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>5.3</v>
+        <v>10.5</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>6.65</v>
+        <v>-7.83</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U5" s="3" t="n">
-        <v>3.03</v>
+        <v>2.21</v>
       </c>
       <c r="V5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W5" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X5" s="3" t="n">
         <v>0</v>
@@ -916,22 +946,22 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46200</v>
+        <v>46206</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>28</v>
@@ -940,49 +970,49 @@
         <v>29</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-31.5</v>
+        <v>-18.5</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>173.5</v>
+        <v>184.5</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-33.82</v>
+        <v>-10.11</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>162.05</v>
+        <v>179.7</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>27.48</v>
+        <v>12.49</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>165.62</v>
+        <v>183.82</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>6.95</v>
+        <v>-10.42</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>5.83</v>
+        <v>-8.94</v>
       </c>
       <c r="V6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W6" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X6" s="3" t="n">
         <v>0</v>
@@ -990,22 +1020,22 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46200</v>
+        <v>46206</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>28</v>
@@ -1014,57 +1044,57 @@
         <v>31</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>-31.5</v>
+        <v>-18.5</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>173.5</v>
+        <v>184.5</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>-33.82</v>
+        <v>-10.15</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>162.05</v>
+        <v>179.44</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>27.48</v>
+        <v>12.49</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>165.62</v>
+        <v>183.82</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>6.95</v>
+        <v>-10.42</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T7" s="3" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="U7" s="3" t="n">
-        <v>5.83</v>
+        <v>-8.94</v>
       </c>
       <c r="V7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W7" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X7" s="3" t="n">
-        <v>0</v>
+        <v>-0.27</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46200</v>
+        <v>46207</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>41</v>
@@ -1079,7 +1109,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>28</v>
@@ -1088,49 +1118,49 @@
         <v>29</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-36.5</v>
+        <v>-15.5</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>170.5</v>
+        <v>171.5</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>-41.71</v>
+        <v>-16.41</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>153.57</v>
+        <v>173.01</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>40.75</v>
+        <v>9.77</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>157.14</v>
+        <v>177.13</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>-5.75</v>
+        <v>8.17</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S8" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U8" s="3" t="n">
-        <v>-6.48</v>
+        <v>-7.18</v>
       </c>
       <c r="V8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W8" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X8" s="3" t="n">
         <v>0</v>
@@ -1138,7 +1168,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46200</v>
+        <v>46207</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>41</v>
@@ -1153,7 +1183,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>28</v>
@@ -1162,49 +1192,49 @@
         <v>31</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>-36.5</v>
+        <v>-15.5</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>170.5</v>
+        <v>171.5</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>-41.71</v>
+        <v>-16.41</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>153.57</v>
+        <v>173.01</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>40.75</v>
+        <v>9.77</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>157.14</v>
+        <v>177.13</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>-5.75</v>
+        <v>8.17</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S9" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U9" s="3" t="n">
-        <v>-6.48</v>
+        <v>-7.18</v>
       </c>
       <c r="V9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W9" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X9" s="3" t="n">
         <v>0</v>
@@ -1212,22 +1242,22 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46200</v>
+        <v>46207</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>28</v>
@@ -1238,45 +1268,47 @@
       <c r="I10" s="3" t="n">
         <v>20.5</v>
       </c>
-      <c r="J10" s="3"/>
+      <c r="J10" s="3" t="n">
+        <v>178.5</v>
+      </c>
       <c r="K10" s="3" t="n">
-        <v>24.58</v>
+        <v>15.1</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>156.91</v>
+        <v>165.93</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>-14.63</v>
+        <v>-14.6</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>160.48</v>
+        <v>170.04</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>-15.47</v>
+        <v>-6.25</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S10" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U10" s="3" t="n">
-        <v>12.44</v>
+        <v>5.03</v>
       </c>
       <c r="V10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W10" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X10" s="3" t="n">
         <v>0</v>
@@ -1284,22 +1316,22 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46200</v>
+        <v>46207</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>28</v>
@@ -1310,45 +1342,47 @@
       <c r="I11" s="3" t="n">
         <v>20.5</v>
       </c>
-      <c r="J11" s="3"/>
+      <c r="J11" s="3" t="n">
+        <v>178.5</v>
+      </c>
       <c r="K11" s="3" t="n">
-        <v>24.58</v>
+        <v>15.1</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>156.91</v>
+        <v>165.93</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>-14.63</v>
+        <v>-14.6</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>160.48</v>
+        <v>170.04</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>-15.47</v>
+        <v>-6.25</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S11" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U11" s="3" t="n">
-        <v>12.44</v>
+        <v>5.03</v>
       </c>
       <c r="V11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W11" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X11" s="3" t="n">
         <v>0</v>
@@ -1356,22 +1390,22 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46201</v>
+        <v>46207</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>28</v>
@@ -1380,47 +1414,49 @@
         <v>29</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>-27.5</v>
-      </c>
-      <c r="J12" s="3"/>
+        <v>-8.5</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>173.5</v>
+      </c>
       <c r="K12" s="3" t="n">
-        <v>-35.01</v>
+        <v>-9.31</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>167.3</v>
+        <v>159.71</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>22.56</v>
+        <v>2.02</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>170.87</v>
+        <v>163.83</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>10.5</v>
+        <v>5.3</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>11.6</v>
+        <v>5.03</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S12" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U12" s="3" t="n">
-        <v>11.82</v>
+        <v>1.95</v>
       </c>
       <c r="V12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W12" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X12" s="3" t="n">
         <v>0</v>
@@ -1428,22 +1464,22 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46201</v>
+        <v>46207</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>28</v>
@@ -1452,47 +1488,49 @@
         <v>31</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-27.5</v>
-      </c>
-      <c r="J13" s="3"/>
+        <v>-8.5</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>173.5</v>
+      </c>
       <c r="K13" s="3" t="n">
-        <v>-35.01</v>
+        <v>-9.31</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>167.3</v>
+        <v>159.71</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>22.56</v>
+        <v>2.02</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>170.87</v>
+        <v>163.83</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>10.5</v>
+        <v>5.3</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>11.6</v>
+        <v>5.03</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S13" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U13" s="3" t="n">
-        <v>11.82</v>
+        <v>1.95</v>
       </c>
       <c r="V13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W13" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X13" s="3" t="n">
         <v>0</v>
@@ -1500,7 +1538,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46201</v>
+        <v>46207</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>54</v>
@@ -1515,7 +1553,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>28</v>
@@ -1524,47 +1562,49 @@
         <v>29</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-14.5</v>
-      </c>
-      <c r="J14" s="3"/>
+        <v>35.5</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>167.5</v>
+      </c>
       <c r="K14" s="3" t="n">
-        <v>-20.19</v>
+        <v>22.91</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>174.53</v>
+        <v>158.58</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>10.09</v>
+        <v>-28.22</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>178.1</v>
+        <v>162.69</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="P14" s="3" t="n">
         <v>3.2</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>13.39</v>
+        <v>-5.31</v>
       </c>
       <c r="R14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>6.32</v>
+        <v>0.89</v>
       </c>
       <c r="V14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W14" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X14" s="3" t="n">
         <v>0</v>
@@ -1572,7 +1612,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46201</v>
+        <v>46207</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>54</v>
@@ -1584,10 +1624,10 @@
         <v>56</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>28</v>
@@ -1596,49 +1636,347 @@
         <v>31</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-14.5</v>
-      </c>
-      <c r="J15" s="3"/>
+        <v>35.5</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>167.5</v>
+      </c>
       <c r="K15" s="3" t="n">
-        <v>-20.19</v>
+        <v>22.78</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>174.53</v>
+        <v>157.69</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>10.09</v>
+        <v>-28.22</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>178.1</v>
+        <v>162.69</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="P15" s="3" t="n">
         <v>3.2</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>13.39</v>
+        <v>-5.31</v>
       </c>
       <c r="R15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S15" s="3" t="n">
-        <v>-3.76</v>
+        <v>-4.75</v>
       </c>
       <c r="T15" s="3" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="U15" s="3" t="n">
-        <v>6.32</v>
+        <v>0.89</v>
       </c>
       <c r="V15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W15" s="3" t="n">
-        <v>-3.57</v>
+        <v>-4.11</v>
       </c>
       <c r="X15" s="3" t="n">
+        <v>-0.89</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>178.5</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>25.95</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>163.81</v>
+      </c>
+      <c r="M16" s="3" t="n">
+        <v>-18.08</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>167.93</v>
+      </c>
+      <c r="O16" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="P16" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="Q16" s="3" t="n">
+        <v>-16.02</v>
+      </c>
+      <c r="R16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="3" t="n">
+        <v>-4.75</v>
+      </c>
+      <c r="T16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="3" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="V16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="3" t="n">
+        <v>-4.11</v>
+      </c>
+      <c r="X16" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>178.5</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>25.95</v>
+      </c>
+      <c r="L17" s="3" t="n">
+        <v>163.81</v>
+      </c>
+      <c r="M17" s="3" t="n">
+        <v>-18.08</v>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>167.93</v>
+      </c>
+      <c r="O17" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="P17" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="Q17" s="3" t="n">
+        <v>-16.02</v>
+      </c>
+      <c r="R17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="3" t="n">
+        <v>-4.75</v>
+      </c>
+      <c r="T17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" s="3" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="V17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" s="3" t="n">
+        <v>-4.11</v>
+      </c>
+      <c r="X17" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>-15.5</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>171.5</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>-19.68</v>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>166.78</v>
+      </c>
+      <c r="M18" s="3" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>170.9</v>
+      </c>
+      <c r="O18" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P18" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="Q18" s="3" t="n">
+        <v>-7.74</v>
+      </c>
+      <c r="R18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="3" t="n">
+        <v>-4.75</v>
+      </c>
+      <c r="T18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" s="3" t="n">
+        <v>14.31</v>
+      </c>
+      <c r="V18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" s="3" t="n">
+        <v>-4.11</v>
+      </c>
+      <c r="X18" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>-15.5</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>171.5</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>-19.68</v>
+      </c>
+      <c r="L19" s="3" t="n">
+        <v>166.78</v>
+      </c>
+      <c r="M19" s="3" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>170.9</v>
+      </c>
+      <c r="O19" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="P19" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="Q19" s="3" t="n">
+        <v>-7.74</v>
+      </c>
+      <c r="R19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="3" t="n">
+        <v>-4.75</v>
+      </c>
+      <c r="T19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="3" t="n">
+        <v>14.31</v>
+      </c>
+      <c r="V19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="3" t="n">
+        <v>-4.11</v>
+      </c>
+      <c r="X19" s="3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-07-11 09:44:57
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -86,133 +86,121 @@
     <t xml:space="preserve">rain_total_adj</t>
   </si>
   <si>
-    <t xml:space="preserve">19:30</t>
+    <t xml:space="preserve">18:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optus Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collingwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marvel Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neutral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interstate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">greater western sydney</t>
   </si>
   <si>
     <t xml:space="preserve">geelong cats</t>
   </si>
   <si>
+    <t xml:space="preserve">ENGIE Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hawthorn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SameCitySameGround</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adelaide Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">western bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">west coast eagles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:40</t>
+  </si>
+  <si>
     <t xml:space="preserve">brisbane lions</t>
   </si>
   <si>
-    <t xml:space="preserve">GMHBA Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Rain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Interstate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather Adjusted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">west coast eagles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optus Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UTAS Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neutral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corroboree Group Oval Manuka</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People First Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SameCitySameGround</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:15</t>
-  </si>
-  <si>
     <t xml:space="preserve">essendon</t>
   </si>
   <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marvel Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adelaide Oval</t>
+    <t xml:space="preserve">Gabba</t>
   </si>
 </sst>
 </file>
@@ -551,9 +539,9 @@
     <col min="1" max="1" width="5.7099999026863" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="5.7099999026863" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="22.7099995718197" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="16.7099996885961" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="17.7099996691334" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="16.7099996885961" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="28.7099994550433" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="14.7099997275216" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="13.7099997469844" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="16.7099996885961" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="17.7099996691334" hidden="0" customWidth="1"/>
@@ -650,7 +638,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46205</v>
+        <v>46212</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>24</v>
@@ -674,31 +662,31 @@
         <v>29</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>-14.5</v>
+        <v>-12.5</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>172.5</v>
+        <v>175.5</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-13.97</v>
+        <v>-36.52</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>185.4</v>
+        <v>168.25</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>12.41</v>
+        <v>14.57</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>189.52</v>
+        <v>172.36</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>30</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>5.3</v>
+        <v>10.5</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>0.27</v>
+        <v>18.31</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
@@ -710,7 +698,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="3" t="n">
-        <v>8.14</v>
+        <v>0.8</v>
       </c>
       <c r="V2" s="3" t="n">
         <v>0</v>
@@ -724,7 +712,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46205</v>
+        <v>46212</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>24</v>
@@ -736,7 +724,7 @@
         <v>26</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>3.8</v>
+        <v>1.7</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>27</v>
@@ -748,31 +736,31 @@
         <v>31</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>-14.5</v>
+        <v>-12.5</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>172.5</v>
+        <v>175.5</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>-14.46</v>
+        <v>-36.74</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>182.04</v>
+        <v>166.74</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>12.41</v>
+        <v>14.57</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>189.52</v>
+        <v>172.36</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>30</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>5.3</v>
+        <v>10.5</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>0.27</v>
+        <v>18.31</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>0</v>
@@ -781,10 +769,10 @@
         <v>-4.75</v>
       </c>
       <c r="T3" s="3" t="n">
-        <v>0.49</v>
+        <v>0.22</v>
       </c>
       <c r="U3" s="3" t="n">
-        <v>8.14</v>
+        <v>0.8</v>
       </c>
       <c r="V3" s="3" t="n">
         <v>0</v>
@@ -793,12 +781,12 @@
         <v>-4.11</v>
       </c>
       <c r="X3" s="3" t="n">
-        <v>-3.36</v>
+        <v>-1.51</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46206</v>
+        <v>46213</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>32</v>
@@ -822,31 +810,31 @@
         <v>29</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>30.5</v>
+        <v>-17.5</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>172.5</v>
+        <v>174.5</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>29.92</v>
+        <v>-22.21</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>163.9</v>
+        <v>165.19</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>-31.21</v>
+        <v>22.74</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>168.02</v>
+        <v>169.3</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>36</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>10.5</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>-7.83</v>
+        <v>-14.71</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>0</v>
@@ -858,7 +846,7 @@
         <v>0</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>2.21</v>
+        <v>7.95</v>
       </c>
       <c r="V4" s="3" t="n">
         <v>0</v>
@@ -872,7 +860,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46206</v>
+        <v>46213</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>32</v>
@@ -896,31 +884,31 @@
         <v>31</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>30.5</v>
+        <v>-17.5</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>172.5</v>
+        <v>174.5</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>29.92</v>
+        <v>-22.21</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>163.9</v>
+        <v>165.19</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>-31.21</v>
+        <v>22.74</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>168.02</v>
+        <v>169.3</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>36</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>10.5</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>-7.83</v>
+        <v>-14.71</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>0</v>
@@ -932,7 +920,7 @@
         <v>0</v>
       </c>
       <c r="U5" s="3" t="n">
-        <v>2.21</v>
+        <v>7.95</v>
       </c>
       <c r="V5" s="3" t="n">
         <v>0</v>
@@ -946,7 +934,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46206</v>
+        <v>46214</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>37</v>
@@ -961,7 +949,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>28</v>
@@ -970,31 +958,31 @@
         <v>29</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-18.5</v>
+        <v>-9.5</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>184.5</v>
+        <v>171.5</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-10.11</v>
+        <v>-14.94</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>179.7</v>
+        <v>158.8</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>12.49</v>
+        <v>7.14</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>183.82</v>
+        <v>162.91</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="P6" s="3" t="n">
         <v>5.3</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>-10.42</v>
+        <v>0.7</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>0</v>
@@ -1006,7 +994,7 @@
         <v>0</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>-8.94</v>
+        <v>3.47</v>
       </c>
       <c r="V6" s="3" t="n">
         <v>0</v>
@@ -1020,7 +1008,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46206</v>
+        <v>46214</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>37</v>
@@ -1032,10 +1020,10 @@
         <v>39</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>28</v>
@@ -1044,31 +1032,31 @@
         <v>31</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>-18.5</v>
+        <v>-9.5</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>184.5</v>
+        <v>171.5</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>-10.15</v>
+        <v>-14.94</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>179.44</v>
+        <v>158.8</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>12.49</v>
+        <v>7.14</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>183.82</v>
+        <v>162.91</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="P7" s="3" t="n">
         <v>5.3</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>-10.42</v>
+        <v>0.7</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>0</v>
@@ -1077,10 +1065,10 @@
         <v>-4.75</v>
       </c>
       <c r="T7" s="3" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="U7" s="3" t="n">
-        <v>-8.94</v>
+        <v>3.47</v>
       </c>
       <c r="V7" s="3" t="n">
         <v>0</v>
@@ -1089,12 +1077,12 @@
         <v>-4.11</v>
       </c>
       <c r="X7" s="3" t="n">
-        <v>-0.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46207</v>
+        <v>46214</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>41</v>
@@ -1118,31 +1106,31 @@
         <v>29</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>-15.5</v>
+        <v>8.5</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>171.5</v>
+        <v>185.5</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>-16.41</v>
+        <v>19.22</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>173.01</v>
+        <v>180.28</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>9.77</v>
+        <v>-14.99</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>177.13</v>
+        <v>184.4</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="P8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>8.17</v>
+        <v>-22.88</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>0</v>
@@ -1154,7 +1142,7 @@
         <v>0</v>
       </c>
       <c r="U8" s="3" t="n">
-        <v>-7.18</v>
+        <v>10.93</v>
       </c>
       <c r="V8" s="3" t="n">
         <v>0</v>
@@ -1168,7 +1156,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46207</v>
+        <v>46214</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>41</v>
@@ -1192,31 +1180,31 @@
         <v>31</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>-15.5</v>
+        <v>8.5</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>171.5</v>
+        <v>185.5</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>-16.41</v>
+        <v>19.22</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>173.01</v>
+        <v>180.28</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>9.77</v>
+        <v>-14.99</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>177.13</v>
+        <v>184.4</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="P9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>8.17</v>
+        <v>-22.88</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>0</v>
@@ -1228,7 +1216,7 @@
         <v>0</v>
       </c>
       <c r="U9" s="3" t="n">
-        <v>-7.18</v>
+        <v>10.93</v>
       </c>
       <c r="V9" s="3" t="n">
         <v>0</v>
@@ -1242,22 +1230,22 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46207</v>
+        <v>46214</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>28</v>
@@ -1266,31 +1254,31 @@
         <v>29</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>20.5</v>
+        <v>12.5</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>178.5</v>
+        <v>171.5</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>15.1</v>
+        <v>-15.98</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>165.93</v>
+        <v>164.32</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>-14.6</v>
+        <v>-8.38</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>170.04</v>
+        <v>168.43</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>-6.25</v>
+        <v>39.59</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>0</v>
@@ -1302,7 +1290,7 @@
         <v>0</v>
       </c>
       <c r="U10" s="3" t="n">
-        <v>5.03</v>
+        <v>-2.47</v>
       </c>
       <c r="V10" s="3" t="n">
         <v>0</v>
@@ -1316,22 +1304,22 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46207</v>
+        <v>46214</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>28</v>
@@ -1340,31 +1328,31 @@
         <v>31</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>20.5</v>
+        <v>12.5</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>178.5</v>
+        <v>171.5</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>15.1</v>
+        <v>-16.65</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>165.93</v>
+        <v>159.71</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>-14.6</v>
+        <v>-8.38</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>170.04</v>
+        <v>168.43</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>-6.25</v>
+        <v>39.59</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>0</v>
@@ -1373,10 +1361,10 @@
         <v>-4.75</v>
       </c>
       <c r="T11" s="3" t="n">
-        <v>0</v>
+        <v>0.67</v>
       </c>
       <c r="U11" s="3" t="n">
-        <v>5.03</v>
+        <v>-2.47</v>
       </c>
       <c r="V11" s="3" t="n">
         <v>0</v>
@@ -1385,27 +1373,27 @@
         <v>-4.11</v>
       </c>
       <c r="X11" s="3" t="n">
-        <v>0</v>
+        <v>-4.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46207</v>
+        <v>46214</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="E12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>53</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>28</v>
@@ -1414,31 +1402,31 @@
         <v>29</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>-8.5</v>
+        <v>-17.5</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>173.5</v>
+        <v>161.5</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>-9.31</v>
+        <v>-27.78</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>159.71</v>
+        <v>165.48</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>2.02</v>
+        <v>12.9</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>163.83</v>
+        <v>169.59</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="P12" s="3" t="n">
         <v>5.3</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>5.03</v>
+        <v>16.23</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0</v>
@@ -1450,7 +1438,7 @@
         <v>0</v>
       </c>
       <c r="U12" s="3" t="n">
-        <v>1.95</v>
+        <v>3.93</v>
       </c>
       <c r="V12" s="3" t="n">
         <v>0</v>
@@ -1464,22 +1452,22 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46207</v>
+        <v>46214</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="n">
+        <v>12.92</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>53</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>28</v>
@@ -1488,31 +1476,31 @@
         <v>31</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-8.5</v>
+        <v>-17.5</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>173.5</v>
+        <v>161.5</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-9.31</v>
+        <v>-29.45</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>159.71</v>
+        <v>154.04</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>2.02</v>
+        <v>12.9</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>163.83</v>
+        <v>169.59</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="P13" s="3" t="n">
         <v>5.3</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>5.03</v>
+        <v>16.23</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0</v>
@@ -1521,10 +1509,10 @@
         <v>-4.75</v>
       </c>
       <c r="T13" s="3" t="n">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="U13" s="3" t="n">
-        <v>1.95</v>
+        <v>3.93</v>
       </c>
       <c r="V13" s="3" t="n">
         <v>0</v>
@@ -1533,27 +1521,27 @@
         <v>-4.11</v>
       </c>
       <c r="X13" s="3" t="n">
-        <v>0</v>
+        <v>-11.44</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46207</v>
+        <v>46215</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="D14" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>56</v>
-      </c>
       <c r="E14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>28</v>
@@ -1562,31 +1550,31 @@
         <v>29</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>35.5</v>
+        <v>-36.5</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>167.5</v>
+        <v>176.5</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>22.91</v>
+        <v>-46.39</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>158.58</v>
+        <v>172.27</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>-28.22</v>
+        <v>43.41</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>162.69</v>
+        <v>176.38</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>3.2</v>
+        <v>5.3</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>-5.31</v>
+        <v>5.72</v>
       </c>
       <c r="R14" s="3" t="n">
         <v>0</v>
@@ -1598,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>0.89</v>
+        <v>-1.97</v>
       </c>
       <c r="V14" s="3" t="n">
         <v>0</v>
@@ -1612,22 +1600,22 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46207</v>
+        <v>46215</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>56</v>
-      </c>
       <c r="E15" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>28</v>
@@ -1636,31 +1624,31 @@
         <v>31</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>35.5</v>
+        <v>-36.5</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>167.5</v>
+        <v>176.5</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>22.78</v>
+        <v>-46.39</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>157.69</v>
+        <v>172.27</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>-28.22</v>
+        <v>43.41</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>162.69</v>
+        <v>176.38</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>3.2</v>
+        <v>5.3</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>-5.31</v>
+        <v>5.72</v>
       </c>
       <c r="R15" s="3" t="n">
         <v>0</v>
@@ -1669,10 +1657,10 @@
         <v>-4.75</v>
       </c>
       <c r="T15" s="3" t="n">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="U15" s="3" t="n">
-        <v>0.89</v>
+        <v>-1.97</v>
       </c>
       <c r="V15" s="3" t="n">
         <v>0</v>
@@ -1681,27 +1669,27 @@
         <v>-4.11</v>
       </c>
       <c r="X15" s="3" t="n">
-        <v>-0.89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46208</v>
+        <v>46215</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>28</v>
@@ -1710,31 +1698,31 @@
         <v>29</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>29.5</v>
+        <v>-41.5</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>178.5</v>
+        <v>172.5</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>25.95</v>
+        <v>-41.18</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>163.81</v>
+        <v>167.28</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>-18.08</v>
+        <v>36.43</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>167.93</v>
+        <v>171.39</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="P16" s="3" t="n">
         <v>3.2</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>-16.02</v>
+        <v>-0.89</v>
       </c>
       <c r="R16" s="3" t="n">
         <v>0</v>
@@ -1746,7 +1734,7 @@
         <v>0</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>9.93</v>
+        <v>-0.54</v>
       </c>
       <c r="V16" s="3" t="n">
         <v>0</v>
@@ -1760,22 +1748,22 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46208</v>
+        <v>46215</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0</v>
+        <v>5.4</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>28</v>
@@ -1784,31 +1772,31 @@
         <v>31</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>29.5</v>
+        <v>-41.5</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>178.5</v>
+        <v>172.5</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>25.95</v>
+        <v>-41.88</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>163.81</v>
+        <v>162.5</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>-18.08</v>
+        <v>36.43</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>167.93</v>
+        <v>171.39</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="P17" s="3" t="n">
         <v>3.2</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>-16.02</v>
+        <v>-0.89</v>
       </c>
       <c r="R17" s="3" t="n">
         <v>0</v>
@@ -1817,10 +1805,10 @@
         <v>-4.75</v>
       </c>
       <c r="T17" s="3" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="U17" s="3" t="n">
-        <v>9.93</v>
+        <v>-0.54</v>
       </c>
       <c r="V17" s="3" t="n">
         <v>0</v>
@@ -1829,27 +1817,27 @@
         <v>-4.11</v>
       </c>
       <c r="X17" s="3" t="n">
-        <v>0</v>
+        <v>-4.78</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46208</v>
+        <v>46215</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>28</v>
@@ -1858,31 +1846,31 @@
         <v>29</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>-15.5</v>
+        <v>-62.5</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>171.5</v>
+        <v>187.5</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>-19.68</v>
+        <v>-55.8</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>166.78</v>
+        <v>174.99</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>17.09</v>
+        <v>40.94</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>170.9</v>
+        <v>179.1</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="P18" s="3" t="n">
         <v>5.3</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>-7.74</v>
+        <v>5.16</v>
       </c>
       <c r="R18" s="3" t="n">
         <v>0</v>
@@ -1894,7 +1882,7 @@
         <v>0</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>14.31</v>
+        <v>10.56</v>
       </c>
       <c r="V18" s="3" t="n">
         <v>0</v>
@@ -1908,22 +1896,22 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46208</v>
+        <v>46215</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0</v>
+        <v>1.17</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>28</v>
@@ -1932,31 +1920,31 @@
         <v>31</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>-15.5</v>
+        <v>-62.5</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>171.5</v>
+        <v>187.5</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>-19.68</v>
+        <v>-55.95</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>166.78</v>
+        <v>173.95</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>17.09</v>
+        <v>40.94</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>170.9</v>
+        <v>179.1</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="P19" s="3" t="n">
         <v>5.3</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>-7.74</v>
+        <v>5.16</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>0</v>
@@ -1965,10 +1953,10 @@
         <v>-4.75</v>
       </c>
       <c r="T19" s="3" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="U19" s="3" t="n">
-        <v>14.31</v>
+        <v>10.56</v>
       </c>
       <c r="V19" s="3" t="n">
         <v>0</v>
@@ -1977,7 +1965,7 @@
         <v>-4.11</v>
       </c>
       <c r="X19" s="3" t="n">
-        <v>0</v>
+        <v>-1.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-07-14 18:08:57
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -86,121 +86,100 @@
     <t xml:space="preserve">rain_total_adj</t>
   </si>
   <si>
+    <t xml:space="preserve">19:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GMHBA Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SameStateOther</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interstate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adelaide Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marvel Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SameCityDiffGround</t>
+  </si>
+  <si>
     <t xml:space="preserve">18:10</t>
   </si>
   <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
+    <t xml:space="preserve">west coast eagles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
   </si>
   <si>
     <t xml:space="preserve">Optus Stadium</t>
   </si>
   <si>
-    <t xml:space="preserve">FT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Rain</t>
-  </si>
-  <si>
     <t xml:space="preserve">Perth</t>
   </si>
   <si>
-    <t xml:space="preserve">Weather Adjusted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:40</t>
+    <t xml:space="preserve">19:35</t>
   </si>
   <si>
     <t xml:space="preserve">collingwood</t>
   </si>
   <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marvel Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neutral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Interstate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENGIE Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:35</t>
-  </si>
-  <si>
     <t xml:space="preserve">carlton</t>
   </si>
   <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
     <t xml:space="preserve">MCG</t>
   </si>
   <si>
     <t xml:space="preserve">SameCitySameGround</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adelaide Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">west coast eagles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gabba</t>
   </si>
 </sst>
 </file>
@@ -538,8 +517,8 @@
   <cols>
     <col min="1" max="1" width="5.7099999026863" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="5.7099999026863" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="22.7099995718197" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="17.7099996691334" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="17.7099996691334" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="14.7099997275216" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="16.7099996885961" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="14.7099997275216" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="13.7099997469844" hidden="0" customWidth="1"/>
@@ -638,7 +617,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46212</v>
+        <v>46219</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>24</v>
@@ -665,46 +644,46 @@
         <v>-12.5</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>175.5</v>
+        <v>182.5</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>-36.52</v>
+        <v>-25.95</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>168.25</v>
+        <v>173.74</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>14.57</v>
+        <v>20.7</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>172.36</v>
+        <v>178.45</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>30</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>10.5</v>
+        <v>4.8</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>18.31</v>
+        <v>7.88</v>
       </c>
       <c r="R2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U2" s="3" t="n">
-        <v>0.8</v>
+        <v>2.44</v>
       </c>
       <c r="V2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W2" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X2" s="3" t="n">
         <v>0</v>
@@ -712,7 +691,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46212</v>
+        <v>46219</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>24</v>
@@ -724,7 +703,7 @@
         <v>26</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1.7</v>
+        <v>0.1</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>27</v>
@@ -739,54 +718,54 @@
         <v>-12.5</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>175.5</v>
+        <v>182.5</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>-36.74</v>
+        <v>-25.96</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>166.74</v>
+        <v>173.65</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>14.57</v>
+        <v>20.7</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>172.36</v>
+        <v>178.45</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>30</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>10.5</v>
+        <v>4.8</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>18.31</v>
+        <v>7.88</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S3" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T3" s="3" t="n">
-        <v>0.22</v>
+        <v>0.01</v>
       </c>
       <c r="U3" s="3" t="n">
-        <v>0.8</v>
+        <v>2.44</v>
       </c>
       <c r="V3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W3" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X3" s="3" t="n">
-        <v>-1.51</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46213</v>
+        <v>46220</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>32</v>
@@ -810,49 +789,49 @@
         <v>29</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>-17.5</v>
+        <v>-12.5</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>174.5</v>
+        <v>179.5</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>-22.21</v>
+        <v>-2.32</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>165.19</v>
+        <v>170.06</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>22.74</v>
+        <v>4.91</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>169.3</v>
+        <v>174.78</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>36</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>-14.71</v>
+        <v>-12.23</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>7.95</v>
+        <v>-3.1</v>
       </c>
       <c r="V4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W4" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X4" s="3" t="n">
         <v>0</v>
@@ -860,7 +839,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46213</v>
+        <v>46220</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>32</v>
@@ -872,7 +851,7 @@
         <v>34</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0</v>
+        <v>5.8</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>35</v>
@@ -884,57 +863,57 @@
         <v>31</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-17.5</v>
+        <v>-12.5</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>174.5</v>
+        <v>179.5</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>-22.21</v>
+        <v>-2.86</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>165.19</v>
+        <v>165.04</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>22.74</v>
+        <v>4.91</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>169.3</v>
+        <v>174.78</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>36</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>-14.71</v>
+        <v>-12.23</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T5" s="3" t="n">
-        <v>0</v>
+        <v>0.54</v>
       </c>
       <c r="U5" s="3" t="n">
-        <v>7.95</v>
+        <v>-3.1</v>
       </c>
       <c r="V5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W5" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X5" s="3" t="n">
-        <v>0</v>
+        <v>-5.02</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>37</v>
@@ -949,7 +928,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>28</v>
@@ -958,49 +937,49 @@
         <v>29</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-9.5</v>
+        <v>47.5</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>171.5</v>
+        <v>169.5</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>-14.94</v>
+        <v>24.6</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>158.8</v>
+        <v>153.17</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>7.14</v>
+        <v>-16.27</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>162.91</v>
+        <v>157.88</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="P6" s="3" t="n">
         <v>5.3</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>0.7</v>
+        <v>-7.82</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>3.47</v>
+        <v>9.63</v>
       </c>
       <c r="V6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W6" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X6" s="3" t="n">
         <v>0</v>
@@ -1008,7 +987,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>37</v>
@@ -1023,7 +1002,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>28</v>
@@ -1032,49 +1011,49 @@
         <v>31</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>-9.5</v>
+        <v>47.5</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>171.5</v>
+        <v>169.5</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>-14.94</v>
+        <v>24.6</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>158.8</v>
+        <v>153.17</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>7.14</v>
+        <v>-16.27</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>162.91</v>
+        <v>157.88</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="P7" s="3" t="n">
         <v>5.3</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>0.7</v>
+        <v>-7.82</v>
       </c>
       <c r="R7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U7" s="3" t="n">
-        <v>3.47</v>
+        <v>9.63</v>
       </c>
       <c r="V7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W7" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X7" s="3" t="n">
         <v>0</v>
@@ -1082,7 +1061,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>41</v>
@@ -1106,49 +1085,49 @@
         <v>29</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>8.5</v>
+        <v>14.5</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>185.5</v>
+        <v>178.5</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>19.22</v>
+        <v>5.93</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>180.28</v>
+        <v>176.86</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>-14.99</v>
+        <v>-16.04</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>184.4</v>
+        <v>181.57</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>-22.88</v>
+        <v>13.65</v>
       </c>
       <c r="R8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S8" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U8" s="3" t="n">
-        <v>10.93</v>
+        <v>7.54</v>
       </c>
       <c r="V8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W8" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X8" s="3" t="n">
         <v>0</v>
@@ -1156,7 +1135,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>41</v>
@@ -1180,49 +1159,49 @@
         <v>31</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>8.5</v>
+        <v>14.5</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>185.5</v>
+        <v>178.5</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>19.22</v>
+        <v>5.93</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>180.28</v>
+        <v>176.86</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>-14.99</v>
+        <v>-16.04</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>184.4</v>
+        <v>181.57</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>-22.88</v>
+        <v>13.65</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S9" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U9" s="3" t="n">
-        <v>10.93</v>
+        <v>7.54</v>
       </c>
       <c r="V9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W9" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X9" s="3" t="n">
         <v>0</v>
@@ -1230,22 +1209,22 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>28</v>
@@ -1254,49 +1233,49 @@
         <v>29</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>12.5</v>
+        <v>44.5</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>171.5</v>
+        <v>169.5</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>-15.98</v>
+        <v>33.17</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>164.32</v>
+        <v>178.17</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>-8.38</v>
+        <v>-34.07</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>168.43</v>
+        <v>182.88</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>3.2</v>
+        <v>10.5</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>39.59</v>
+        <v>-2.77</v>
       </c>
       <c r="R10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S10" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U10" s="3" t="n">
-        <v>-2.47</v>
+        <v>9.82</v>
       </c>
       <c r="V10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W10" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X10" s="3" t="n">
         <v>0</v>
@@ -1304,22 +1283,22 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>5.2</v>
+        <v>5.13</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>28</v>
@@ -1328,72 +1307,72 @@
         <v>31</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>12.5</v>
+        <v>44.5</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>171.5</v>
+        <v>169.5</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>-16.65</v>
+        <v>32.69</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>159.71</v>
+        <v>173.72</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>-8.38</v>
+        <v>-34.07</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>168.43</v>
+        <v>182.88</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>3.2</v>
+        <v>10.5</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>39.59</v>
+        <v>-2.77</v>
       </c>
       <c r="R11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S11" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T11" s="3" t="n">
-        <v>0.67</v>
+        <v>0.48</v>
       </c>
       <c r="U11" s="3" t="n">
-        <v>-2.47</v>
+        <v>9.82</v>
       </c>
       <c r="V11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W11" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X11" s="3" t="n">
-        <v>-4.6</v>
+        <v>-4.44</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>28</v>
@@ -1402,49 +1381,49 @@
         <v>29</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>-17.5</v>
+        <v>-6.5</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>161.5</v>
+        <v>170.5</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>-27.78</v>
+        <v>-23.89</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>165.48</v>
+        <v>153.18</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>12.9</v>
+        <v>12.32</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>169.59</v>
+        <v>157.89</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>5.3</v>
+        <v>3.2</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>16.23</v>
+        <v>14.29</v>
       </c>
       <c r="R12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S12" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="U12" s="3" t="n">
-        <v>3.93</v>
+        <v>-2.69</v>
       </c>
       <c r="V12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W12" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X12" s="3" t="n">
         <v>0</v>
@@ -1452,22 +1431,22 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46214</v>
+        <v>46221</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>12.92</v>
+        <v>0</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>28</v>
@@ -1476,496 +1455,52 @@
         <v>31</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>-17.5</v>
+        <v>-6.5</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>161.5</v>
+        <v>170.5</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>-29.45</v>
+        <v>-23.89</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>154.04</v>
+        <v>153.18</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>12.9</v>
+        <v>12.32</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>169.59</v>
+        <v>157.89</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>5.3</v>
+        <v>3.2</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>16.23</v>
+        <v>14.29</v>
       </c>
       <c r="R13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S13" s="3" t="n">
-        <v>-4.75</v>
+        <v>-4.42</v>
       </c>
       <c r="T13" s="3" t="n">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="U13" s="3" t="n">
-        <v>3.93</v>
+        <v>-2.69</v>
       </c>
       <c r="V13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W13" s="3" t="n">
-        <v>-4.11</v>
+        <v>-4.72</v>
       </c>
       <c r="X13" s="3" t="n">
-        <v>-11.44</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>46215</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I14" s="3" t="n">
-        <v>-36.5</v>
-      </c>
-      <c r="J14" s="3" t="n">
-        <v>176.5</v>
-      </c>
-      <c r="K14" s="3" t="n">
-        <v>-46.39</v>
-      </c>
-      <c r="L14" s="3" t="n">
-        <v>172.27</v>
-      </c>
-      <c r="M14" s="3" t="n">
-        <v>43.41</v>
-      </c>
-      <c r="N14" s="3" t="n">
-        <v>176.38</v>
-      </c>
-      <c r="O14" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="P14" s="3" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="Q14" s="3" t="n">
-        <v>5.72</v>
-      </c>
-      <c r="R14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="3" t="n">
-        <v>-4.75</v>
-      </c>
-      <c r="T14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U14" s="3" t="n">
-        <v>-1.97</v>
-      </c>
-      <c r="V14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W14" s="3" t="n">
-        <v>-4.11</v>
-      </c>
-      <c r="X14" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>46215</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I15" s="3" t="n">
-        <v>-36.5</v>
-      </c>
-      <c r="J15" s="3" t="n">
-        <v>176.5</v>
-      </c>
-      <c r="K15" s="3" t="n">
-        <v>-46.39</v>
-      </c>
-      <c r="L15" s="3" t="n">
-        <v>172.27</v>
-      </c>
-      <c r="M15" s="3" t="n">
-        <v>43.41</v>
-      </c>
-      <c r="N15" s="3" t="n">
-        <v>176.38</v>
-      </c>
-      <c r="O15" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="P15" s="3" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="Q15" s="3" t="n">
-        <v>5.72</v>
-      </c>
-      <c r="R15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="3" t="n">
-        <v>-4.75</v>
-      </c>
-      <c r="T15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" s="3" t="n">
-        <v>-1.97</v>
-      </c>
-      <c r="V15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W15" s="3" t="n">
-        <v>-4.11</v>
-      </c>
-      <c r="X15" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>46215</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I16" s="3" t="n">
-        <v>-41.5</v>
-      </c>
-      <c r="J16" s="3" t="n">
-        <v>172.5</v>
-      </c>
-      <c r="K16" s="3" t="n">
-        <v>-41.18</v>
-      </c>
-      <c r="L16" s="3" t="n">
-        <v>167.28</v>
-      </c>
-      <c r="M16" s="3" t="n">
-        <v>36.43</v>
-      </c>
-      <c r="N16" s="3" t="n">
-        <v>171.39</v>
-      </c>
-      <c r="O16" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="P16" s="3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="Q16" s="3" t="n">
-        <v>-0.89</v>
-      </c>
-      <c r="R16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="3" t="n">
-        <v>-4.75</v>
-      </c>
-      <c r="T16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U16" s="3" t="n">
-        <v>-0.54</v>
-      </c>
-      <c r="V16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W16" s="3" t="n">
-        <v>-4.11</v>
-      </c>
-      <c r="X16" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>46215</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I17" s="3" t="n">
-        <v>-41.5</v>
-      </c>
-      <c r="J17" s="3" t="n">
-        <v>172.5</v>
-      </c>
-      <c r="K17" s="3" t="n">
-        <v>-41.88</v>
-      </c>
-      <c r="L17" s="3" t="n">
-        <v>162.5</v>
-      </c>
-      <c r="M17" s="3" t="n">
-        <v>36.43</v>
-      </c>
-      <c r="N17" s="3" t="n">
-        <v>171.39</v>
-      </c>
-      <c r="O17" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="P17" s="3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="Q17" s="3" t="n">
-        <v>-0.89</v>
-      </c>
-      <c r="R17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" s="3" t="n">
-        <v>-4.75</v>
-      </c>
-      <c r="T17" s="3" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="U17" s="3" t="n">
-        <v>-0.54</v>
-      </c>
-      <c r="V17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W17" s="3" t="n">
-        <v>-4.11</v>
-      </c>
-      <c r="X17" s="3" t="n">
-        <v>-4.78</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>46215</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I18" s="3" t="n">
-        <v>-62.5</v>
-      </c>
-      <c r="J18" s="3" t="n">
-        <v>187.5</v>
-      </c>
-      <c r="K18" s="3" t="n">
-        <v>-55.8</v>
-      </c>
-      <c r="L18" s="3" t="n">
-        <v>174.99</v>
-      </c>
-      <c r="M18" s="3" t="n">
-        <v>40.94</v>
-      </c>
-      <c r="N18" s="3" t="n">
-        <v>179.1</v>
-      </c>
-      <c r="O18" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="P18" s="3" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="Q18" s="3" t="n">
-        <v>5.16</v>
-      </c>
-      <c r="R18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" s="3" t="n">
-        <v>-4.75</v>
-      </c>
-      <c r="T18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U18" s="3" t="n">
-        <v>10.56</v>
-      </c>
-      <c r="V18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W18" s="3" t="n">
-        <v>-4.11</v>
-      </c>
-      <c r="X18" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>46215</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I19" s="3" t="n">
-        <v>-62.5</v>
-      </c>
-      <c r="J19" s="3" t="n">
-        <v>187.5</v>
-      </c>
-      <c r="K19" s="3" t="n">
-        <v>-55.95</v>
-      </c>
-      <c r="L19" s="3" t="n">
-        <v>173.95</v>
-      </c>
-      <c r="M19" s="3" t="n">
-        <v>40.94</v>
-      </c>
-      <c r="N19" s="3" t="n">
-        <v>179.1</v>
-      </c>
-      <c r="O19" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="P19" s="3" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="Q19" s="3" t="n">
-        <v>5.16</v>
-      </c>
-      <c r="R19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" s="3" t="n">
-        <v>-4.75</v>
-      </c>
-      <c r="T19" s="3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="U19" s="3" t="n">
-        <v>10.56</v>
-      </c>
-      <c r="V19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W19" s="3" t="n">
-        <v>-4.11</v>
-      </c>
-      <c r="X19" s="3" t="n">
-        <v>-1.03</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-07-25 13:10:46
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -946,52 +946,52 @@
         <v>4.36660785533764</v>
       </c>
       <c r="R2" t="n">
-        <v>-5.68122316188563</v>
+        <v>-9.05039241406247</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.254325413552674</v>
+        <v>-3.37223231229803</v>
       </c>
       <c r="T2" t="n">
-        <v>1.12368956519145</v>
+        <v>4.22936177423395</v>
       </c>
       <c r="U2" t="n">
-        <v>-0.657282145641784</v>
+        <v>2.60847014545934</v>
       </c>
       <c r="V2" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W2" t="n">
-        <v>82.605705131632</v>
+        <v>74.7923314509488</v>
       </c>
       <c r="X2" t="n">
-        <v>81.8850233137941</v>
+        <v>74.482992068601</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.720681817837928</v>
+        <v>0.309339382347787</v>
       </c>
       <c r="Z2" t="n">
-        <v>164.490728445426</v>
+        <v>149.27532351955</v>
       </c>
       <c r="AA2" t="n">
         <v>0</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.840633563247109</v>
+        <v>0.360826457389771</v>
       </c>
       <c r="AC2" t="n">
-        <v>165.803946192675</v>
+        <v>153.2261744013</v>
       </c>
       <c r="AD2" t="n">
-        <v>2.0723329515782</v>
+        <v>1.96974538087368</v>
       </c>
       <c r="AE2" t="n">
-        <v>2.1552643484454</v>
+        <v>4.14058592115706</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.79301476941613</v>
+        <v>2.27908476322146</v>
       </c>
       <c r="AG2" t="n">
-        <v>166.645992793872</v>
+        <v>153.415909440707</v>
       </c>
       <c r="AH2" t="s">
         <v>73</v>
@@ -1012,22 +1012,22 @@
         <v>0</v>
       </c>
       <c r="AN2" t="n">
-        <v>2.79301476941613</v>
+        <v>2.27908476322146</v>
       </c>
       <c r="AO2" t="n">
-        <v>166.645992793872</v>
+        <v>153.415909440707</v>
       </c>
       <c r="AP2" t="n">
-        <v>84.7195037816438</v>
+        <v>77.8474971019642</v>
       </c>
       <c r="AQ2" t="n">
-        <v>81.9264890122277</v>
+        <v>75.5684123387427</v>
       </c>
       <c r="AR2" t="n">
-        <v>2.79301476941613</v>
+        <v>2.27908476322146</v>
       </c>
       <c r="AS2" t="n">
-        <v>166.645992793872</v>
+        <v>153.415909440707</v>
       </c>
       <c r="AT2" t="s">
         <v>76</v>
@@ -1136,52 +1136,52 @@
         <v>4.04168960651118</v>
       </c>
       <c r="R3" t="n">
-        <v>2.79203927018599</v>
+        <v>3.17650055692725</v>
       </c>
       <c r="S3" t="n">
-        <v>-17.8480171010685</v>
+        <v>-17.3776995174184</v>
       </c>
       <c r="T3" t="n">
-        <v>3.06294734082283</v>
+        <v>2.65273024751581</v>
       </c>
       <c r="U3" t="n">
-        <v>-13.2768330293885</v>
+        <v>-13.7681964082168</v>
       </c>
       <c r="V3" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W3" t="n">
-        <v>103.536059323037</v>
+        <v>103.233431851201</v>
       </c>
       <c r="X3" t="n">
-        <v>62.5145329750602</v>
+        <v>62.216615514612</v>
       </c>
       <c r="Y3" t="n">
-        <v>41.021526347977</v>
+        <v>41.0168163365894</v>
       </c>
       <c r="Z3" t="n">
-        <v>166.050592298097</v>
+        <v>165.450047365814</v>
       </c>
       <c r="AA3" t="n">
         <v>0</v>
       </c>
       <c r="AB3" t="n">
-        <v>47.8492325048363</v>
+        <v>47.8437385495877</v>
       </c>
       <c r="AC3" t="n">
-        <v>167.043838946479</v>
+        <v>166.083016270805</v>
       </c>
       <c r="AD3" t="n">
-        <v>8.78008736302831</v>
+        <v>8.74518051882998</v>
       </c>
       <c r="AE3" t="n">
-        <v>1.83529324957746</v>
+        <v>0.822703944398826</v>
       </c>
       <c r="AF3" t="n">
-        <v>49.8016137110053</v>
+        <v>49.7619968554194</v>
       </c>
       <c r="AG3" t="n">
-        <v>167.885885547675</v>
+        <v>166.272751310212</v>
       </c>
       <c r="AH3" t="s">
         <v>73</v>
@@ -1202,22 +1202,22 @@
         <v>0</v>
       </c>
       <c r="AN3" t="n">
-        <v>49.8016137110053</v>
+        <v>49.7619968554194</v>
       </c>
       <c r="AO3" t="n">
-        <v>167.885885547675</v>
+        <v>166.272751310212</v>
       </c>
       <c r="AP3" t="n">
-        <v>108.84374962934</v>
+        <v>108.017374082816</v>
       </c>
       <c r="AQ3" t="n">
-        <v>59.0421359183348</v>
+        <v>58.2553772273965</v>
       </c>
       <c r="AR3" t="n">
-        <v>49.8016137110053</v>
+        <v>49.7619968554194</v>
       </c>
       <c r="AS3" t="n">
-        <v>167.885885547675</v>
+        <v>166.272751310212</v>
       </c>
       <c r="AT3" t="s">
         <v>76</v>
@@ -1326,52 +1326,52 @@
         <v>4.04168960651118</v>
       </c>
       <c r="R4" t="n">
-        <v>8.45417626471137</v>
+        <v>8.98047298291742</v>
       </c>
       <c r="S4" t="n">
-        <v>-15.245244174749</v>
+        <v>-14.786750403476</v>
       </c>
       <c r="T4" t="n">
-        <v>6.26237576757176</v>
+        <v>5.6818360724727</v>
       </c>
       <c r="U4" t="n">
-        <v>-10.7312038123684</v>
+        <v>-11.1491536585899</v>
       </c>
       <c r="V4" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W4" t="n">
-        <v>106.652567100542</v>
+        <v>106.418361527565</v>
       </c>
       <c r="X4" t="n">
-        <v>61.9178774746307</v>
+        <v>61.7784588035975</v>
       </c>
       <c r="Y4" t="n">
-        <v>44.7346896259117</v>
+        <v>44.6399027239672</v>
       </c>
       <c r="Z4" t="n">
-        <v>168.570444575173</v>
+        <v>168.196820331162</v>
       </c>
       <c r="AA4" t="n">
         <v>0</v>
       </c>
       <c r="AB4" t="n">
-        <v>52.1804222198938</v>
+        <v>52.0698587934848</v>
       </c>
       <c r="AC4" t="n">
-        <v>169.046800021351</v>
+        <v>168.266350342075</v>
       </c>
       <c r="AD4" t="n">
-        <v>9.3981138001511</v>
+        <v>9.34821437534936</v>
       </c>
       <c r="AE4" t="n">
-        <v>1.31840204737409</v>
+        <v>0.2592650503195</v>
       </c>
       <c r="AF4" t="n">
-        <v>54.1328034260628</v>
+        <v>53.9881170993165</v>
       </c>
       <c r="AG4" t="n">
-        <v>169.888846622547</v>
+        <v>168.456085381482</v>
       </c>
       <c r="AH4" t="s">
         <v>73</v>
@@ -1392,22 +1392,22 @@
         <v>0</v>
       </c>
       <c r="AN4" t="n">
-        <v>54.1328034260628</v>
+        <v>53.9881170993165</v>
       </c>
       <c r="AO4" t="n">
-        <v>169.888846622547</v>
+        <v>168.456085381482</v>
       </c>
       <c r="AP4" t="n">
-        <v>112.010825024305</v>
+        <v>111.222101240399</v>
       </c>
       <c r="AQ4" t="n">
-        <v>57.8780215982422</v>
+        <v>57.2339841410826</v>
       </c>
       <c r="AR4" t="n">
-        <v>54.1328034260628</v>
+        <v>53.9881170993165</v>
       </c>
       <c r="AS4" t="n">
-        <v>169.888846622547</v>
+        <v>168.456085381482</v>
       </c>
       <c r="AT4" t="s">
         <v>76</v>
@@ -1516,52 +1516,52 @@
         <v>4.04168960651118</v>
       </c>
       <c r="R5" t="n">
-        <v>3.17154102324608</v>
+        <v>3.58268626667377</v>
       </c>
       <c r="S5" t="n">
-        <v>8.71503778612408</v>
+        <v>8.99221483822378</v>
       </c>
       <c r="T5" t="n">
-        <v>0.295534331495312</v>
+        <v>-0.0929066414405306</v>
       </c>
       <c r="U5" t="n">
-        <v>3.2539565204658</v>
+        <v>2.96481935449112</v>
       </c>
       <c r="V5" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W5" t="n">
-        <v>87.3847715262429</v>
+        <v>86.90660179824</v>
       </c>
       <c r="X5" t="n">
-        <v>91.8450008715802</v>
+        <v>91.3321667592105</v>
       </c>
       <c r="Y5" t="n">
-        <v>-4.46022934533731</v>
+        <v>-4.42556496097048</v>
       </c>
       <c r="Z5" t="n">
-        <v>179.229772397823</v>
+        <v>178.238768557451</v>
       </c>
       <c r="AA5" t="n">
         <v>0</v>
       </c>
       <c r="AB5" t="n">
-        <v>-5.20259897595116</v>
+        <v>-5.16216498104967</v>
       </c>
       <c r="AC5" t="n">
-        <v>177.519605712107</v>
+        <v>176.248418019661</v>
       </c>
       <c r="AD5" t="n">
-        <v>1.21001157555517</v>
+        <v>1.1816582857525</v>
       </c>
       <c r="AE5" t="n">
-        <v>-0.868120084519857</v>
+        <v>-1.80061549838226</v>
       </c>
       <c r="AF5" t="n">
-        <v>-3.25021776978214</v>
+        <v>-3.24390667521797</v>
       </c>
       <c r="AG5" t="n">
-        <v>178.361652313303</v>
+        <v>176.438153059068</v>
       </c>
       <c r="AH5" t="s">
         <v>73</v>
@@ -1582,22 +1582,22 @@
         <v>0</v>
       </c>
       <c r="AN5" t="n">
-        <v>-3.25021776978214</v>
+        <v>-3.24390667521797</v>
       </c>
       <c r="AO5" t="n">
-        <v>178.361652313303</v>
+        <v>176.438153059068</v>
       </c>
       <c r="AP5" t="n">
-        <v>87.5557172717606</v>
+        <v>86.5971231919252</v>
       </c>
       <c r="AQ5" t="n">
-        <v>90.8059350415427</v>
+        <v>89.8410298671431</v>
       </c>
       <c r="AR5" t="n">
-        <v>-3.25021776978214</v>
+        <v>-3.24390667521797</v>
       </c>
       <c r="AS5" t="n">
-        <v>178.361652313303</v>
+        <v>176.438153059068</v>
       </c>
       <c r="AT5" t="s">
         <v>76</v>
@@ -1706,52 +1706,52 @@
         <v>4.36660785533764</v>
       </c>
       <c r="R6" t="n">
-        <v>13.581762825117</v>
+        <v>14.0266071378466</v>
       </c>
       <c r="S6" t="n">
-        <v>-6.88175771798916</v>
+        <v>-6.44780265080128</v>
       </c>
       <c r="T6" t="n">
-        <v>0.955307037766845</v>
+        <v>0.497474391585373</v>
       </c>
       <c r="U6" t="n">
-        <v>2.16006869446571</v>
+        <v>1.78319384794129</v>
       </c>
       <c r="V6" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W6" t="n">
-        <v>99.0513402785272</v>
+        <v>98.6946073003759</v>
       </c>
       <c r="X6" t="n">
-        <v>75.4259735367822</v>
+        <v>75.1393091127463</v>
       </c>
       <c r="Y6" t="n">
-        <v>23.6253667417449</v>
+        <v>23.5552981876296</v>
       </c>
       <c r="Z6" t="n">
-        <v>174.477313815309</v>
+        <v>173.833916413122</v>
       </c>
       <c r="AA6" t="n">
         <v>0</v>
       </c>
       <c r="AB6" t="n">
-        <v>27.5576207635075</v>
+        <v>27.4758898569414</v>
       </c>
       <c r="AC6" t="n">
-        <v>173.742007462671</v>
+        <v>172.747122540588</v>
       </c>
       <c r="AD6" t="n">
-        <v>5.88463522793156</v>
+        <v>5.83884997514354</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.106740248558084</v>
+        <v>-0.897058833127202</v>
       </c>
       <c r="AF6" t="n">
-        <v>29.5100019696765</v>
+        <v>29.3941481627731</v>
       </c>
       <c r="AG6" t="n">
-        <v>174.584054063867</v>
+        <v>172.936857579995</v>
       </c>
       <c r="AH6" t="s">
         <v>73</v>
@@ -1772,22 +1772,22 @@
         <v>1</v>
       </c>
       <c r="AN6" t="n">
-        <v>34.7110869408165</v>
+        <v>34.5952331339132</v>
       </c>
       <c r="AO6" t="n">
-        <v>174.584054063867</v>
+        <v>172.936857579995</v>
       </c>
       <c r="AP6" t="n">
-        <v>104.647570502342</v>
+        <v>103.766045356954</v>
       </c>
       <c r="AQ6" t="n">
-        <v>69.9364835615255</v>
+        <v>69.170812223041</v>
       </c>
       <c r="AR6" t="n">
-        <v>34.7110869408165</v>
+        <v>34.5952331339132</v>
       </c>
       <c r="AS6" t="n">
-        <v>174.584054063867</v>
+        <v>172.936857579995</v>
       </c>
       <c r="AT6" t="s">
         <v>76</v>
@@ -1896,52 +1896,52 @@
         <v>4.04168960651118</v>
       </c>
       <c r="R7" t="n">
-        <v>-6.16354687135813</v>
+        <v>-5.79948184305096</v>
       </c>
       <c r="S7" t="n">
-        <v>-0.103070263939211</v>
+        <v>0.230711257521621</v>
       </c>
       <c r="T7" t="n">
-        <v>-9.14961910059401</v>
+        <v>-9.45562114698717</v>
       </c>
       <c r="U7" t="n">
-        <v>0.566525293770441</v>
+        <v>0.227480976658517</v>
       </c>
       <c r="V7" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W7" t="n">
-        <v>80.7371148583341</v>
+        <v>80.2617720663479</v>
       </c>
       <c r="X7" t="n">
-        <v>92.4720462536063</v>
+        <v>91.933377684055</v>
       </c>
       <c r="Y7" t="n">
-        <v>-11.7349313952722</v>
+        <v>-11.6716056177071</v>
       </c>
       <c r="Z7" t="n">
-        <v>173.20916111194</v>
+        <v>172.195149750403</v>
       </c>
       <c r="AA7" t="n">
         <v>0</v>
       </c>
       <c r="AB7" t="n">
-        <v>-13.6881172094264</v>
+        <v>-13.6142513608337</v>
       </c>
       <c r="AC7" t="n">
-        <v>172.733987855748</v>
+        <v>171.4445121193</v>
       </c>
       <c r="AD7" t="n">
-        <v>-0.000804607985177785</v>
+        <v>-0.0243874372948847</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.366873345003968</v>
+        <v>-0.560902591695934</v>
       </c>
       <c r="AF7" t="n">
-        <v>-11.7357360032574</v>
+        <v>-11.695993055002</v>
       </c>
       <c r="AG7" t="n">
-        <v>173.576034456944</v>
+        <v>171.634247158707</v>
       </c>
       <c r="AH7" t="s">
         <v>73</v>
@@ -1962,22 +1962,22 @@
         <v>0</v>
       </c>
       <c r="AN7" t="n">
-        <v>-11.7357360032574</v>
+        <v>-11.695993055002</v>
       </c>
       <c r="AO7" t="n">
-        <v>173.576034456944</v>
+        <v>171.634247158707</v>
       </c>
       <c r="AP7" t="n">
-        <v>80.9201492268434</v>
+        <v>79.9691270518525</v>
       </c>
       <c r="AQ7" t="n">
-        <v>92.6558852301008</v>
+        <v>91.6651201068545</v>
       </c>
       <c r="AR7" t="n">
-        <v>-11.7357360032574</v>
+        <v>-11.695993055002</v>
       </c>
       <c r="AS7" t="n">
-        <v>173.576034456944</v>
+        <v>171.634247158707</v>
       </c>
       <c r="AT7" t="s">
         <v>76</v>
@@ -2084,52 +2084,52 @@
         <v>4.04168960651118</v>
       </c>
       <c r="R8" t="n">
-        <v>0.440470146506572</v>
+        <v>0.972883879086474</v>
       </c>
       <c r="S8" t="n">
-        <v>12.6835963702746</v>
+        <v>13.1083107414624</v>
       </c>
       <c r="T8" t="n">
-        <v>6.60031461689015</v>
+        <v>6.07380893713595</v>
       </c>
       <c r="U8" t="n">
-        <v>4.26325641347021</v>
+        <v>3.87191859069258</v>
       </c>
       <c r="V8" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W8" t="n">
-        <v>83.644400756499</v>
+        <v>83.3897001744513</v>
       </c>
       <c r="X8" t="n">
-        <v>89.5087791703359</v>
+        <v>89.2815470838727</v>
       </c>
       <c r="Y8" t="n">
-        <v>-5.86437841383687</v>
+        <v>-5.89184690942139</v>
       </c>
       <c r="Z8" t="n">
-        <v>173.153179926835</v>
+        <v>172.671247258324</v>
       </c>
       <c r="AA8" t="n">
         <v>0</v>
       </c>
       <c r="AB8" t="n">
-        <v>-6.8404574671284</v>
+        <v>-6.87249787490436</v>
       </c>
       <c r="AC8" t="n">
-        <v>172.689489955728</v>
+        <v>171.822948897077</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.976302152877496</v>
+        <v>0.93760734034872</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.378356630089031</v>
+        <v>-0.658563321840346</v>
       </c>
       <c r="AF8" t="n">
-        <v>-4.88807626095938</v>
+        <v>-4.95423956907267</v>
       </c>
       <c r="AG8" t="n">
-        <v>173.531536556924</v>
+        <v>172.012683936484</v>
       </c>
       <c r="AH8" t="s">
         <v>73</v>
@@ -2150,22 +2150,22 @@
         <v>0</v>
       </c>
       <c r="AN8" t="n">
-        <v>-4.88807626095938</v>
+        <v>-4.95423956907267</v>
       </c>
       <c r="AO8" t="n">
-        <v>173.531536556924</v>
+        <v>172.012683936484</v>
       </c>
       <c r="AP8" t="n">
-        <v>84.3217301479823</v>
+        <v>83.5292221837055</v>
       </c>
       <c r="AQ8" t="n">
-        <v>89.2098064089416</v>
+        <v>88.4834617527781</v>
       </c>
       <c r="AR8" t="n">
-        <v>-4.88807626095938</v>
+        <v>-4.95423956907267</v>
       </c>
       <c r="AS8" t="n">
-        <v>173.531536556924</v>
+        <v>172.012683936484</v>
       </c>
       <c r="AT8" t="s">
         <v>76</v>
@@ -2268,52 +2268,52 @@
         <v>4.36660785533764</v>
       </c>
       <c r="R9" t="n">
-        <v>7.59284523522869</v>
+        <v>8.0026390629484</v>
       </c>
       <c r="S9" t="n">
-        <v>2.79203927018599</v>
+        <v>3.17650055692725</v>
       </c>
       <c r="T9" t="n">
-        <v>11.7622045018175</v>
+        <v>11.3281622276035</v>
       </c>
       <c r="U9" t="n">
-        <v>3.06294734082283</v>
+        <v>2.65273024751581</v>
       </c>
       <c r="V9" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W9" t="n">
-        <v>92.1595440422817</v>
+        <v>91.8011028259032</v>
       </c>
       <c r="X9" t="n">
-        <v>74.2928730609067</v>
+        <v>73.9329244844568</v>
       </c>
       <c r="Y9" t="n">
-        <v>17.866670981375</v>
+        <v>17.8681783414465</v>
       </c>
       <c r="Z9" t="n">
-        <v>166.452417103188</v>
+        <v>165.73402731036</v>
       </c>
       <c r="AA9" t="n">
         <v>0</v>
       </c>
       <c r="AB9" t="n">
-        <v>20.8404359853222</v>
+        <v>20.8421942334653</v>
       </c>
       <c r="AC9" t="n">
-        <v>167.363238401295</v>
+        <v>166.30874409626</v>
       </c>
       <c r="AD9" t="n">
-        <v>4.92614621011625</v>
+        <v>4.89227419785055</v>
       </c>
       <c r="AE9" t="n">
-        <v>1.75286789930269</v>
+        <v>0.764451825306908</v>
       </c>
       <c r="AF9" t="n">
-        <v>22.7928171914912</v>
+        <v>22.760452539297</v>
       </c>
       <c r="AG9" t="n">
-        <v>168.205285002491</v>
+        <v>166.498479135667</v>
       </c>
       <c r="AH9" t="s">
         <v>73</v>
@@ -2334,22 +2334,22 @@
         <v>0</v>
       </c>
       <c r="AN9" t="n">
-        <v>22.7928171914912</v>
+        <v>22.760452539297</v>
       </c>
       <c r="AO9" t="n">
-        <v>168.205285002491</v>
+        <v>166.498479135667</v>
       </c>
       <c r="AP9" t="n">
-        <v>95.4990510969912</v>
+        <v>94.6294658374819</v>
       </c>
       <c r="AQ9" t="n">
-        <v>72.7062339055</v>
+        <v>71.8690132981849</v>
       </c>
       <c r="AR9" t="n">
-        <v>22.7928171914912</v>
+        <v>22.760452539297</v>
       </c>
       <c r="AS9" t="n">
-        <v>168.205285002491</v>
+        <v>166.498479135667</v>
       </c>
       <c r="AT9" t="s">
         <v>76</v>
@@ -2452,52 +2452,52 @@
         <v>4.36660785533764</v>
       </c>
       <c r="R10" t="n">
-        <v>-5.68122316188563</v>
+        <v>-9.05039241406247</v>
       </c>
       <c r="S10" t="n">
-        <v>13.581762825117</v>
+        <v>14.0266071378466</v>
       </c>
       <c r="T10" t="n">
-        <v>1.12368956519145</v>
+        <v>4.22936177423395</v>
       </c>
       <c r="U10" t="n">
-        <v>0.955307037766845</v>
+        <v>0.497474391585373</v>
       </c>
       <c r="V10" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W10" t="n">
-        <v>80.9931159482234</v>
+        <v>76.9033272048228</v>
       </c>
       <c r="X10" t="n">
-        <v>95.7211115524638</v>
+        <v>91.8818315187456</v>
       </c>
       <c r="Y10" t="n">
-        <v>-14.7279956042404</v>
+        <v>-14.9785043139229</v>
       </c>
       <c r="Z10" t="n">
-        <v>176.714227500687</v>
+        <v>168.785158723568</v>
       </c>
       <c r="AA10" t="n">
         <v>0</v>
       </c>
       <c r="AB10" t="n">
-        <v>-17.1793531040139</v>
+        <v>-17.4715569920994</v>
       </c>
       <c r="AC10" t="n">
-        <v>175.520068454747</v>
+        <v>168.734004303207</v>
       </c>
       <c r="AD10" t="n">
-        <v>-0.498976293604454</v>
+        <v>-0.574794372344873</v>
       </c>
       <c r="AE10" t="n">
-        <v>-0.352112444744192</v>
+        <v>0.138580619045571</v>
       </c>
       <c r="AF10" t="n">
-        <v>-15.2269718978448</v>
+        <v>-15.5532986862677</v>
       </c>
       <c r="AG10" t="n">
-        <v>176.362115055943</v>
+        <v>168.923739342614</v>
       </c>
       <c r="AH10" t="s">
         <v>73</v>
@@ -2518,31 +2518,31 @@
         <v>0</v>
       </c>
       <c r="AN10" t="n">
-        <v>-15.2269718978448</v>
+        <v>-15.5532986862677</v>
       </c>
       <c r="AO10" t="n">
-        <v>176.362115055943</v>
+        <v>168.923739342614</v>
       </c>
       <c r="AP10" t="n">
-        <v>80.5675715790491</v>
+        <v>76.6852203281731</v>
       </c>
       <c r="AQ10" t="n">
-        <v>95.7945434768939</v>
+        <v>92.2385190144409</v>
       </c>
       <c r="AR10" t="n">
-        <v>-15.2269718978448</v>
+        <v>-15.5532986862677</v>
       </c>
       <c r="AS10" t="n">
-        <v>176.362115055943</v>
+        <v>168.923739342614</v>
       </c>
       <c r="AT10" t="s">
         <v>76</v>
       </c>
       <c r="AU10" t="n">
-        <v>-0.215666589616726</v>
+        <v>-0.209528460864614</v>
       </c>
       <c r="AV10" t="n">
-        <v>-0.215666589616726</v>
+        <v>-0.209528460864614</v>
       </c>
       <c r="AW10" t="n">
         <v>1</v>
@@ -2551,7 +2551,7 @@
         <v>1</v>
       </c>
       <c r="AY10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AZ10" t="n">
         <v>0</v>
@@ -2572,7 +2572,7 @@
         <v>8</v>
       </c>
       <c r="BF10" t="n">
-        <v>-2.58799907540072</v>
+        <v>-2.51434153037536</v>
       </c>
       <c r="BG10"/>
       <c r="BH10"/>
@@ -2636,52 +2636,52 @@
         <v>4.04168960651118</v>
       </c>
       <c r="R11" t="n">
-        <v>8.45417626471137</v>
+        <v>8.98047298291742</v>
       </c>
       <c r="S11" t="n">
-        <v>-6.16354687135813</v>
+        <v>-5.79948184305096</v>
       </c>
       <c r="T11" t="n">
-        <v>6.26237576757176</v>
+        <v>5.6818360724727</v>
       </c>
       <c r="U11" t="n">
-        <v>-9.14961910059401</v>
+        <v>-9.45562114698717</v>
       </c>
       <c r="V11" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W11" t="n">
-        <v>105.070982388768</v>
+        <v>104.724829015962</v>
       </c>
       <c r="X11" t="n">
-        <v>70.9995747780216</v>
+        <v>70.7657273640226</v>
       </c>
       <c r="Y11" t="n">
-        <v>34.0714076107464</v>
+        <v>33.9591016519394</v>
       </c>
       <c r="Z11" t="n">
-        <v>176.07055716679</v>
+        <v>175.490556379985</v>
       </c>
       <c r="AA11" t="n">
         <v>0</v>
       </c>
       <c r="AB11" t="n">
-        <v>39.7423218898351</v>
+        <v>39.6113234991597</v>
       </c>
       <c r="AC11" t="n">
-        <v>175.008432659436</v>
+        <v>174.063939958375</v>
       </c>
       <c r="AD11" t="n">
-        <v>7.62329548525772</v>
+        <v>7.57048015305196</v>
       </c>
       <c r="AE11" t="n">
-        <v>-0.220077906157228</v>
+        <v>-1.23688138220271</v>
       </c>
       <c r="AF11" t="n">
-        <v>41.6947030960042</v>
+        <v>41.5295818049914</v>
       </c>
       <c r="AG11" t="n">
-        <v>175.850479260632</v>
+        <v>174.253674997782</v>
       </c>
       <c r="AH11" t="s">
         <v>73</v>
@@ -2702,22 +2702,22 @@
         <v>0</v>
       </c>
       <c r="AN11" t="n">
-        <v>41.6947030960042</v>
+        <v>41.5295818049914</v>
       </c>
       <c r="AO11" t="n">
-        <v>175.850479260632</v>
+        <v>174.253674997782</v>
       </c>
       <c r="AP11" t="n">
-        <v>108.772591178318</v>
+        <v>107.891628401387</v>
       </c>
       <c r="AQ11" t="n">
-        <v>67.0778880823141</v>
+        <v>66.3620465963952</v>
       </c>
       <c r="AR11" t="n">
-        <v>41.6947030960042</v>
+        <v>41.5295818049914</v>
       </c>
       <c r="AS11" t="n">
-        <v>175.850479260632</v>
+        <v>174.253674997782</v>
       </c>
       <c r="AT11" t="s">
         <v>76</v>
@@ -2820,52 +2820,52 @@
         <v>4.36660785533764</v>
       </c>
       <c r="R12" t="n">
-        <v>-0.103070263939211</v>
+        <v>0.230711257521621</v>
       </c>
       <c r="S12" t="n">
-        <v>8.71503778612408</v>
+        <v>8.99221483822378</v>
       </c>
       <c r="T12" t="n">
-        <v>0.566525293770441</v>
+        <v>0.227480976658517</v>
       </c>
       <c r="U12" t="n">
-        <v>3.2539565204658</v>
+        <v>2.96481935449112</v>
       </c>
       <c r="V12" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W12" t="n">
-        <v>84.2726193634709</v>
+        <v>83.7170859135011</v>
       </c>
       <c r="X12" t="n">
-        <v>91.4115507848919</v>
+        <v>90.8493200166982</v>
       </c>
       <c r="Y12" t="n">
-        <v>-7.13893142142102</v>
+        <v>-7.13223410319712</v>
       </c>
       <c r="Z12" t="n">
-        <v>175.684170148363</v>
+        <v>174.566405930199</v>
       </c>
       <c r="AA12" t="n">
         <v>0</v>
       </c>
       <c r="AB12" t="n">
-        <v>-8.32714966581202</v>
+        <v>-8.31933763234121</v>
       </c>
       <c r="AC12" t="n">
-        <v>174.701304275449</v>
+        <v>173.329358254882</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.764162961778017</v>
+        <v>0.731154776687601</v>
       </c>
       <c r="AE12" t="n">
-        <v>-0.140819271717673</v>
+        <v>-1.04731263591071</v>
       </c>
       <c r="AF12" t="n">
-        <v>-6.374768459643</v>
+        <v>-6.40107932650952</v>
       </c>
       <c r="AG12" t="n">
-        <v>175.543350876645</v>
+        <v>173.519093294289</v>
       </c>
       <c r="AH12" t="s">
         <v>73</v>
@@ -2886,22 +2886,22 @@
         <v>0</v>
       </c>
       <c r="AN12" t="n">
-        <v>-6.374768459643</v>
+        <v>-6.40107932650952</v>
       </c>
       <c r="AO12" t="n">
-        <v>175.543350876645</v>
+        <v>173.519093294289</v>
       </c>
       <c r="AP12" t="n">
-        <v>84.584291208501</v>
+        <v>83.5590069838896</v>
       </c>
       <c r="AQ12" t="n">
-        <v>90.959059668144</v>
+        <v>89.9600863103991</v>
       </c>
       <c r="AR12" t="n">
-        <v>-6.374768459643</v>
+        <v>-6.40107932650952</v>
       </c>
       <c r="AS12" t="n">
-        <v>175.543350876645</v>
+        <v>173.519093294289</v>
       </c>
       <c r="AT12" t="s">
         <v>76</v>
@@ -3004,52 +3004,52 @@
         <v>4.36660785533764</v>
       </c>
       <c r="R13" t="n">
-        <v>-6.88175771798916</v>
+        <v>-6.44780265080128</v>
       </c>
       <c r="S13" t="n">
-        <v>3.17154102324608</v>
+        <v>3.58268626667377</v>
       </c>
       <c r="T13" t="n">
-        <v>2.16006869446571</v>
+        <v>1.78319384794129</v>
       </c>
       <c r="U13" t="n">
-        <v>0.295534331495312</v>
+        <v>-0.0929066414405306</v>
       </c>
       <c r="V13" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W13" t="n">
-        <v>80.4523540983914</v>
+        <v>80.0962980011099</v>
       </c>
       <c r="X13" t="n">
-        <v>84.2745106213186</v>
+        <v>83.8840785738655</v>
       </c>
       <c r="Y13" t="n">
-        <v>-3.82215652292722</v>
+        <v>-3.78778057275559</v>
       </c>
       <c r="Z13" t="n">
-        <v>164.72686471971</v>
+        <v>163.980376574975</v>
       </c>
       <c r="AA13" t="n">
         <v>0</v>
       </c>
       <c r="AB13" t="n">
-        <v>-4.45832401710328</v>
+        <v>-4.41822646397024</v>
       </c>
       <c r="AC13" t="n">
-        <v>165.991644404217</v>
+        <v>164.914815494234</v>
       </c>
       <c r="AD13" t="n">
-        <v>1.31621371199295</v>
+        <v>1.28781241461705</v>
       </c>
       <c r="AE13" t="n">
-        <v>2.10682628570305</v>
+        <v>1.12417395866535</v>
       </c>
       <c r="AF13" t="n">
-        <v>-2.50594281093426</v>
+        <v>-2.49996815813855</v>
       </c>
       <c r="AG13" t="n">
-        <v>166.833691005413</v>
+        <v>165.104550533641</v>
       </c>
       <c r="AH13" t="s">
         <v>73</v>
@@ -3070,22 +3070,22 @@
         <v>1</v>
       </c>
       <c r="AN13" t="n">
-        <v>-6.57221634692945</v>
+        <v>-6.56624169413373</v>
       </c>
       <c r="AO13" t="n">
-        <v>166.833691005413</v>
+        <v>165.104550533641</v>
       </c>
       <c r="AP13" t="n">
-        <v>80.1307373292418</v>
+        <v>79.2691544197535</v>
       </c>
       <c r="AQ13" t="n">
-        <v>86.7029536761713</v>
+        <v>85.8353961138872</v>
       </c>
       <c r="AR13" t="n">
-        <v>-6.57221634692945</v>
+        <v>-6.56624169413373</v>
       </c>
       <c r="AS13" t="n">
-        <v>166.833691005413</v>
+        <v>165.104550533641</v>
       </c>
       <c r="AT13" t="s">
         <v>76</v>
@@ -3188,52 +3188,52 @@
         <v>4.36660785533764</v>
       </c>
       <c r="R14" t="n">
-        <v>-15.245244174749</v>
+        <v>-14.786750403476</v>
       </c>
       <c r="S14" t="n">
-        <v>4.17405053946832</v>
+        <v>4.53456158984908</v>
       </c>
       <c r="T14" t="n">
-        <v>-10.7312038123684</v>
+        <v>-11.1491536585899</v>
       </c>
       <c r="U14" t="n">
-        <v>7.51129500129918</v>
+        <v>7.11859047173502</v>
       </c>
       <c r="V14" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W14" t="n">
-        <v>64.8731069718277</v>
+        <v>64.5458531352596</v>
       </c>
       <c r="X14" t="n">
-        <v>98.168292644375</v>
+        <v>97.7683014035719</v>
       </c>
       <c r="Y14" t="n">
-        <v>-33.2951856725473</v>
+        <v>-33.2224482683123</v>
       </c>
       <c r="Z14" t="n">
-        <v>163.041399616203</v>
+        <v>162.314154538832</v>
       </c>
       <c r="AA14" t="n">
         <v>0</v>
       </c>
       <c r="AB14" t="n">
-        <v>-38.8369039957963</v>
+        <v>-38.7520600302765</v>
       </c>
       <c r="AC14" t="n">
-        <v>164.651914680339</v>
+        <v>163.590381553859</v>
       </c>
       <c r="AD14" t="n">
-        <v>-3.58933711707994</v>
+        <v>-3.61135345613244</v>
       </c>
       <c r="AE14" t="n">
-        <v>2.45256166533204</v>
+        <v>1.46596205443402</v>
       </c>
       <c r="AF14" t="n">
-        <v>-36.8845227896272</v>
+        <v>-36.8338017244448</v>
       </c>
       <c r="AG14" t="n">
-        <v>165.493961281535</v>
+        <v>163.780116593266</v>
       </c>
       <c r="AH14" t="s">
         <v>73</v>
@@ -3254,22 +3254,22 @@
         <v>0</v>
       </c>
       <c r="AN14" t="n">
-        <v>-36.8845227896272</v>
+        <v>-36.8338017244448</v>
       </c>
       <c r="AO14" t="n">
-        <v>165.493961281535</v>
+        <v>163.780116593266</v>
       </c>
       <c r="AP14" t="n">
-        <v>64.3047192459537</v>
+        <v>63.4731574344104</v>
       </c>
       <c r="AQ14" t="n">
-        <v>101.189242035581</v>
+        <v>100.306959158855</v>
       </c>
       <c r="AR14" t="n">
-        <v>-36.8845227896272</v>
+        <v>-36.8338017244448</v>
       </c>
       <c r="AS14" t="n">
-        <v>165.493961281535</v>
+        <v>163.780116593266</v>
       </c>
       <c r="AT14" t="s">
         <v>76</v>
@@ -3372,52 +3372,52 @@
         <v>4.36660785533764</v>
       </c>
       <c r="R15" t="n">
-        <v>-17.8480171010685</v>
+        <v>-17.3776995174184</v>
       </c>
       <c r="S15" t="n">
-        <v>-14.4897762539447</v>
+        <v>-14.1384162654208</v>
       </c>
       <c r="T15" t="n">
-        <v>-13.2768330293885</v>
+        <v>-13.7681964082168</v>
       </c>
       <c r="U15" t="n">
-        <v>-11.7628852734437</v>
+        <v>-12.0351504959748</v>
       </c>
       <c r="V15" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W15" t="n">
-        <v>81.5445143202511</v>
+        <v>81.108644989027</v>
       </c>
       <c r="X15" t="n">
-        <v>82.0500950679821</v>
+        <v>81.714366297929</v>
       </c>
       <c r="Y15" t="n">
-        <v>-0.505580747730932</v>
+        <v>-0.605721308902005</v>
       </c>
       <c r="Z15" t="n">
-        <v>163.594609388233</v>
+        <v>162.823011286956</v>
       </c>
       <c r="AA15" t="n">
         <v>0</v>
       </c>
       <c r="AB15" t="n">
-        <v>-0.589730634178105</v>
+        <v>-0.706538793728116</v>
       </c>
       <c r="AC15" t="n">
-        <v>165.091645870019</v>
+        <v>163.994857748139</v>
       </c>
       <c r="AD15" t="n">
-        <v>1.86823131972185</v>
+        <v>1.81744082100558</v>
       </c>
       <c r="AE15" t="n">
-        <v>2.33908308298143</v>
+        <v>1.36158150058958</v>
       </c>
       <c r="AF15" t="n">
-        <v>1.36265057199092</v>
+        <v>1.21171951210357</v>
       </c>
       <c r="AG15" t="n">
-        <v>165.933692471215</v>
+        <v>164.184592787546</v>
       </c>
       <c r="AH15" t="s">
         <v>73</v>
@@ -3438,22 +3438,22 @@
         <v>0</v>
       </c>
       <c r="AN15" t="n">
-        <v>1.36265057199092</v>
+        <v>1.21171951210357</v>
       </c>
       <c r="AO15" t="n">
-        <v>165.933692471215</v>
+        <v>164.184592787546</v>
       </c>
       <c r="AP15" t="n">
-        <v>83.6481715216028</v>
+        <v>82.6981561498246</v>
       </c>
       <c r="AQ15" t="n">
-        <v>82.2855209496119</v>
+        <v>81.486436637721</v>
       </c>
       <c r="AR15" t="n">
-        <v>1.36265057199092</v>
+        <v>1.21171951210357</v>
       </c>
       <c r="AS15" t="n">
-        <v>165.933692471215</v>
+        <v>164.184592787546</v>
       </c>
       <c r="AT15" t="s">
         <v>76</v>
@@ -3556,52 +3556,52 @@
         <v>4.36660785533764</v>
       </c>
       <c r="R16" t="n">
-        <v>-0.254325413552674</v>
+        <v>-3.37223231229803</v>
       </c>
       <c r="S16" t="n">
-        <v>5.06144149762435</v>
+        <v>5.36518709307108</v>
       </c>
       <c r="T16" t="n">
-        <v>-0.657282145641784</v>
+        <v>2.60847014545934</v>
       </c>
       <c r="U16" t="n">
-        <v>-2.2396517235907</v>
+        <v>-2.5368186863159</v>
       </c>
       <c r="V16" t="n">
-        <v>85.4463422202071</v>
+        <v>84.2678900828018</v>
       </c>
       <c r="W16" t="n">
-        <v>89.6149724579139</v>
+        <v>85.6157803844885</v>
       </c>
       <c r="X16" t="n">
-        <v>88.9817619358044</v>
+        <v>84.8413031027447</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.633210522109508</v>
+        <v>0.774477281743785</v>
       </c>
       <c r="Z16" t="n">
-        <v>178.596734393718</v>
+        <v>170.457083487233</v>
       </c>
       <c r="AA16" t="n">
         <v>0</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.738603367410311</v>
+        <v>0.903382853419824</v>
       </c>
       <c r="AC16" t="n">
-        <v>177.016421262498</v>
+        <v>170.062971184401</v>
       </c>
       <c r="AD16" t="n">
-        <v>2.05777405146983</v>
+        <v>2.04716387750773</v>
       </c>
       <c r="AE16" t="n">
-        <v>-0.738266530024218</v>
+        <v>-0.204377263424901</v>
       </c>
       <c r="AF16" t="n">
-        <v>2.69098457357933</v>
+        <v>2.82164115925152</v>
       </c>
       <c r="AG16" t="n">
-        <v>177.858467863694</v>
+        <v>170.252706223808</v>
       </c>
       <c r="AH16" t="s">
         <v>73</v>
@@ -3622,31 +3622,31 @@
         <v>0</v>
       </c>
       <c r="AN16" t="n">
-        <v>2.69098457357933</v>
+        <v>2.82164115925152</v>
       </c>
       <c r="AO16" t="n">
-        <v>177.858467863694</v>
+        <v>170.252706223808</v>
       </c>
       <c r="AP16" t="n">
-        <v>90.2747262186367</v>
+        <v>86.5371736915299</v>
       </c>
       <c r="AQ16" t="n">
-        <v>87.5837416450574</v>
+        <v>83.7155325322784</v>
       </c>
       <c r="AR16" t="n">
-        <v>2.69098457357933</v>
+        <v>2.82164115925152</v>
       </c>
       <c r="AS16" t="n">
-        <v>177.858467863694</v>
+        <v>170.252706223808</v>
       </c>
       <c r="AT16" t="s">
         <v>76</v>
       </c>
       <c r="AU16" t="n">
-        <v>-0.0113874818808137</v>
+        <v>-0.00382177638505476</v>
       </c>
       <c r="AV16" t="n">
-        <v>-0.0113874818808137</v>
+        <v>-0.00382177638505476</v>
       </c>
       <c r="AW16" t="n">
         <v>1</v>
@@ -3655,7 +3655,7 @@
         <v>1</v>
       </c>
       <c r="AY16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AZ16" t="n">
         <v>0</v>
@@ -3676,7 +3676,7 @@
         <v>8</v>
       </c>
       <c r="BF16" t="n">
-        <v>-0.136649782569765</v>
+        <v>-0.0458613166206572</v>
       </c>
       <c r="BG16"/>
       <c r="BH16"/>

</xml_diff>

<commit_message>
Update model outputs 2026-07-25 13:32:09
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -894,7 +894,7 @@
         <v>63</v>
       </c>
       <c r="I2" t="n">
-        <v>3.9</v>
+        <v>0.1</v>
       </c>
       <c r="J2" t="s">
         <v>64</v>
@@ -906,52 +906,52 @@
         <v>4.36660785533764</v>
       </c>
       <c r="M2" t="n">
-        <v>-9.05039241406247</v>
+        <v>-8.231423515375</v>
       </c>
       <c r="N2" t="n">
-        <v>-3.37223231229803</v>
+        <v>-2.84772393333651</v>
       </c>
       <c r="O2" t="n">
-        <v>4.22936177423395</v>
+        <v>3.70579755184498</v>
       </c>
       <c r="P2" t="n">
-        <v>2.60847014545934</v>
+        <v>1.82362378307202</v>
       </c>
       <c r="Q2" t="n">
-        <v>84.2678900828018</v>
+        <v>84.5026220881096</v>
       </c>
       <c r="R2" t="n">
-        <v>74.7923314509488</v>
+        <v>76.6308787173314</v>
       </c>
       <c r="S2" t="n">
-        <v>74.482992068601</v>
+        <v>75.7657966752593</v>
       </c>
       <c r="T2" t="n">
-        <v>0.309339382347787</v>
+        <v>0.865082042072103</v>
       </c>
       <c r="U2" t="n">
-        <v>149.27532351955</v>
+        <v>152.396675392591</v>
       </c>
       <c r="V2" t="n">
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>0.360826457389771</v>
+        <v>1.00906805406835</v>
       </c>
       <c r="X2" t="n">
-        <v>153.2261744013</v>
+        <v>155.803550931902</v>
       </c>
       <c r="Y2" t="n">
-        <v>1.96974538087368</v>
+        <v>2.09069960238078</v>
       </c>
       <c r="Z2" t="n">
-        <v>4.14058592115706</v>
+        <v>3.73075692018166</v>
       </c>
       <c r="AA2" t="n">
-        <v>2.27908476322146</v>
+        <v>2.95578164445289</v>
       </c>
       <c r="AB2" t="n">
-        <v>153.415909440707</v>
+        <v>156.127432312772</v>
       </c>
       <c r="AC2" t="s">
         <v>65</v>
@@ -972,22 +972,22 @@
         <v>0</v>
       </c>
       <c r="AI2" t="n">
-        <v>2.27908476322146</v>
+        <v>2.95578164445289</v>
       </c>
       <c r="AJ2" t="n">
-        <v>153.415909440707</v>
+        <v>156.127432312772</v>
       </c>
       <c r="AK2" t="n">
-        <v>77.8474971019642</v>
+        <v>79.5416069786126</v>
       </c>
       <c r="AL2" t="n">
-        <v>75.5684123387427</v>
+        <v>76.5858253341598</v>
       </c>
       <c r="AM2" t="n">
-        <v>2.27908476322146</v>
+        <v>2.95578164445289</v>
       </c>
       <c r="AN2" t="n">
-        <v>153.415909440707</v>
+        <v>156.127432312772</v>
       </c>
       <c r="AO2" t="s">
         <v>68</v>
@@ -1044,10 +1044,10 @@
         <v>0</v>
       </c>
       <c r="BG2" t="n">
-        <v>-6.5</v>
+        <v>-1.5</v>
       </c>
       <c r="BH2" t="n">
-        <v>171.5</v>
+        <v>183.5</v>
       </c>
     </row>
     <row r="3">
@@ -1076,7 +1076,7 @@
         <v>63</v>
       </c>
       <c r="I3" t="n">
-        <v>3.9</v>
+        <v>0.1</v>
       </c>
       <c r="J3" t="s">
         <v>73</v>
@@ -1088,52 +1088,52 @@
         <v>4.04168960651118</v>
       </c>
       <c r="M3" t="n">
-        <v>3.17650055692725</v>
+        <v>3.09488116534422</v>
       </c>
       <c r="N3" t="n">
-        <v>-17.3776995174184</v>
+        <v>-17.4710723134453</v>
       </c>
       <c r="O3" t="n">
-        <v>2.65273024751581</v>
+        <v>2.72850384716259</v>
       </c>
       <c r="P3" t="n">
-        <v>-13.7681964082168</v>
+        <v>-13.6690780343948</v>
       </c>
       <c r="Q3" t="n">
-        <v>84.2678900828018</v>
+        <v>84.5026220881096</v>
       </c>
       <c r="R3" t="n">
-        <v>103.233431851201</v>
+        <v>103.287426091104</v>
       </c>
       <c r="S3" t="n">
-        <v>62.216615514612</v>
+        <v>62.2822011242462</v>
       </c>
       <c r="T3" t="n">
-        <v>41.0168163365894</v>
+        <v>41.0052249668581</v>
       </c>
       <c r="U3" t="n">
-        <v>165.450047365814</v>
+        <v>165.56962721535</v>
       </c>
       <c r="V3" t="n">
         <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>47.8437385495877</v>
+        <v>47.8302178887371</v>
       </c>
       <c r="X3" t="n">
-        <v>166.083016270805</v>
+        <v>166.274367011953</v>
       </c>
       <c r="Y3" t="n">
-        <v>8.74518051882998</v>
+        <v>8.77170651226357</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.822703944398826</v>
+        <v>1.02862117747251</v>
       </c>
       <c r="AA3" t="n">
-        <v>49.7619968554194</v>
+        <v>49.7769314791217</v>
       </c>
       <c r="AB3" t="n">
-        <v>166.272751310212</v>
+        <v>166.598248392823</v>
       </c>
       <c r="AC3" t="s">
         <v>65</v>
@@ -1154,22 +1154,22 @@
         <v>0</v>
       </c>
       <c r="AI3" t="n">
-        <v>49.7619968554194</v>
+        <v>49.7769314791217</v>
       </c>
       <c r="AJ3" t="n">
-        <v>166.272751310212</v>
+        <v>166.598248392823</v>
       </c>
       <c r="AK3" t="n">
-        <v>108.017374082816</v>
+        <v>108.187589935972</v>
       </c>
       <c r="AL3" t="n">
-        <v>58.2553772273965</v>
+        <v>58.4106584568506</v>
       </c>
       <c r="AM3" t="n">
-        <v>49.7619968554194</v>
+        <v>49.7769314791217</v>
       </c>
       <c r="AN3" t="n">
-        <v>166.272751310212</v>
+        <v>166.598248392823</v>
       </c>
       <c r="AO3" t="s">
         <v>68</v>
@@ -1226,10 +1226,10 @@
         <v>0</v>
       </c>
       <c r="BG3" t="n">
-        <v>-41.5</v>
+        <v>-39.5</v>
       </c>
       <c r="BH3" t="n">
-        <v>170.5</v>
+        <v>175.5</v>
       </c>
     </row>
     <row r="4">
@@ -1258,7 +1258,7 @@
         <v>77</v>
       </c>
       <c r="I4" t="n">
-        <v>5.2</v>
+        <v>0.3</v>
       </c>
       <c r="J4" t="s">
         <v>73</v>
@@ -1270,52 +1270,52 @@
         <v>4.04168960651118</v>
       </c>
       <c r="M4" t="n">
-        <v>8.98047298291742</v>
+        <v>8.86976323115598</v>
       </c>
       <c r="N4" t="n">
-        <v>-14.786750403476</v>
+        <v>-14.880627213056</v>
       </c>
       <c r="O4" t="n">
-        <v>5.6818360724727</v>
+        <v>5.78725224626711</v>
       </c>
       <c r="P4" t="n">
-        <v>-11.1491536585899</v>
+        <v>-11.0566604250312</v>
       </c>
       <c r="Q4" t="n">
-        <v>84.2678900828018</v>
+        <v>84.5026220881096</v>
       </c>
       <c r="R4" t="n">
-        <v>106.418361527565</v>
+        <v>106.449890547552</v>
       </c>
       <c r="S4" t="n">
-        <v>61.7784588035975</v>
+        <v>61.8138978255309</v>
       </c>
       <c r="T4" t="n">
-        <v>44.6399027239672</v>
+        <v>44.6359927220215</v>
       </c>
       <c r="U4" t="n">
-        <v>168.196820331162</v>
+        <v>168.263788373083</v>
       </c>
       <c r="V4" t="n">
         <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>52.0698587934848</v>
+        <v>52.0652980028744</v>
       </c>
       <c r="X4" t="n">
-        <v>168.266350342075</v>
+        <v>168.415881408437</v>
       </c>
       <c r="Y4" t="n">
-        <v>9.34821437534936</v>
+        <v>9.37601887123745</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.2592650503195</v>
+        <v>0.475974416224157</v>
       </c>
       <c r="AA4" t="n">
-        <v>53.9881170993165</v>
+        <v>54.0120115932589</v>
       </c>
       <c r="AB4" t="n">
-        <v>168.456085381482</v>
+        <v>168.739762789307</v>
       </c>
       <c r="AC4" t="s">
         <v>65</v>
@@ -1336,22 +1336,22 @@
         <v>0</v>
       </c>
       <c r="AI4" t="n">
-        <v>53.9881170993165</v>
+        <v>54.0120115932589</v>
       </c>
       <c r="AJ4" t="n">
-        <v>168.456085381482</v>
+        <v>168.739762789307</v>
       </c>
       <c r="AK4" t="n">
-        <v>111.222101240399</v>
+        <v>111.375887191283</v>
       </c>
       <c r="AL4" t="n">
-        <v>57.2339841410826</v>
+        <v>57.3638755980243</v>
       </c>
       <c r="AM4" t="n">
-        <v>53.9881170993165</v>
+        <v>54.0120115932589</v>
       </c>
       <c r="AN4" t="n">
-        <v>168.456085381482</v>
+        <v>168.739762789307</v>
       </c>
       <c r="AO4" t="s">
         <v>68</v>
@@ -1408,10 +1408,10 @@
         <v>0</v>
       </c>
       <c r="BG4" t="n">
-        <v>-53.5</v>
+        <v>-60.5</v>
       </c>
       <c r="BH4" t="n">
-        <v>169.5</v>
+        <v>174.5</v>
       </c>
     </row>
     <row r="5">
@@ -1452,52 +1452,52 @@
         <v>4.04168960651118</v>
       </c>
       <c r="M5" t="n">
-        <v>3.58268626667377</v>
+        <v>3.49664833230434</v>
       </c>
       <c r="N5" t="n">
-        <v>8.99221483822378</v>
+        <v>8.93391889397961</v>
       </c>
       <c r="O5" t="n">
-        <v>-0.0929066414405306</v>
+        <v>-0.0109544506269164</v>
       </c>
       <c r="P5" t="n">
-        <v>2.96481935449112</v>
+        <v>3.01989457768139</v>
       </c>
       <c r="Q5" t="n">
-        <v>84.2678900828018</v>
+        <v>84.5026220881096</v>
       </c>
       <c r="R5" t="n">
-        <v>86.90660179824</v>
+        <v>87.0002206459882</v>
       </c>
       <c r="S5" t="n">
-        <v>91.3321667592105</v>
+        <v>91.4266506294606</v>
       </c>
       <c r="T5" t="n">
-        <v>-4.42556496097048</v>
+        <v>-4.4264299834724</v>
       </c>
       <c r="U5" t="n">
-        <v>178.238768557451</v>
+        <v>178.426871275449</v>
       </c>
       <c r="V5" t="n">
         <v>0</v>
       </c>
       <c r="W5" t="n">
-        <v>-5.16216498104967</v>
+        <v>-5.16317397965361</v>
       </c>
       <c r="X5" t="n">
-        <v>176.248418019661</v>
+        <v>176.494235699016</v>
       </c>
       <c r="Y5" t="n">
-        <v>1.1816582857525</v>
+        <v>1.20996959420333</v>
       </c>
       <c r="Z5" t="n">
-        <v>-1.80061549838226</v>
+        <v>-1.60875419556273</v>
       </c>
       <c r="AA5" t="n">
-        <v>-3.24390667521797</v>
+        <v>-3.21646038926907</v>
       </c>
       <c r="AB5" t="n">
-        <v>176.438153059068</v>
+        <v>176.818117079886</v>
       </c>
       <c r="AC5" t="s">
         <v>65</v>
@@ -1518,22 +1518,22 @@
         <v>0</v>
       </c>
       <c r="AI5" t="n">
-        <v>-3.24390667521797</v>
+        <v>-3.21646038926907</v>
       </c>
       <c r="AJ5" t="n">
-        <v>176.438153059068</v>
+        <v>176.818117079886</v>
       </c>
       <c r="AK5" t="n">
-        <v>86.5971231919252</v>
+        <v>86.8008283453085</v>
       </c>
       <c r="AL5" t="n">
-        <v>89.8410298671431</v>
+        <v>90.0172887345775</v>
       </c>
       <c r="AM5" t="n">
-        <v>-3.24390667521797</v>
+        <v>-3.21646038926907</v>
       </c>
       <c r="AN5" t="n">
-        <v>176.438153059068</v>
+        <v>176.818117079886</v>
       </c>
       <c r="AO5" t="s">
         <v>68</v>
@@ -1590,7 +1590,7 @@
         <v>0</v>
       </c>
       <c r="BG5" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="BH5" t="n">
         <v>184.5</v>
@@ -1634,52 +1634,52 @@
         <v>4.36660785533764</v>
       </c>
       <c r="M6" t="n">
-        <v>14.0266071378466</v>
+        <v>13.9328444129302</v>
       </c>
       <c r="N6" t="n">
-        <v>-6.44780265080128</v>
+        <v>-6.53669914053842</v>
       </c>
       <c r="O6" t="n">
-        <v>0.497474391585373</v>
+        <v>0.584067706476322</v>
       </c>
       <c r="P6" t="n">
-        <v>1.78319384794129</v>
+        <v>1.87318109154961</v>
       </c>
       <c r="Q6" t="n">
-        <v>84.2678900828018</v>
+        <v>84.5026220881096</v>
       </c>
       <c r="R6" t="n">
-        <v>98.6946073003759</v>
+        <v>98.745589337159</v>
       </c>
       <c r="S6" t="n">
-        <v>75.1393091127463</v>
+        <v>75.1985513134261</v>
       </c>
       <c r="T6" t="n">
-        <v>23.5552981876296</v>
+        <v>23.547038023733</v>
       </c>
       <c r="U6" t="n">
-        <v>173.833916413122</v>
+        <v>173.944140650585</v>
       </c>
       <c r="V6" t="n">
         <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>27.4758898569414</v>
+        <v>27.4662548545901</v>
       </c>
       <c r="X6" t="n">
-        <v>172.747122540588</v>
+        <v>172.931036763735</v>
       </c>
       <c r="Y6" t="n">
-        <v>5.83884997514354</v>
+        <v>5.86593042124168</v>
       </c>
       <c r="Z6" t="n">
-        <v>-0.897058833127202</v>
+        <v>-0.689222505979491</v>
       </c>
       <c r="AA6" t="n">
-        <v>29.3941481627731</v>
+        <v>29.4129684449746</v>
       </c>
       <c r="AB6" t="n">
-        <v>172.936857579995</v>
+        <v>173.254918144606</v>
       </c>
       <c r="AC6" t="s">
         <v>65</v>
@@ -1700,22 +1700,22 @@
         <v>1</v>
       </c>
       <c r="AI6" t="n">
-        <v>34.5952331339132</v>
+        <v>34.6140534161147</v>
       </c>
       <c r="AJ6" t="n">
-        <v>172.936857579995</v>
+        <v>173.254918144606</v>
       </c>
       <c r="AK6" t="n">
-        <v>103.766045356954</v>
+        <v>103.93448578036</v>
       </c>
       <c r="AL6" t="n">
-        <v>69.170812223041</v>
+        <v>69.3204323642455</v>
       </c>
       <c r="AM6" t="n">
-        <v>34.5952331339132</v>
+        <v>34.6140534161147</v>
       </c>
       <c r="AN6" t="n">
-        <v>172.936857579995</v>
+        <v>173.254918144606</v>
       </c>
       <c r="AO6" t="s">
         <v>68</v>
@@ -1772,10 +1772,10 @@
         <v>0</v>
       </c>
       <c r="BG6" t="n">
-        <v>-38.5</v>
+        <v>-40.5</v>
       </c>
       <c r="BH6" t="n">
-        <v>190.5</v>
+        <v>188.5</v>
       </c>
     </row>
     <row r="7">
@@ -1804,7 +1804,7 @@
         <v>63</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="J7" t="s">
         <v>73</v>
@@ -1816,52 +1816,52 @@
         <v>4.04168960651118</v>
       </c>
       <c r="M7" t="n">
-        <v>-5.79948184305096</v>
+        <v>-5.87348772315684</v>
       </c>
       <c r="N7" t="n">
-        <v>0.230711257521621</v>
+        <v>0.161880397188689</v>
       </c>
       <c r="O7" t="n">
-        <v>-9.45562114698717</v>
+        <v>-9.38323686146525</v>
       </c>
       <c r="P7" t="n">
-        <v>0.227480976658517</v>
+        <v>0.293689850565083</v>
       </c>
       <c r="Q7" t="n">
-        <v>84.2678900828018</v>
+        <v>84.5026220881096</v>
       </c>
       <c r="R7" t="n">
-        <v>80.2617720663479</v>
+        <v>80.3562893176433</v>
       </c>
       <c r="S7" t="n">
-        <v>91.933377684055</v>
+        <v>92.026894543508</v>
       </c>
       <c r="T7" t="n">
-        <v>-11.6716056177071</v>
+        <v>-11.6706052258647</v>
       </c>
       <c r="U7" t="n">
-        <v>172.195149750403</v>
+        <v>172.383183861151</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>-13.6142513608337</v>
+        <v>-13.6130844617413</v>
       </c>
       <c r="X7" t="n">
-        <v>171.4445121193</v>
+        <v>171.690275264644</v>
       </c>
       <c r="Y7" t="n">
-        <v>-0.0243874372948847</v>
+        <v>0.00423435450792731</v>
       </c>
       <c r="Z7" t="n">
-        <v>-0.560902591695934</v>
+        <v>-0.369027215637193</v>
       </c>
       <c r="AA7" t="n">
-        <v>-11.695993055002</v>
+        <v>-11.6663708713568</v>
       </c>
       <c r="AB7" t="n">
-        <v>171.634247158707</v>
+        <v>172.014156645514</v>
       </c>
       <c r="AC7" t="s">
         <v>65</v>
@@ -1882,22 +1882,22 @@
         <v>0</v>
       </c>
       <c r="AI7" t="n">
-        <v>-11.695993055002</v>
+        <v>-11.6663708713568</v>
       </c>
       <c r="AJ7" t="n">
-        <v>171.634247158707</v>
+        <v>172.014156645514</v>
       </c>
       <c r="AK7" t="n">
-        <v>79.9691270518525</v>
+        <v>80.1738928870786</v>
       </c>
       <c r="AL7" t="n">
-        <v>91.6651201068545</v>
+        <v>91.8402637584354</v>
       </c>
       <c r="AM7" t="n">
-        <v>-11.695993055002</v>
+        <v>-11.6663708713568</v>
       </c>
       <c r="AN7" t="n">
-        <v>171.634247158707</v>
+        <v>172.014156645514</v>
       </c>
       <c r="AO7" t="s">
         <v>68</v>
@@ -1985,7 +1985,9 @@
       <c r="H8" t="s">
         <v>77</v>
       </c>
-      <c r="I8"/>
+      <c r="I8" t="n">
+        <v>0.3</v>
+      </c>
       <c r="J8" t="s">
         <v>73</v>
       </c>
@@ -1996,52 +1998,52 @@
         <v>4.04168960651118</v>
       </c>
       <c r="M8" t="n">
-        <v>0.972883879086474</v>
+        <v>0.865985744184762</v>
       </c>
       <c r="N8" t="n">
-        <v>13.1083107414624</v>
+        <v>13.0166116730311</v>
       </c>
       <c r="O8" t="n">
-        <v>6.07380893713595</v>
+        <v>6.18968514004415</v>
       </c>
       <c r="P8" t="n">
-        <v>3.87191859069258</v>
+        <v>3.95504012487703</v>
       </c>
       <c r="Q8" t="n">
-        <v>84.2678900828018</v>
+        <v>84.5026220881096</v>
       </c>
       <c r="R8" t="n">
-        <v>83.3897001744513</v>
+        <v>83.4344125106729</v>
       </c>
       <c r="S8" t="n">
-        <v>89.2815470838727</v>
+        <v>89.3087038178409</v>
       </c>
       <c r="T8" t="n">
-        <v>-5.89184690942139</v>
+        <v>-5.87429130716799</v>
       </c>
       <c r="U8" t="n">
-        <v>172.671247258324</v>
+        <v>172.743116328514</v>
       </c>
       <c r="V8" t="n">
         <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>-6.87249787490436</v>
+        <v>-6.85202028255786</v>
       </c>
       <c r="X8" t="n">
-        <v>171.822948897077</v>
+        <v>171.976375655634</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.93760734034872</v>
+        <v>0.968984614994671</v>
       </c>
       <c r="Z8" t="n">
-        <v>-0.658563321840346</v>
+        <v>-0.44285929200915</v>
       </c>
       <c r="AA8" t="n">
-        <v>-4.95423956907267</v>
+        <v>-4.90530669217332</v>
       </c>
       <c r="AB8" t="n">
-        <v>172.012683936484</v>
+        <v>172.300257036505</v>
       </c>
       <c r="AC8" t="s">
         <v>65</v>
@@ -2062,22 +2064,22 @@
         <v>0</v>
       </c>
       <c r="AI8" t="n">
-        <v>-4.95423956907267</v>
+        <v>-4.90530669217332</v>
       </c>
       <c r="AJ8" t="n">
-        <v>172.012683936484</v>
+        <v>172.300257036505</v>
       </c>
       <c r="AK8" t="n">
-        <v>83.5292221837055</v>
+        <v>83.6974751721657</v>
       </c>
       <c r="AL8" t="n">
-        <v>88.4834617527781</v>
+        <v>88.602781864339</v>
       </c>
       <c r="AM8" t="n">
-        <v>-4.95423956907267</v>
+        <v>-4.90530669217332</v>
       </c>
       <c r="AN8" t="n">
-        <v>172.012683936484</v>
+        <v>172.300257036505</v>
       </c>
       <c r="AO8" t="s">
         <v>68</v>
@@ -2133,7 +2135,9 @@
       <c r="BF8" t="n">
         <v>0</v>
       </c>
-      <c r="BG8"/>
+      <c r="BG8" t="n">
+        <v>1</v>
+      </c>
       <c r="BH8"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-07-25 13:40:55
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -32,12 +32,6 @@
     <t xml:space="preserve">Projected Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Projected Home Score</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Projected Away Score</t>
-  </si>
-  <si>
     <t xml:space="preserve">Market Line</t>
   </si>
   <si>
@@ -48,18 +42,6 @@
   </si>
   <si>
     <t xml:space="preserve">Forecast Rain mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Round</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Player Margin Adjustment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Home Lineup Changes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Away Lineup Changes</t>
   </si>
   <si>
     <t xml:space="preserve">13:05</t>
@@ -475,16 +457,10 @@
     <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="15.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="20.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="20.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="12.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="14.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="16.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="5.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="24.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="19.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="19.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="12.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="14.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,73 +494,37 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" t="s">
-        <v>15</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
         <v>46228</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E2" t="n">
-        <v>2.95578164445289</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
-        <v>156.127432312772</v>
+        <v>156.1</v>
       </c>
       <c r="G2" t="n">
-        <v>79.5416069786126</v>
+        <v>-1.5</v>
       </c>
       <c r="H2" t="n">
-        <v>76.5858253341598</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-1.5</v>
+        <v>183.5</v>
+      </c>
+      <c r="I2" t="s">
+        <v>13</v>
       </c>
       <c r="J2" t="n">
-        <v>183.5</v>
-      </c>
-      <c r="K2" t="s">
-        <v>19</v>
-      </c>
-      <c r="L2" t="n">
         <v>0.1</v>
-      </c>
-      <c r="M2" t="n">
-        <v>21</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>2</v>
-      </c>
-      <c r="P2" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -592,49 +532,31 @@
         <v>46228</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E3" t="n">
-        <v>49.7769314791217</v>
+        <v>49.8</v>
       </c>
       <c r="F3" t="n">
-        <v>166.598248392823</v>
+        <v>166.6</v>
       </c>
       <c r="G3" t="n">
-        <v>108.187589935972</v>
+        <v>-39.5</v>
       </c>
       <c r="H3" t="n">
-        <v>58.4106584568506</v>
-      </c>
-      <c r="I3" t="n">
-        <v>-39.5</v>
+        <v>175.5</v>
+      </c>
+      <c r="I3" t="s">
+        <v>13</v>
       </c>
       <c r="J3" t="n">
-        <v>175.5</v>
-      </c>
-      <c r="K3" t="s">
-        <v>19</v>
-      </c>
-      <c r="L3" t="n">
         <v>0.1</v>
-      </c>
-      <c r="M3" t="n">
-        <v>21</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -642,49 +564,31 @@
         <v>46228</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E4" t="n">
-        <v>54.0120115932589</v>
+        <v>54</v>
       </c>
       <c r="F4" t="n">
-        <v>168.739762789307</v>
+        <v>168.7</v>
       </c>
       <c r="G4" t="n">
-        <v>111.375887191283</v>
+        <v>-60.5</v>
       </c>
       <c r="H4" t="n">
-        <v>57.3638755980243</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-60.5</v>
+        <v>174.5</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
       </c>
       <c r="J4" t="n">
-        <v>174.5</v>
-      </c>
-      <c r="K4" t="s">
-        <v>26</v>
-      </c>
-      <c r="L4" t="n">
         <v>0.3</v>
-      </c>
-      <c r="M4" t="n">
-        <v>21</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P4" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -692,49 +596,31 @@
         <v>46228</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="E5" t="n">
-        <v>-3.21646038926907</v>
+        <v>-3.2</v>
       </c>
       <c r="F5" t="n">
-        <v>176.818117079886</v>
+        <v>176.8</v>
       </c>
       <c r="G5" t="n">
-        <v>86.8008283453085</v>
+        <v>11.5</v>
       </c>
       <c r="H5" t="n">
-        <v>90.0172887345775</v>
-      </c>
-      <c r="I5" t="n">
-        <v>11.5</v>
+        <v>184.5</v>
+      </c>
+      <c r="I5" t="s">
+        <v>24</v>
       </c>
       <c r="J5" t="n">
-        <v>184.5</v>
-      </c>
-      <c r="K5" t="s">
-        <v>30</v>
-      </c>
-      <c r="L5" t="n">
         <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>21</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>1</v>
-      </c>
-      <c r="P5" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -742,49 +628,31 @@
         <v>46229</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E6" t="n">
-        <v>34.6140534161147</v>
+        <v>34.6</v>
       </c>
       <c r="F6" t="n">
-        <v>173.254918144606</v>
+        <v>173.3</v>
       </c>
       <c r="G6" t="n">
-        <v>103.93448578036</v>
+        <v>-40.5</v>
       </c>
       <c r="H6" t="n">
-        <v>69.3204323642455</v>
-      </c>
-      <c r="I6" t="n">
-        <v>-40.5</v>
+        <v>188.5</v>
+      </c>
+      <c r="I6" t="s">
+        <v>28</v>
       </c>
       <c r="J6" t="n">
-        <v>188.5</v>
-      </c>
-      <c r="K6" t="s">
-        <v>34</v>
-      </c>
-      <c r="L6" t="n">
         <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>21</v>
-      </c>
-      <c r="N6" t="n">
-        <v>5.20108497114003</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -792,49 +660,31 @@
         <v>46229</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E7" t="n">
-        <v>-11.6663708713568</v>
+        <v>-11.7</v>
       </c>
       <c r="F7" t="n">
-        <v>172.014156645514</v>
+        <v>172</v>
       </c>
       <c r="G7" t="n">
-        <v>80.1738928870786</v>
+        <v>12.5</v>
       </c>
       <c r="H7" t="n">
-        <v>91.8402637584354</v>
-      </c>
-      <c r="I7" t="n">
-        <v>12.5</v>
+        <v>176.5</v>
+      </c>
+      <c r="I7" t="s">
+        <v>13</v>
       </c>
       <c r="J7" t="n">
-        <v>176.5</v>
-      </c>
-      <c r="K7" t="s">
-        <v>19</v>
-      </c>
-      <c r="L7" t="n">
         <v>0.2</v>
-      </c>
-      <c r="M7" t="n">
-        <v>21</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>2</v>
-      </c>
-      <c r="P7" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -842,47 +692,29 @@
         <v>46233</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E8" t="n">
-        <v>-4.90530669217332</v>
+        <v>-4.9</v>
       </c>
       <c r="F8" t="n">
-        <v>172.300257036505</v>
+        <v>172.3</v>
       </c>
       <c r="G8" t="n">
-        <v>83.6974751721657</v>
-      </c>
-      <c r="H8" t="n">
-        <v>88.602781864339</v>
-      </c>
-      <c r="I8" t="n">
         <v>1</v>
       </c>
-      <c r="J8"/>
-      <c r="K8" t="s">
-        <v>26</v>
-      </c>
-      <c r="L8" t="n">
+      <c r="H8"/>
+      <c r="I8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" t="n">
         <v>0.3</v>
-      </c>
-      <c r="M8" t="n">
-        <v>21</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-07-29 08:21:10
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,79 +44,73 @@
     <t xml:space="preserve">Forecast Rain mm</t>
   </si>
   <si>
+    <t xml:space="preserve">19:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collingwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">western bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optus Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marvel Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hawthorn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UTAS Stadium</t>
+  </si>
+  <si>
     <t xml:space="preserve">13:05</t>
   </si>
   <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marvel Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:35</t>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
   </si>
   <si>
     <t xml:space="preserve">greater western sydney</t>
   </si>
   <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENGIE Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gabba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
+    <t xml:space="preserve">Adelaide Oval</t>
   </si>
 </sst>
 </file>
@@ -453,8 +447,8 @@
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="5.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="22.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="13.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="22.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="15.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
@@ -497,7 +491,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46228</v>
+        <v>46233</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -509,27 +503,25 @@
         <v>12</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>-4.9</v>
       </c>
       <c r="F2" t="n">
-        <v>156.1</v>
+        <v>174.1</v>
       </c>
       <c r="G2" t="n">
-        <v>-1.5</v>
-      </c>
-      <c r="H2" t="n">
-        <v>183.5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H2"/>
       <c r="I2" t="s">
         <v>13</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46228</v>
+        <v>46234</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -541,115 +533,105 @@
         <v>16</v>
       </c>
       <c r="E3" t="n">
-        <v>49.8</v>
+        <v>22.1</v>
       </c>
       <c r="F3" t="n">
-        <v>166.6</v>
+        <v>168.4</v>
       </c>
       <c r="G3" t="n">
-        <v>-39.5</v>
-      </c>
-      <c r="H3" t="n">
-        <v>175.5</v>
-      </c>
+        <v>-31.5</v>
+      </c>
+      <c r="H3"/>
       <c r="I3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46228</v>
+        <v>46235</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E4" t="n">
-        <v>54</v>
+        <v>-16.2</v>
       </c>
       <c r="F4" t="n">
-        <v>168.7</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-60.5</v>
-      </c>
-      <c r="H4" t="n">
-        <v>174.5</v>
-      </c>
+        <v>179</v>
+      </c>
+      <c r="G4"/>
+      <c r="H4"/>
       <c r="I4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46228</v>
+        <v>46235</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E5" t="n">
-        <v>-3.2</v>
+        <v>44.9</v>
       </c>
       <c r="F5" t="n">
-        <v>176.8</v>
+        <v>176</v>
       </c>
       <c r="G5" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="H5" t="n">
-        <v>184.5</v>
-      </c>
+        <v>-30.5</v>
+      </c>
+      <c r="H5"/>
       <c r="I5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46229</v>
+        <v>46235</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E6" t="n">
-        <v>34.6</v>
+        <v>-7.6</v>
       </c>
       <c r="F6" t="n">
-        <v>173.3</v>
+        <v>177.2</v>
       </c>
       <c r="G6" t="n">
-        <v>-40.5</v>
-      </c>
-      <c r="H6" t="n">
-        <v>188.5</v>
-      </c>
+        <v>6.5</v>
+      </c>
+      <c r="H6"/>
       <c r="I6" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -657,7 +639,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46229</v>
+        <v>46235</v>
       </c>
       <c r="B7" t="s">
         <v>29</v>
@@ -669,52 +651,20 @@
         <v>31</v>
       </c>
       <c r="E7" t="n">
-        <v>-11.7</v>
+        <v>-2</v>
       </c>
       <c r="F7" t="n">
-        <v>172</v>
+        <v>169.8</v>
       </c>
       <c r="G7" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="H7" t="n">
-        <v>176.5</v>
-      </c>
+        <v>4.5</v>
+      </c>
+      <c r="H7"/>
       <c r="I7" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46233</v>
-      </c>
-      <c r="B8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-4.9</v>
-      </c>
-      <c r="F8" t="n">
-        <v>172.3</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8"/>
-      <c r="I8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-07-31 09:34:53
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,73 +44,94 @@
     <t xml:space="preserve">Forecast Rain mm</t>
   </si>
   <si>
-    <t xml:space="preserve">19:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
+    <t xml:space="preserve">18:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">western bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optus Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marvel Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hawthorn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UTAS Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">greater western sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adelaide Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">west coast eagles</t>
   </si>
   <si>
     <t xml:space="preserve">MCG</t>
   </si>
   <si>
-    <t xml:space="preserve">18:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optus Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marvel Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UTAS Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adelaide Oval</t>
+    <t xml:space="preserve">15:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People First Stadium</t>
   </si>
 </sst>
 </file>
@@ -447,13 +468,13 @@
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="5.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="13.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="15.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="22.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="15.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="12.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="14.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="20.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
@@ -491,7 +512,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -503,25 +524,25 @@
         <v>12</v>
       </c>
       <c r="E2" t="n">
-        <v>-4.9</v>
+        <v>22</v>
       </c>
       <c r="F2" t="n">
-        <v>174.1</v>
+        <v>168.4</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>-31.5</v>
       </c>
       <c r="H2"/>
       <c r="I2" t="s">
         <v>13</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -533,14 +554,12 @@
         <v>16</v>
       </c>
       <c r="E3" t="n">
-        <v>22.1</v>
+        <v>-16.3</v>
       </c>
       <c r="F3" t="n">
-        <v>168.4</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-31.5</v>
-      </c>
+        <v>179.1</v>
+      </c>
+      <c r="G3"/>
       <c r="H3"/>
       <c r="I3" t="s">
         <v>17</v>
@@ -563,18 +582,20 @@
         <v>20</v>
       </c>
       <c r="E4" t="n">
-        <v>-16.2</v>
+        <v>44.8</v>
       </c>
       <c r="F4" t="n">
-        <v>179</v>
-      </c>
-      <c r="G4"/>
+        <v>175.9</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-30.5</v>
+      </c>
       <c r="H4"/>
       <c r="I4" t="s">
         <v>21</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="5">
@@ -591,20 +612,20 @@
         <v>24</v>
       </c>
       <c r="E5" t="n">
-        <v>44.9</v>
+        <v>-7.7</v>
       </c>
       <c r="F5" t="n">
-        <v>176</v>
+        <v>177.1</v>
       </c>
       <c r="G5" t="n">
-        <v>-30.5</v>
+        <v>6.5</v>
       </c>
       <c r="H5"/>
       <c r="I5" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -612,26 +633,26 @@
         <v>46235</v>
       </c>
       <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
         <v>26</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>27</v>
       </c>
-      <c r="D6" t="s">
-        <v>28</v>
-      </c>
       <c r="E6" t="n">
-        <v>-7.6</v>
+        <v>-2</v>
       </c>
       <c r="F6" t="n">
-        <v>177.2</v>
+        <v>169.8</v>
       </c>
       <c r="G6" t="n">
-        <v>6.5</v>
+        <v>4.5</v>
       </c>
       <c r="H6"/>
       <c r="I6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -639,7 +660,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="B7" t="s">
         <v>29</v>
@@ -651,20 +672,78 @@
         <v>31</v>
       </c>
       <c r="E7" t="n">
-        <v>-2</v>
+        <v>-39.1</v>
       </c>
       <c r="F7" t="n">
-        <v>169.8</v>
+        <v>166.3</v>
       </c>
       <c r="G7" t="n">
-        <v>4.5</v>
+        <v>38</v>
       </c>
       <c r="H7"/>
       <c r="I7" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B8" t="s">
         <v>32</v>
       </c>
-      <c r="J7" t="n">
-        <v>0</v>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F8" t="n">
+        <v>166.1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8"/>
+      <c r="I8" t="s">
+        <v>35</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>180.1</v>
+      </c>
+      <c r="G9"/>
+      <c r="H9"/>
+      <c r="I9" t="s">
+        <v>39</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-08-01 08:29:10
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,94 +44,88 @@
     <t xml:space="preserve">Forecast Rain mm</t>
   </si>
   <si>
-    <t xml:space="preserve">18:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
+    <t xml:space="preserve">19:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marvel Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hawthorn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UTAS Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">greater western sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adelaide Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">west coast eagles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People First Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:30</t>
   </si>
   <si>
     <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optus Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marvel Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UTAS Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adelaide Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">west coast eagles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People First Stadium</t>
   </si>
 </sst>
 </file>
@@ -468,7 +462,7 @@
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="5.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="15.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="16.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="22.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="15.71" hidden="0" customWidth="1"/>
@@ -512,7 +506,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -524,20 +518,18 @@
         <v>12</v>
       </c>
       <c r="E2" t="n">
-        <v>22</v>
+        <v>-16.3</v>
       </c>
       <c r="F2" t="n">
-        <v>168.4</v>
-      </c>
-      <c r="G2" t="n">
-        <v>-31.5</v>
-      </c>
+        <v>178.4</v>
+      </c>
+      <c r="G2"/>
       <c r="H2"/>
       <c r="I2" t="s">
         <v>13</v>
       </c>
       <c r="J2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -554,12 +546,14 @@
         <v>16</v>
       </c>
       <c r="E3" t="n">
-        <v>-16.3</v>
+        <v>44.7</v>
       </c>
       <c r="F3" t="n">
-        <v>179.1</v>
-      </c>
-      <c r="G3"/>
+        <v>175.3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-30.5</v>
+      </c>
       <c r="H3"/>
       <c r="I3" t="s">
         <v>17</v>
@@ -582,20 +576,20 @@
         <v>20</v>
       </c>
       <c r="E4" t="n">
-        <v>44.8</v>
+        <v>-7.5</v>
       </c>
       <c r="F4" t="n">
-        <v>175.9</v>
+        <v>176.7</v>
       </c>
       <c r="G4" t="n">
-        <v>-30.5</v>
+        <v>6.5</v>
       </c>
       <c r="H4"/>
       <c r="I4" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -603,26 +597,26 @@
         <v>46235</v>
       </c>
       <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
         <v>22</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
       <c r="E5" t="n">
-        <v>-7.7</v>
+        <v>-2</v>
       </c>
       <c r="F5" t="n">
-        <v>177.1</v>
+        <v>169.2</v>
       </c>
       <c r="G5" t="n">
-        <v>6.5</v>
+        <v>4.5</v>
       </c>
       <c r="H5"/>
       <c r="I5" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -630,7 +624,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="B6" t="s">
         <v>25</v>
@@ -642,17 +636,17 @@
         <v>27</v>
       </c>
       <c r="E6" t="n">
-        <v>-2</v>
+        <v>-38.9</v>
       </c>
       <c r="F6" t="n">
-        <v>169.8</v>
+        <v>165.7</v>
       </c>
       <c r="G6" t="n">
-        <v>4.5</v>
+        <v>38</v>
       </c>
       <c r="H6"/>
       <c r="I6" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -663,29 +657,29 @@
         <v>46236</v>
       </c>
       <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
         <v>29</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>30</v>
       </c>
-      <c r="D7" t="s">
-        <v>31</v>
-      </c>
       <c r="E7" t="n">
-        <v>-39.1</v>
+        <v>0.9</v>
       </c>
       <c r="F7" t="n">
-        <v>166.3</v>
+        <v>165.6</v>
       </c>
       <c r="G7" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="H7"/>
       <c r="I7" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -702,25 +696,23 @@
         <v>34</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>166.1</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
+        <v>179.6</v>
+      </c>
+      <c r="G8"/>
       <c r="H8"/>
       <c r="I8" t="s">
         <v>35</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46236</v>
+        <v>46240</v>
       </c>
       <c r="B9" t="s">
         <v>36</v>
@@ -729,21 +721,21 @@
         <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="E9" t="n">
-        <v>2.1</v>
+        <v>32.3</v>
       </c>
       <c r="F9" t="n">
-        <v>180.1</v>
+        <v>171</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
       <c r="I9" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="J9" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-08-01 09:35:57
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -523,8 +523,12 @@
       <c r="F2" t="n">
         <v>178.4</v>
       </c>
-      <c r="G2"/>
-      <c r="H2"/>
+      <c r="G2" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>184.5</v>
+      </c>
       <c r="I2" t="s">
         <v>13</v>
       </c>
@@ -552,9 +556,11 @@
         <v>175.3</v>
       </c>
       <c r="G3" t="n">
-        <v>-30.5</v>
-      </c>
-      <c r="H3"/>
+        <v>-41.5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>182.5</v>
+      </c>
       <c r="I3" t="s">
         <v>17</v>
       </c>
@@ -582,9 +588,11 @@
         <v>176.7</v>
       </c>
       <c r="G4" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="H4"/>
+        <v>13.5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>182.5</v>
+      </c>
       <c r="I4" t="s">
         <v>13</v>
       </c>
@@ -612,9 +620,11 @@
         <v>169.2</v>
       </c>
       <c r="G5" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="H5"/>
+        <v>-2.5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>168.5</v>
+      </c>
       <c r="I5" t="s">
         <v>24</v>
       </c>
@@ -642,9 +652,11 @@
         <v>165.7</v>
       </c>
       <c r="G6" t="n">
-        <v>38</v>
-      </c>
-      <c r="H6"/>
+        <v>39.5</v>
+      </c>
+      <c r="H6" t="n">
+        <v>173.5</v>
+      </c>
       <c r="I6" t="s">
         <v>13</v>
       </c>
@@ -672,9 +684,11 @@
         <v>165.6</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7"/>
+        <v>6.5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>166.5</v>
+      </c>
       <c r="I7" t="s">
         <v>31</v>
       </c>
@@ -701,8 +715,12 @@
       <c r="F8" t="n">
         <v>179.6</v>
       </c>
-      <c r="G8"/>
-      <c r="H8"/>
+      <c r="G8" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>178.5</v>
+      </c>
       <c r="I8" t="s">
         <v>35</v>
       </c>

</xml_diff>

<commit_message>
Update model outputs 2026-08-02 14:49:30
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -26,7 +26,10 @@
     <t xml:space="preserve">Away Team</t>
   </si>
   <si>
-    <t xml:space="preserve">Projected Line</t>
+    <t xml:space="preserve">PROD Projected Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM-only Projected Line</t>
   </si>
   <si>
     <t xml:space="preserve">Projected Total</t>
@@ -44,88 +47,49 @@
     <t xml:space="preserve">Forecast Rain mm</t>
   </si>
   <si>
-    <t xml:space="preserve">19:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
+    <t xml:space="preserve">16:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
   </si>
   <si>
     <t xml:space="preserve">Marvel Stadium</t>
   </si>
   <si>
-    <t xml:space="preserve">13:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
+    <t xml:space="preserve">13:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">west coast eagles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People First Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">western bulldogs</t>
   </si>
   <si>
     <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UTAS Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adelaide Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">west coast eagles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People First Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
   </si>
 </sst>
 </file>
@@ -463,13 +427,14 @@
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="5.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="16.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="22.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="15.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="12.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="20.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="16.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="19.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="24.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="15.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="12.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="20.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,256 +468,143 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" t="n">
-        <v>-16.3</v>
+        <v>-38.9</v>
       </c>
       <c r="F2" t="n">
-        <v>178.4</v>
+        <v>-38.9</v>
       </c>
       <c r="G2" t="n">
-        <v>23.5</v>
+        <v>165.7</v>
       </c>
       <c r="H2" t="n">
-        <v>184.5</v>
-      </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>173.5</v>
+      </c>
+      <c r="J2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E3" t="n">
-        <v>44.7</v>
+        <v>0.9</v>
       </c>
       <c r="F3" t="n">
-        <v>175.3</v>
+        <v>0.9</v>
       </c>
       <c r="G3" t="n">
-        <v>-41.5</v>
+        <v>165.6</v>
       </c>
       <c r="H3" t="n">
-        <v>182.5</v>
-      </c>
-      <c r="I3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>166.5</v>
+      </c>
+      <c r="J3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E4" t="n">
-        <v>-7.5</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>176.7</v>
+        <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>13.5</v>
+        <v>179.6</v>
       </c>
       <c r="H4" t="n">
-        <v>182.5</v>
-      </c>
-      <c r="I4" t="s">
-        <v>13</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
+        <v>9.5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>178.5</v>
+      </c>
+      <c r="J4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46235</v>
+        <v>46240</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E5" t="n">
-        <v>-2</v>
+        <v>32.3</v>
       </c>
       <c r="F5" t="n">
-        <v>169.2</v>
+        <v>32.3</v>
       </c>
       <c r="G5" t="n">
-        <v>-2.5</v>
-      </c>
-      <c r="H5" t="n">
-        <v>168.5</v>
-      </c>
-      <c r="I5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46236</v>
-      </c>
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" t="n">
-        <v>-38.9</v>
-      </c>
-      <c r="F6" t="n">
-        <v>165.7</v>
-      </c>
-      <c r="G6" t="n">
-        <v>39.5</v>
-      </c>
-      <c r="H6" t="n">
-        <v>173.5</v>
-      </c>
-      <c r="I6" t="s">
-        <v>13</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>46236</v>
-      </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="F7" t="n">
-        <v>165.6</v>
-      </c>
-      <c r="G7" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="H7" t="n">
-        <v>166.5</v>
-      </c>
-      <c r="I7" t="s">
-        <v>31</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46236</v>
-      </c>
-      <c r="B8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" t="n">
-        <v>179.6</v>
-      </c>
-      <c r="G8" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="H8" t="n">
-        <v>178.5</v>
-      </c>
-      <c r="I8" t="s">
-        <v>35</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46240</v>
-      </c>
-      <c r="B9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="F9" t="n">
         <v>171</v>
       </c>
-      <c r="G9"/>
-      <c r="H9"/>
-      <c r="I9" t="s">
-        <v>13</v>
-      </c>
-      <c r="J9" t="n">
+      <c r="H5"/>
+      <c r="I5"/>
+      <c r="J5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-08-03 20:11:04
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -32,6 +32,9 @@
     <t xml:space="preserve">TEAM-only Projected Line</t>
   </si>
   <si>
+    <t xml:space="preserve">PLAYER-only Projected Line</t>
+  </si>
+  <si>
     <t xml:space="preserve">Projected Total</t>
   </si>
   <si>
@@ -47,49 +50,76 @@
     <t xml:space="preserve">Forecast Rain mm</t>
   </si>
   <si>
-    <t xml:space="preserve">16:40</t>
+    <t xml:space="preserve">19:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">western bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marvel Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hawthorn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gabba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
   </si>
   <si>
     <t xml:space="preserve">essendon</t>
   </si>
   <si>
+    <t xml:space="preserve">GMHBA Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:05</t>
+  </si>
+  <si>
     <t xml:space="preserve">adelaide crows</t>
   </si>
   <si>
-    <t xml:space="preserve">Marvel Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:10</t>
-  </si>
-  <si>
     <t xml:space="preserve">richmond</t>
   </si>
   <si>
-    <t xml:space="preserve">west coast eagles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People First Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
+    <t xml:space="preserve">Adelaide Oval</t>
   </si>
 </sst>
 </file>
@@ -427,14 +457,15 @@
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="5.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="16.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="19.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="24.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="15.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="12.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="20.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="16.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="26.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="15.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="12.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="14.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,141 +502,222 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46236</v>
+        <v>46240</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>-38.9</v>
+        <v>28.4</v>
       </c>
       <c r="F2" t="n">
-        <v>-38.9</v>
+        <v>28.4</v>
       </c>
       <c r="G2" t="n">
-        <v>165.7</v>
+        <v>2.7</v>
       </c>
       <c r="H2" t="n">
-        <v>39.5</v>
-      </c>
-      <c r="I2" t="n">
-        <v>173.5</v>
-      </c>
-      <c r="J2" t="s">
-        <v>14</v>
-      </c>
-      <c r="K2" t="n">
+        <v>172.7</v>
+      </c>
+      <c r="I2"/>
+      <c r="J2"/>
+      <c r="K2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46236</v>
+        <v>46241</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9</v>
+        <v>4.6</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9</v>
+        <v>4.6</v>
       </c>
       <c r="G3" t="n">
-        <v>165.6</v>
+        <v>7.9</v>
       </c>
       <c r="H3" t="n">
-        <v>6.5</v>
+        <v>187.1</v>
       </c>
       <c r="I3" t="n">
-        <v>166.5</v>
-      </c>
-      <c r="J3" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="J3"/>
+      <c r="K3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46236</v>
+        <v>46242</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>63.1</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>63.1</v>
       </c>
       <c r="G4" t="n">
-        <v>179.6</v>
+        <v>34.4</v>
       </c>
       <c r="H4" t="n">
-        <v>9.5</v>
+        <v>177.8</v>
       </c>
       <c r="I4" t="n">
-        <v>178.5</v>
-      </c>
-      <c r="J4" t="s">
-        <v>22</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.5</v>
+        <v>-60.5</v>
+      </c>
+      <c r="J4"/>
+      <c r="K4" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46240</v>
+        <v>46242</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E5" t="n">
-        <v>32.3</v>
+        <v>-11.2</v>
       </c>
       <c r="F5" t="n">
-        <v>32.3</v>
+        <v>-11.2</v>
       </c>
       <c r="G5" t="n">
-        <v>171</v>
-      </c>
-      <c r="H5"/>
-      <c r="I5"/>
-      <c r="J5" t="s">
-        <v>14</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
+        <v>0.8</v>
+      </c>
+      <c r="H5" t="n">
+        <v>175.4</v>
+      </c>
+      <c r="I5" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="J5"/>
+      <c r="K5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="H6" t="n">
+        <v>172.3</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-32.5</v>
+      </c>
+      <c r="J6"/>
+      <c r="K6" t="s">
+        <v>31</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="F7" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="G7" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="H7" t="n">
+        <v>168.2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-54.5</v>
+      </c>
+      <c r="J7"/>
+      <c r="K7" t="s">
+        <v>35</v>
+      </c>
+      <c r="L7" t="n">
+        <v>22.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-08-04 06:16:59
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -26,13 +26,13 @@
     <t xml:space="preserve">Away Team</t>
   </si>
   <si>
-    <t xml:space="preserve">PROD Projected Line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAM-only Projected Line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PLAYER-only Projected Line</t>
+    <t xml:space="preserve">Selected / Hybrid Home Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAM Home Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLAYER Home Line</t>
   </si>
   <si>
     <t xml:space="preserve">Projected Total</t>
@@ -458,9 +458,9 @@
     <col min="2" max="2" width="5.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="16.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="19.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="24.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="26.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="27.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="14.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="15.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="12.71" hidden="0" customWidth="1"/>
@@ -520,13 +520,13 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>28.4</v>
+        <v>-28.4</v>
       </c>
       <c r="F2" t="n">
-        <v>28.4</v>
+        <v>-28.4</v>
       </c>
       <c r="G2" t="n">
-        <v>2.7</v>
+        <v>-2.7</v>
       </c>
       <c r="H2" t="n">
         <v>172.7</v>
@@ -554,13 +554,13 @@
         <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>4.6</v>
+        <v>-4.6</v>
       </c>
       <c r="F3" t="n">
-        <v>4.6</v>
+        <v>-4.6</v>
       </c>
       <c r="G3" t="n">
-        <v>7.9</v>
+        <v>-7.9</v>
       </c>
       <c r="H3" t="n">
         <v>187.1</v>
@@ -590,13 +590,13 @@
         <v>22</v>
       </c>
       <c r="E4" t="n">
-        <v>63.1</v>
+        <v>-63.1</v>
       </c>
       <c r="F4" t="n">
-        <v>63.1</v>
+        <v>-63.1</v>
       </c>
       <c r="G4" t="n">
-        <v>34.4</v>
+        <v>-34.4</v>
       </c>
       <c r="H4" t="n">
         <v>177.8</v>
@@ -626,13 +626,13 @@
         <v>26</v>
       </c>
       <c r="E5" t="n">
-        <v>-11.2</v>
+        <v>11.2</v>
       </c>
       <c r="F5" t="n">
-        <v>-11.2</v>
+        <v>11.2</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8</v>
+        <v>-0.8</v>
       </c>
       <c r="H5" t="n">
         <v>175.4</v>
@@ -662,13 +662,13 @@
         <v>30</v>
       </c>
       <c r="E6" t="n">
-        <v>32.2</v>
+        <v>-32.2</v>
       </c>
       <c r="F6" t="n">
-        <v>32.2</v>
+        <v>-32.2</v>
       </c>
       <c r="G6" t="n">
-        <v>39.6</v>
+        <v>-39.6</v>
       </c>
       <c r="H6" t="n">
         <v>172.3</v>
@@ -698,13 +698,13 @@
         <v>34</v>
       </c>
       <c r="E7" t="n">
-        <v>59.6</v>
+        <v>-59.6</v>
       </c>
       <c r="F7" t="n">
-        <v>59.6</v>
+        <v>-59.6</v>
       </c>
       <c r="G7" t="n">
-        <v>39.3</v>
+        <v>-39.3</v>
       </c>
       <c r="H7" t="n">
         <v>168.2</v>

</xml_diff>

<commit_message>
Update model outputs 2026-08-04 21:45:29
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -120,6 +120,39 @@
   </si>
   <si>
     <t xml:space="preserve">Adelaide Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">west coast eagles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collingwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optus Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">greater western sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corroboree Group Oval Manuka</t>
   </si>
 </sst>
 </file>
@@ -456,7 +489,7 @@
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="5.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="16.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="22.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="27.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="14.71" hidden="0" customWidth="1"/>
@@ -464,7 +497,7 @@
     <col min="8" max="8" width="15.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="12.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="14.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="28.71" hidden="0" customWidth="1"/>
     <col min="12" max="12" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
@@ -720,6 +753,114 @@
         <v>22.5</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>170.6</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="J8"/>
+      <c r="K8" t="s">
+        <v>15</v>
+      </c>
+      <c r="L8" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="G9" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="H9" t="n">
+        <v>165.6</v>
+      </c>
+      <c r="I9" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J9"/>
+      <c r="K9" t="s">
+        <v>42</v>
+      </c>
+      <c r="L9" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-12.7</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-12.7</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="H10" t="n">
+        <v>178.9</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="J10"/>
+      <c r="K10" t="s">
+        <v>46</v>
+      </c>
+      <c r="L10" t="n">
+        <v>15.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update model outputs 2026-08-05 10:53:45
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -6,7 +6,7 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="AFL V2 Projections" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AFL JOINT Projections" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -26,7 +26,7 @@
     <t xml:space="preserve">Away Team</t>
   </si>
   <si>
-    <t xml:space="preserve">Selected / Hybrid Home Line</t>
+    <t xml:space="preserve">Selected / JOINT Home Line</t>
   </si>
   <si>
     <t xml:space="preserve">TEAM Home Line</t>
@@ -491,7 +491,7 @@
     <col min="2" max="2" width="5.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="22.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="27.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="26.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="14.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="15.71" hidden="0" customWidth="1"/>
@@ -553,7 +553,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>-28.4</v>
+        <v>-20.7</v>
       </c>
       <c r="F2" t="n">
         <v>-28.4</v>
@@ -587,7 +587,7 @@
         <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>-4.6</v>
+        <v>-5.9</v>
       </c>
       <c r="F3" t="n">
         <v>-4.6</v>
@@ -623,7 +623,7 @@
         <v>22</v>
       </c>
       <c r="E4" t="n">
-        <v>-63.1</v>
+        <v>-57.4</v>
       </c>
       <c r="F4" t="n">
         <v>-63.1</v>
@@ -659,7 +659,7 @@
         <v>26</v>
       </c>
       <c r="E5" t="n">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="F5" t="n">
         <v>11.2</v>
@@ -695,7 +695,7 @@
         <v>30</v>
       </c>
       <c r="E6" t="n">
-        <v>-32.2</v>
+        <v>-37.1</v>
       </c>
       <c r="F6" t="n">
         <v>-32.2</v>
@@ -731,7 +731,7 @@
         <v>34</v>
       </c>
       <c r="E7" t="n">
-        <v>-59.6</v>
+        <v>-48.6</v>
       </c>
       <c r="F7" t="n">
         <v>-59.6</v>
@@ -767,7 +767,7 @@
         <v>38</v>
       </c>
       <c r="E8" t="n">
-        <v>-5.2</v>
+        <v>5.9</v>
       </c>
       <c r="F8" t="n">
         <v>-5.2</v>
@@ -803,7 +803,7 @@
         <v>41</v>
       </c>
       <c r="E9" t="n">
-        <v>30.2</v>
+        <v>37.1</v>
       </c>
       <c r="F9" t="n">
         <v>30.2</v>
@@ -839,7 +839,7 @@
         <v>45</v>
       </c>
       <c r="E10" t="n">
-        <v>-12.7</v>
+        <v>-5.3</v>
       </c>
       <c r="F10" t="n">
         <v>-12.7</v>

</xml_diff>

<commit_message>
Update model outputs 2026-08-05 12:15:01
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -553,13 +553,13 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>-20.7</v>
+        <v>-20.9</v>
       </c>
       <c r="F2" t="n">
         <v>-28.4</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.7</v>
+        <v>-2.8</v>
       </c>
       <c r="H2" t="n">
         <v>172.7</v>
@@ -575,35 +575,33 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46241</v>
+        <v>46240</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>-5.9</v>
+        <v>-20.9</v>
       </c>
       <c r="F3" t="n">
-        <v>-4.6</v>
+        <v>-28.4</v>
       </c>
       <c r="G3" t="n">
-        <v>-7.9</v>
+        <v>-2.8</v>
       </c>
       <c r="H3" t="n">
-        <v>187.1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>-10.5</v>
-      </c>
+        <v>172.7</v>
+      </c>
+      <c r="I3"/>
       <c r="J3"/>
       <c r="K3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -611,74 +609,74 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46242</v>
+        <v>46241</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E4" t="n">
-        <v>-57.4</v>
+        <v>-5.9</v>
       </c>
       <c r="F4" t="n">
-        <v>-63.1</v>
+        <v>-4.6</v>
       </c>
       <c r="G4" t="n">
-        <v>-34.4</v>
+        <v>-7.9</v>
       </c>
       <c r="H4" t="n">
-        <v>177.8</v>
+        <v>187.1</v>
       </c>
       <c r="I4" t="n">
-        <v>-60.5</v>
+        <v>-10.5</v>
       </c>
       <c r="J4"/>
       <c r="K4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46242</v>
+        <v>46241</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E5" t="n">
-        <v>11.5</v>
+        <v>-5.9</v>
       </c>
       <c r="F5" t="n">
-        <v>11.2</v>
+        <v>-4.6</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.8</v>
+        <v>-7.9</v>
       </c>
       <c r="H5" t="n">
-        <v>175.4</v>
+        <v>187.1</v>
       </c>
       <c r="I5" t="n">
-        <v>15.5</v>
+        <v>-10.5</v>
       </c>
       <c r="J5"/>
       <c r="K5" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="L5" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -686,35 +684,35 @@
         <v>46242</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E6" t="n">
-        <v>-37.1</v>
+        <v>-57.4</v>
       </c>
       <c r="F6" t="n">
-        <v>-32.2</v>
+        <v>-63.1</v>
       </c>
       <c r="G6" t="n">
-        <v>-39.6</v>
+        <v>-34.5</v>
       </c>
       <c r="H6" t="n">
-        <v>172.3</v>
+        <v>176.6</v>
       </c>
       <c r="I6" t="n">
-        <v>-32.5</v>
+        <v>-60.5</v>
       </c>
       <c r="J6"/>
       <c r="K6" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="L6" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="7">
@@ -722,142 +720,466 @@
         <v>46242</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="E7" t="n">
-        <v>-48.6</v>
+        <v>-57.4</v>
       </c>
       <c r="F7" t="n">
-        <v>-59.6</v>
+        <v>-63.1</v>
       </c>
       <c r="G7" t="n">
-        <v>-39.3</v>
+        <v>-34.5</v>
       </c>
       <c r="H7" t="n">
-        <v>168.2</v>
+        <v>177.8</v>
       </c>
       <c r="I7" t="n">
-        <v>-54.5</v>
+        <v>-60.5</v>
       </c>
       <c r="J7"/>
       <c r="K7" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="L7" t="n">
-        <v>22.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46243</v>
+        <v>46242</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="E8" t="n">
-        <v>5.9</v>
+        <v>11.6</v>
       </c>
       <c r="F8" t="n">
-        <v>-5.2</v>
+        <v>11.2</v>
       </c>
       <c r="G8" t="n">
-        <v>5.1</v>
+        <v>-0.8</v>
       </c>
       <c r="H8" t="n">
-        <v>170.6</v>
+        <v>171.7</v>
       </c>
       <c r="I8" t="n">
-        <v>-9.5</v>
+        <v>15.5</v>
       </c>
       <c r="J8"/>
       <c r="K8" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="L8" t="n">
-        <v>3.1</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46243</v>
+        <v>46242</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="E9" t="n">
-        <v>37.1</v>
+        <v>11.6</v>
       </c>
       <c r="F9" t="n">
-        <v>30.2</v>
+        <v>11.2</v>
       </c>
       <c r="G9" t="n">
-        <v>31.6</v>
+        <v>-0.8</v>
       </c>
       <c r="H9" t="n">
-        <v>165.6</v>
+        <v>175.4</v>
       </c>
       <c r="I9" t="n">
-        <v>24.5</v>
+        <v>15.5</v>
       </c>
       <c r="J9"/>
       <c r="K9" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="L9" t="n">
-        <v>2.8</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46243</v>
+        <v>46242</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="E10" t="n">
-        <v>-5.3</v>
+        <v>-37.1</v>
       </c>
       <c r="F10" t="n">
-        <v>-12.7</v>
+        <v>-32.2</v>
       </c>
       <c r="G10" t="n">
-        <v>-4.4</v>
+        <v>-39.6</v>
       </c>
       <c r="H10" t="n">
-        <v>178.9</v>
+        <v>171.6</v>
       </c>
       <c r="I10" t="n">
-        <v>-10.5</v>
+        <v>-32.5</v>
       </c>
       <c r="J10"/>
       <c r="K10" t="s">
+        <v>31</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-37.1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-32.2</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-39.6</v>
+      </c>
+      <c r="H11" t="n">
+        <v>172.3</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-32.5</v>
+      </c>
+      <c r="J11"/>
+      <c r="K11" t="s">
+        <v>31</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-48.6</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-59.6</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-39.3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>160.2</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-54.5</v>
+      </c>
+      <c r="J12"/>
+      <c r="K12" t="s">
+        <v>35</v>
+      </c>
+      <c r="L12" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-48.6</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-59.6</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-39.3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>168.2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-54.5</v>
+      </c>
+      <c r="J13"/>
+      <c r="K13" t="s">
+        <v>35</v>
+      </c>
+      <c r="L13" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="G14" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>170.6</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="J14"/>
+      <c r="K14" t="s">
+        <v>15</v>
+      </c>
+      <c r="L14" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="G15" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>170.6</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="J15"/>
+      <c r="K15" t="s">
+        <v>15</v>
+      </c>
+      <c r="L15" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E16" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="G16" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="H16" t="n">
+        <v>159.8</v>
+      </c>
+      <c r="I16" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J16"/>
+      <c r="K16" t="s">
+        <v>42</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" t="n">
+        <v>37.1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="G17" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>165.6</v>
+      </c>
+      <c r="I17" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J17"/>
+      <c r="K17" t="s">
+        <v>42</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-12.7</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>170.9</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="J18"/>
+      <c r="K18" t="s">
         <v>46</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L18" t="n">
+        <v>15.8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>46243</v>
+      </c>
+      <c r="B19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-12.7</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="H19" t="n">
+        <v>178.9</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="J19"/>
+      <c r="K19" t="s">
+        <v>46</v>
+      </c>
+      <c r="L19" t="n">
         <v>15.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-08-05 13:07:21
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -553,13 +553,13 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>-20.9</v>
+        <v>-20.7</v>
       </c>
       <c r="F2" t="n">
         <v>-28.4</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.8</v>
+        <v>-2.7</v>
       </c>
       <c r="H2" t="n">
         <v>172.7</v>
@@ -587,13 +587,13 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>-20.9</v>
+        <v>-20.7</v>
       </c>
       <c r="F3" t="n">
         <v>-28.4</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.8</v>
+        <v>-2.7</v>
       </c>
       <c r="H3" t="n">
         <v>172.7</v>
@@ -699,7 +699,7 @@
         <v>-63.1</v>
       </c>
       <c r="G6" t="n">
-        <v>-34.5</v>
+        <v>-34.4</v>
       </c>
       <c r="H6" t="n">
         <v>176.6</v>
@@ -735,7 +735,7 @@
         <v>-63.1</v>
       </c>
       <c r="G7" t="n">
-        <v>-34.5</v>
+        <v>-34.4</v>
       </c>
       <c r="H7" t="n">
         <v>177.8</v>
@@ -765,7 +765,7 @@
         <v>26</v>
       </c>
       <c r="E8" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="F8" t="n">
         <v>11.2</v>
@@ -801,7 +801,7 @@
         <v>26</v>
       </c>
       <c r="E9" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="F9" t="n">
         <v>11.2</v>
@@ -918,7 +918,7 @@
         <v>-39.3</v>
       </c>
       <c r="H12" t="n">
-        <v>160.2</v>
+        <v>154.7</v>
       </c>
       <c r="I12" t="n">
         <v>-54.5</v>
@@ -1059,7 +1059,7 @@
         <v>30.2</v>
       </c>
       <c r="G16" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="H16" t="n">
         <v>159.8</v>
@@ -1095,7 +1095,7 @@
         <v>30.2</v>
       </c>
       <c r="G17" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="H17" t="n">
         <v>165.6</v>
@@ -1131,10 +1131,10 @@
         <v>-12.7</v>
       </c>
       <c r="G18" t="n">
-        <v>-4.5</v>
+        <v>-4.4</v>
       </c>
       <c r="H18" t="n">
-        <v>170.9</v>
+        <v>166.8</v>
       </c>
       <c r="I18" t="n">
         <v>-10.5</v>
@@ -1167,7 +1167,7 @@
         <v>-12.7</v>
       </c>
       <c r="G19" t="n">
-        <v>-4.5</v>
+        <v>-4.4</v>
       </c>
       <c r="H19" t="n">
         <v>178.9</v>

</xml_diff>

<commit_message>
Update model outputs 2026-08-05 13:18:10
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -38,6 +38,9 @@
     <t xml:space="preserve">Projected Total</t>
   </si>
   <si>
+    <t xml:space="preserve">Projection Type</t>
+  </si>
+  <si>
     <t xml:space="preserve">Market Line</t>
   </si>
   <si>
@@ -59,7 +62,13 @@
     <t xml:space="preserve">north melbourne</t>
   </si>
   <si>
+    <t xml:space="preserve">Weather Adjusted</t>
+  </si>
+  <si>
     <t xml:space="preserve">Marvel Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain</t>
   </si>
   <si>
     <t xml:space="preserve">19:40</t>
@@ -495,10 +504,11 @@
     <col min="6" max="6" width="14.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="15.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="12.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="28.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="16.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="16.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="12.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="28.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -538,19 +548,22 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
         <v>46240</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E2" t="n">
         <v>-20.7</v>
@@ -564,12 +577,15 @@
       <c r="H2" t="n">
         <v>172.7</v>
       </c>
-      <c r="I2"/>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
       <c r="J2"/>
-      <c r="K2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2" t="n">
+      <c r="K2"/>
+      <c r="L2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -578,13 +594,13 @@
         <v>46240</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
         <v>-20.7</v>
@@ -598,12 +614,15 @@
       <c r="H3" t="n">
         <v>172.7</v>
       </c>
-      <c r="I3"/>
+      <c r="I3" t="s">
+        <v>18</v>
+      </c>
       <c r="J3"/>
-      <c r="K3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L3" t="n">
+      <c r="K3"/>
+      <c r="L3" t="s">
+        <v>17</v>
+      </c>
+      <c r="M3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -612,13 +631,13 @@
         <v>46241</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E4" t="n">
         <v>-5.9</v>
@@ -632,14 +651,17 @@
       <c r="H4" t="n">
         <v>187.1</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" t="n">
         <v>-10.5</v>
       </c>
-      <c r="J4"/>
-      <c r="K4" t="s">
-        <v>19</v>
-      </c>
-      <c r="L4" t="n">
+      <c r="K4"/>
+      <c r="L4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -648,13 +670,13 @@
         <v>46241</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E5" t="n">
         <v>-5.9</v>
@@ -668,14 +690,17 @@
       <c r="H5" t="n">
         <v>187.1</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" t="n">
         <v>-10.5</v>
       </c>
-      <c r="J5"/>
-      <c r="K5" t="s">
-        <v>19</v>
-      </c>
-      <c r="L5" t="n">
+      <c r="K5"/>
+      <c r="L5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -684,13 +709,13 @@
         <v>46242</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E6" t="n">
         <v>-57.4</v>
@@ -704,14 +729,17 @@
       <c r="H6" t="n">
         <v>176.6</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" t="n">
         <v>-60.5</v>
       </c>
-      <c r="J6"/>
-      <c r="K6" t="s">
-        <v>23</v>
-      </c>
-      <c r="L6" t="n">
+      <c r="K6"/>
+      <c r="L6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M6" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -720,13 +748,13 @@
         <v>46242</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E7" t="n">
         <v>-57.4</v>
@@ -740,14 +768,17 @@
       <c r="H7" t="n">
         <v>177.8</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" t="n">
         <v>-60.5</v>
       </c>
-      <c r="J7"/>
-      <c r="K7" t="s">
-        <v>23</v>
-      </c>
-      <c r="L7" t="n">
+      <c r="K7"/>
+      <c r="L7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M7" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -756,13 +787,13 @@
         <v>46242</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E8" t="n">
         <v>11.5</v>
@@ -776,14 +807,17 @@
       <c r="H8" t="n">
         <v>171.7</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" t="n">
         <v>15.5</v>
       </c>
-      <c r="J8"/>
-      <c r="K8" t="s">
-        <v>27</v>
-      </c>
-      <c r="L8" t="n">
+      <c r="K8"/>
+      <c r="L8" t="s">
+        <v>30</v>
+      </c>
+      <c r="M8" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -792,13 +826,13 @@
         <v>46242</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E9" t="n">
         <v>11.5</v>
@@ -812,14 +846,17 @@
       <c r="H9" t="n">
         <v>175.4</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" t="n">
         <v>15.5</v>
       </c>
-      <c r="J9"/>
-      <c r="K9" t="s">
-        <v>27</v>
-      </c>
-      <c r="L9" t="n">
+      <c r="K9"/>
+      <c r="L9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M9" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -828,13 +865,13 @@
         <v>46242</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E10" t="n">
         <v>-37.1</v>
@@ -848,14 +885,17 @@
       <c r="H10" t="n">
         <v>171.6</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J10" t="n">
         <v>-32.5</v>
       </c>
-      <c r="J10"/>
-      <c r="K10" t="s">
-        <v>31</v>
-      </c>
-      <c r="L10" t="n">
+      <c r="K10"/>
+      <c r="L10" t="s">
+        <v>34</v>
+      </c>
+      <c r="M10" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -864,13 +904,13 @@
         <v>46242</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E11" t="n">
         <v>-37.1</v>
@@ -884,14 +924,17 @@
       <c r="H11" t="n">
         <v>172.3</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11" t="n">
         <v>-32.5</v>
       </c>
-      <c r="J11"/>
-      <c r="K11" t="s">
-        <v>31</v>
-      </c>
-      <c r="L11" t="n">
+      <c r="K11"/>
+      <c r="L11" t="s">
+        <v>34</v>
+      </c>
+      <c r="M11" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -900,13 +943,13 @@
         <v>46242</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E12" t="n">
         <v>-48.6</v>
@@ -920,14 +963,17 @@
       <c r="H12" t="n">
         <v>154.7</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J12" t="n">
         <v>-54.5</v>
       </c>
-      <c r="J12"/>
-      <c r="K12" t="s">
-        <v>35</v>
-      </c>
-      <c r="L12" t="n">
+      <c r="K12"/>
+      <c r="L12" t="s">
+        <v>38</v>
+      </c>
+      <c r="M12" t="n">
         <v>22.5</v>
       </c>
     </row>
@@ -936,13 +982,13 @@
         <v>46242</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D13" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E13" t="n">
         <v>-48.6</v>
@@ -956,14 +1002,17 @@
       <c r="H13" t="n">
         <v>168.2</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" t="s">
+        <v>18</v>
+      </c>
+      <c r="J13" t="n">
         <v>-54.5</v>
       </c>
-      <c r="J13"/>
-      <c r="K13" t="s">
-        <v>35</v>
-      </c>
-      <c r="L13" t="n">
+      <c r="K13"/>
+      <c r="L13" t="s">
+        <v>38</v>
+      </c>
+      <c r="M13" t="n">
         <v>22.5</v>
       </c>
     </row>
@@ -972,13 +1021,13 @@
         <v>46243</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D14" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E14" t="n">
         <v>5.9</v>
@@ -992,14 +1041,17 @@
       <c r="H14" t="n">
         <v>170.6</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" t="s">
+        <v>16</v>
+      </c>
+      <c r="J14" t="n">
         <v>-9.5</v>
       </c>
-      <c r="J14"/>
-      <c r="K14" t="s">
-        <v>15</v>
-      </c>
-      <c r="L14" t="n">
+      <c r="K14"/>
+      <c r="L14" t="s">
+        <v>17</v>
+      </c>
+      <c r="M14" t="n">
         <v>3.1</v>
       </c>
     </row>
@@ -1008,13 +1060,13 @@
         <v>46243</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D15" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E15" t="n">
         <v>5.9</v>
@@ -1028,14 +1080,17 @@
       <c r="H15" t="n">
         <v>170.6</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" t="n">
         <v>-9.5</v>
       </c>
-      <c r="J15"/>
-      <c r="K15" t="s">
-        <v>15</v>
-      </c>
-      <c r="L15" t="n">
+      <c r="K15"/>
+      <c r="L15" t="s">
+        <v>17</v>
+      </c>
+      <c r="M15" t="n">
         <v>3.1</v>
       </c>
     </row>
@@ -1044,13 +1099,13 @@
         <v>46243</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D16" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E16" t="n">
         <v>37.1</v>
@@ -1064,14 +1119,17 @@
       <c r="H16" t="n">
         <v>159.8</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" t="s">
+        <v>16</v>
+      </c>
+      <c r="J16" t="n">
         <v>24.5</v>
       </c>
-      <c r="J16"/>
-      <c r="K16" t="s">
-        <v>42</v>
-      </c>
-      <c r="L16" t="n">
+      <c r="K16"/>
+      <c r="L16" t="s">
+        <v>45</v>
+      </c>
+      <c r="M16" t="n">
         <v>2.8</v>
       </c>
     </row>
@@ -1080,13 +1138,13 @@
         <v>46243</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D17" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E17" t="n">
         <v>37.1</v>
@@ -1100,14 +1158,17 @@
       <c r="H17" t="n">
         <v>165.6</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" t="n">
         <v>24.5</v>
       </c>
-      <c r="J17"/>
-      <c r="K17" t="s">
-        <v>42</v>
-      </c>
-      <c r="L17" t="n">
+      <c r="K17"/>
+      <c r="L17" t="s">
+        <v>45</v>
+      </c>
+      <c r="M17" t="n">
         <v>2.8</v>
       </c>
     </row>
@@ -1116,13 +1177,13 @@
         <v>46243</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E18" t="n">
         <v>-5.3</v>
@@ -1136,14 +1197,17 @@
       <c r="H18" t="n">
         <v>166.8</v>
       </c>
-      <c r="I18" t="n">
+      <c r="I18" t="s">
+        <v>16</v>
+      </c>
+      <c r="J18" t="n">
         <v>-10.5</v>
       </c>
-      <c r="J18"/>
-      <c r="K18" t="s">
-        <v>46</v>
-      </c>
-      <c r="L18" t="n">
+      <c r="K18"/>
+      <c r="L18" t="s">
+        <v>49</v>
+      </c>
+      <c r="M18" t="n">
         <v>15.8</v>
       </c>
     </row>
@@ -1152,13 +1216,13 @@
         <v>46243</v>
       </c>
       <c r="B19" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C19" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E19" t="n">
         <v>-5.3</v>
@@ -1172,14 +1236,17 @@
       <c r="H19" t="n">
         <v>178.9</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I19" t="s">
+        <v>18</v>
+      </c>
+      <c r="J19" t="n">
         <v>-10.5</v>
       </c>
-      <c r="J19"/>
-      <c r="K19" t="s">
-        <v>46</v>
-      </c>
-      <c r="L19" t="n">
+      <c r="K19"/>
+      <c r="L19" t="s">
+        <v>49</v>
+      </c>
+      <c r="M19" t="n">
         <v>15.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-08-08 07:36:13
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -53,91 +53,70 @@
     <t xml:space="preserve">Forecast Rain mm</t>
   </si>
   <si>
-    <t xml:space="preserve">19:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
+    <t xml:space="preserve">16:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
   </si>
   <si>
     <t xml:space="preserve">Weather Adjusted</t>
   </si>
   <si>
+    <t xml:space="preserve">GMHBA Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adelaide Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
     <t xml:space="preserve">Marvel Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Rain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gabba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GMHBA Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adelaide Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
   </si>
   <si>
     <t xml:space="preserve">14:10</t>
@@ -554,7 +533,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46240</v>
+        <v>46242</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -566,32 +545,34 @@
         <v>15</v>
       </c>
       <c r="E2" t="n">
-        <v>-20.7</v>
+        <v>-57.4</v>
       </c>
       <c r="F2" t="n">
-        <v>-28.4</v>
+        <v>-63.1</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.7</v>
+        <v>-34.4</v>
       </c>
       <c r="H2" t="n">
-        <v>172.7</v>
+        <v>176.6</v>
       </c>
       <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="J2"/>
+      <c r="J2" t="n">
+        <v>-60.5</v>
+      </c>
       <c r="K2"/>
       <c r="L2" t="s">
         <v>17</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46240</v>
+        <v>46242</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -603,32 +584,34 @@
         <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>-20.7</v>
+        <v>-57.4</v>
       </c>
       <c r="F3" t="n">
-        <v>-28.4</v>
+        <v>-63.1</v>
       </c>
       <c r="G3" t="n">
-        <v>-2.7</v>
+        <v>-34.4</v>
       </c>
       <c r="H3" t="n">
-        <v>172.7</v>
+        <v>177.8</v>
       </c>
       <c r="I3" t="s">
         <v>18</v>
       </c>
-      <c r="J3"/>
+      <c r="J3" t="n">
+        <v>-60.5</v>
+      </c>
       <c r="K3"/>
       <c r="L3" t="s">
         <v>17</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="B4" t="s">
         <v>19</v>
@@ -640,34 +623,34 @@
         <v>21</v>
       </c>
       <c r="E4" t="n">
-        <v>-5.9</v>
+        <v>11.5</v>
       </c>
       <c r="F4" t="n">
-        <v>-4.6</v>
+        <v>11.2</v>
       </c>
       <c r="G4" t="n">
-        <v>-7.9</v>
+        <v>-0.8</v>
       </c>
       <c r="H4" t="n">
-        <v>187.1</v>
+        <v>171.7</v>
       </c>
       <c r="I4" t="s">
         <v>16</v>
       </c>
       <c r="J4" t="n">
-        <v>-10.5</v>
+        <v>15.5</v>
       </c>
       <c r="K4"/>
       <c r="L4" t="s">
         <v>22</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
@@ -679,29 +662,29 @@
         <v>21</v>
       </c>
       <c r="E5" t="n">
-        <v>-5.9</v>
+        <v>11.5</v>
       </c>
       <c r="F5" t="n">
-        <v>-4.6</v>
+        <v>11.2</v>
       </c>
       <c r="G5" t="n">
-        <v>-7.9</v>
+        <v>-0.8</v>
       </c>
       <c r="H5" t="n">
-        <v>187.1</v>
+        <v>175.4</v>
       </c>
       <c r="I5" t="s">
         <v>18</v>
       </c>
       <c r="J5" t="n">
-        <v>-10.5</v>
+        <v>15.5</v>
       </c>
       <c r="K5"/>
       <c r="L5" t="s">
         <v>22</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="6">
@@ -718,29 +701,29 @@
         <v>25</v>
       </c>
       <c r="E6" t="n">
-        <v>-57.4</v>
+        <v>-37.1</v>
       </c>
       <c r="F6" t="n">
-        <v>-63.1</v>
+        <v>-32.2</v>
       </c>
       <c r="G6" t="n">
-        <v>-34.4</v>
+        <v>-39.6</v>
       </c>
       <c r="H6" t="n">
-        <v>176.6</v>
+        <v>171.6</v>
       </c>
       <c r="I6" t="s">
         <v>16</v>
       </c>
       <c r="J6" t="n">
-        <v>-60.5</v>
+        <v>-32.5</v>
       </c>
       <c r="K6"/>
       <c r="L6" t="s">
         <v>26</v>
       </c>
       <c r="M6" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7">
@@ -757,29 +740,29 @@
         <v>25</v>
       </c>
       <c r="E7" t="n">
-        <v>-57.4</v>
+        <v>-37.1</v>
       </c>
       <c r="F7" t="n">
-        <v>-63.1</v>
+        <v>-32.2</v>
       </c>
       <c r="G7" t="n">
-        <v>-34.4</v>
+        <v>-39.6</v>
       </c>
       <c r="H7" t="n">
-        <v>177.8</v>
+        <v>172.3</v>
       </c>
       <c r="I7" t="s">
         <v>18</v>
       </c>
       <c r="J7" t="n">
-        <v>-60.5</v>
+        <v>-32.5</v>
       </c>
       <c r="K7"/>
       <c r="L7" t="s">
         <v>26</v>
       </c>
       <c r="M7" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8">
@@ -796,29 +779,29 @@
         <v>29</v>
       </c>
       <c r="E8" t="n">
-        <v>11.5</v>
+        <v>-48.6</v>
       </c>
       <c r="F8" t="n">
-        <v>11.2</v>
+        <v>-59.6</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.8</v>
+        <v>-39.3</v>
       </c>
       <c r="H8" t="n">
-        <v>171.7</v>
+        <v>154.7</v>
       </c>
       <c r="I8" t="s">
         <v>16</v>
       </c>
       <c r="J8" t="n">
-        <v>15.5</v>
+        <v>-54.5</v>
       </c>
       <c r="K8"/>
       <c r="L8" t="s">
         <v>30</v>
       </c>
       <c r="M8" t="n">
-        <v>1.4</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="9">
@@ -835,34 +818,34 @@
         <v>29</v>
       </c>
       <c r="E9" t="n">
-        <v>11.5</v>
+        <v>-48.6</v>
       </c>
       <c r="F9" t="n">
-        <v>11.2</v>
+        <v>-59.6</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.8</v>
+        <v>-39.3</v>
       </c>
       <c r="H9" t="n">
-        <v>175.4</v>
+        <v>168.2</v>
       </c>
       <c r="I9" t="s">
         <v>18</v>
       </c>
       <c r="J9" t="n">
-        <v>15.5</v>
+        <v>-54.5</v>
       </c>
       <c r="K9"/>
       <c r="L9" t="s">
         <v>30</v>
       </c>
       <c r="M9" t="n">
-        <v>1.4</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="B10" t="s">
         <v>31</v>
@@ -874,34 +857,34 @@
         <v>33</v>
       </c>
       <c r="E10" t="n">
-        <v>-37.1</v>
+        <v>5.9</v>
       </c>
       <c r="F10" t="n">
-        <v>-32.2</v>
+        <v>-5.2</v>
       </c>
       <c r="G10" t="n">
-        <v>-39.6</v>
+        <v>5.1</v>
       </c>
       <c r="H10" t="n">
-        <v>171.6</v>
+        <v>170.6</v>
       </c>
       <c r="I10" t="s">
         <v>16</v>
       </c>
       <c r="J10" t="n">
-        <v>-32.5</v>
+        <v>-9.5</v>
       </c>
       <c r="K10"/>
       <c r="L10" t="s">
         <v>34</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="B11" t="s">
         <v>31</v>
@@ -913,34 +896,34 @@
         <v>33</v>
       </c>
       <c r="E11" t="n">
-        <v>-37.1</v>
+        <v>5.9</v>
       </c>
       <c r="F11" t="n">
-        <v>-32.2</v>
+        <v>-5.2</v>
       </c>
       <c r="G11" t="n">
-        <v>-39.6</v>
+        <v>5.1</v>
       </c>
       <c r="H11" t="n">
-        <v>172.3</v>
+        <v>170.6</v>
       </c>
       <c r="I11" t="s">
         <v>18</v>
       </c>
       <c r="J11" t="n">
-        <v>-32.5</v>
+        <v>-9.5</v>
       </c>
       <c r="K11"/>
       <c r="L11" t="s">
         <v>34</v>
       </c>
       <c r="M11" t="n">
-        <v>0.2</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="B12" t="s">
         <v>35</v>
@@ -952,34 +935,34 @@
         <v>37</v>
       </c>
       <c r="E12" t="n">
-        <v>-48.6</v>
+        <v>37.1</v>
       </c>
       <c r="F12" t="n">
-        <v>-59.6</v>
+        <v>30.2</v>
       </c>
       <c r="G12" t="n">
-        <v>-39.3</v>
+        <v>31.6</v>
       </c>
       <c r="H12" t="n">
-        <v>154.7</v>
+        <v>159.8</v>
       </c>
       <c r="I12" t="s">
         <v>16</v>
       </c>
       <c r="J12" t="n">
-        <v>-54.5</v>
+        <v>24.5</v>
       </c>
       <c r="K12"/>
       <c r="L12" t="s">
         <v>38</v>
       </c>
       <c r="M12" t="n">
-        <v>22.5</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="B13" t="s">
         <v>35</v>
@@ -991,29 +974,29 @@
         <v>37</v>
       </c>
       <c r="E13" t="n">
-        <v>-48.6</v>
+        <v>37.1</v>
       </c>
       <c r="F13" t="n">
-        <v>-59.6</v>
+        <v>30.2</v>
       </c>
       <c r="G13" t="n">
-        <v>-39.3</v>
+        <v>31.6</v>
       </c>
       <c r="H13" t="n">
-        <v>168.2</v>
+        <v>165.6</v>
       </c>
       <c r="I13" t="s">
         <v>18</v>
       </c>
       <c r="J13" t="n">
-        <v>-54.5</v>
+        <v>24.5</v>
       </c>
       <c r="K13"/>
       <c r="L13" t="s">
         <v>38</v>
       </c>
       <c r="M13" t="n">
-        <v>22.5</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="14">
@@ -1030,29 +1013,29 @@
         <v>41</v>
       </c>
       <c r="E14" t="n">
-        <v>5.9</v>
+        <v>-5.3</v>
       </c>
       <c r="F14" t="n">
-        <v>-5.2</v>
+        <v>-12.7</v>
       </c>
       <c r="G14" t="n">
-        <v>5.1</v>
+        <v>-4.4</v>
       </c>
       <c r="H14" t="n">
-        <v>170.6</v>
+        <v>166.8</v>
       </c>
       <c r="I14" t="s">
         <v>16</v>
       </c>
       <c r="J14" t="n">
-        <v>-9.5</v>
+        <v>-10.5</v>
       </c>
       <c r="K14"/>
       <c r="L14" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="M14" t="n">
-        <v>3.1</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="15">
@@ -1069,184 +1052,28 @@
         <v>41</v>
       </c>
       <c r="E15" t="n">
-        <v>5.9</v>
+        <v>-5.3</v>
       </c>
       <c r="F15" t="n">
-        <v>-5.2</v>
+        <v>-12.7</v>
       </c>
       <c r="G15" t="n">
-        <v>5.1</v>
+        <v>-4.4</v>
       </c>
       <c r="H15" t="n">
-        <v>170.6</v>
+        <v>178.9</v>
       </c>
       <c r="I15" t="s">
         <v>18</v>
       </c>
       <c r="J15" t="n">
-        <v>-9.5</v>
+        <v>-10.5</v>
       </c>
       <c r="K15"/>
       <c r="L15" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="M15" t="n">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B16" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" t="s">
-        <v>44</v>
-      </c>
-      <c r="E16" t="n">
-        <v>37.1</v>
-      </c>
-      <c r="F16" t="n">
-        <v>30.2</v>
-      </c>
-      <c r="G16" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="H16" t="n">
-        <v>159.8</v>
-      </c>
-      <c r="I16" t="s">
-        <v>16</v>
-      </c>
-      <c r="J16" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="K16"/>
-      <c r="L16" t="s">
-        <v>45</v>
-      </c>
-      <c r="M16" t="n">
-        <v>2.8</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B17" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" t="s">
-        <v>43</v>
-      </c>
-      <c r="D17" t="s">
-        <v>44</v>
-      </c>
-      <c r="E17" t="n">
-        <v>37.1</v>
-      </c>
-      <c r="F17" t="n">
-        <v>30.2</v>
-      </c>
-      <c r="G17" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="H17" t="n">
-        <v>165.6</v>
-      </c>
-      <c r="I17" t="s">
-        <v>18</v>
-      </c>
-      <c r="J17" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="K17"/>
-      <c r="L17" t="s">
-        <v>45</v>
-      </c>
-      <c r="M17" t="n">
-        <v>2.8</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" t="s">
-        <v>48</v>
-      </c>
-      <c r="E18" t="n">
-        <v>-5.3</v>
-      </c>
-      <c r="F18" t="n">
-        <v>-12.7</v>
-      </c>
-      <c r="G18" t="n">
-        <v>-4.4</v>
-      </c>
-      <c r="H18" t="n">
-        <v>166.8</v>
-      </c>
-      <c r="I18" t="s">
-        <v>16</v>
-      </c>
-      <c r="J18" t="n">
-        <v>-10.5</v>
-      </c>
-      <c r="K18"/>
-      <c r="L18" t="s">
-        <v>49</v>
-      </c>
-      <c r="M18" t="n">
-        <v>15.8</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B19" t="s">
-        <v>46</v>
-      </c>
-      <c r="C19" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" t="s">
-        <v>48</v>
-      </c>
-      <c r="E19" t="n">
-        <v>-5.3</v>
-      </c>
-      <c r="F19" t="n">
-        <v>-12.7</v>
-      </c>
-      <c r="G19" t="n">
-        <v>-4.4</v>
-      </c>
-      <c r="H19" t="n">
-        <v>178.9</v>
-      </c>
-      <c r="I19" t="s">
-        <v>18</v>
-      </c>
-      <c r="J19" t="n">
-        <v>-10.5</v>
-      </c>
-      <c r="K19"/>
-      <c r="L19" t="s">
-        <v>49</v>
-      </c>
-      <c r="M19" t="n">
         <v>15.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-08-09 10:22:08
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -53,70 +53,22 @@
     <t xml:space="preserve">Forecast Rain mm</t>
   </si>
   <si>
-    <t xml:space="preserve">16:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
+    <t xml:space="preserve">19:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
   </si>
   <si>
     <t xml:space="preserve">Weather Adjusted</t>
   </si>
   <si>
-    <t xml:space="preserve">GMHBA Stadium</t>
+    <t xml:space="preserve">Marvel Stadium</t>
   </si>
   <si>
     <t xml:space="preserve">No Rain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adelaide Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marvel Stadium</t>
   </si>
   <si>
     <t xml:space="preserve">14:10</t>
@@ -533,7 +485,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -545,34 +497,34 @@
         <v>15</v>
       </c>
       <c r="E2" t="n">
-        <v>-57.4</v>
+        <v>5.9</v>
       </c>
       <c r="F2" t="n">
-        <v>-63.1</v>
+        <v>-5.2</v>
       </c>
       <c r="G2" t="n">
-        <v>-34.4</v>
+        <v>5.1</v>
       </c>
       <c r="H2" t="n">
-        <v>176.6</v>
+        <v>170.6</v>
       </c>
       <c r="I2" t="s">
         <v>16</v>
       </c>
       <c r="J2" t="n">
-        <v>-60.5</v>
+        <v>-9.5</v>
       </c>
       <c r="K2"/>
       <c r="L2" t="s">
         <v>17</v>
       </c>
       <c r="M2" t="n">
-        <v>0.3</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -584,34 +536,34 @@
         <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>-57.4</v>
+        <v>5.9</v>
       </c>
       <c r="F3" t="n">
-        <v>-63.1</v>
+        <v>-5.2</v>
       </c>
       <c r="G3" t="n">
-        <v>-34.4</v>
+        <v>5.1</v>
       </c>
       <c r="H3" t="n">
-        <v>177.8</v>
+        <v>170.6</v>
       </c>
       <c r="I3" t="s">
         <v>18</v>
       </c>
       <c r="J3" t="n">
-        <v>-60.5</v>
+        <v>-9.5</v>
       </c>
       <c r="K3"/>
       <c r="L3" t="s">
         <v>17</v>
       </c>
       <c r="M3" t="n">
-        <v>0.3</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="B4" t="s">
         <v>19</v>
@@ -623,34 +575,34 @@
         <v>21</v>
       </c>
       <c r="E4" t="n">
-        <v>11.5</v>
+        <v>37.1</v>
       </c>
       <c r="F4" t="n">
-        <v>11.2</v>
+        <v>30.2</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.8</v>
+        <v>31.6</v>
       </c>
       <c r="H4" t="n">
-        <v>171.7</v>
+        <v>159.8</v>
       </c>
       <c r="I4" t="s">
         <v>16</v>
       </c>
       <c r="J4" t="n">
-        <v>15.5</v>
+        <v>24.5</v>
       </c>
       <c r="K4"/>
       <c r="L4" t="s">
         <v>22</v>
       </c>
       <c r="M4" t="n">
-        <v>1.4</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
@@ -662,34 +614,34 @@
         <v>21</v>
       </c>
       <c r="E5" t="n">
-        <v>11.5</v>
+        <v>37.1</v>
       </c>
       <c r="F5" t="n">
-        <v>11.2</v>
+        <v>30.2</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.8</v>
+        <v>31.6</v>
       </c>
       <c r="H5" t="n">
-        <v>175.4</v>
+        <v>165.6</v>
       </c>
       <c r="I5" t="s">
         <v>18</v>
       </c>
       <c r="J5" t="n">
-        <v>15.5</v>
+        <v>24.5</v>
       </c>
       <c r="K5"/>
       <c r="L5" t="s">
         <v>22</v>
       </c>
       <c r="M5" t="n">
-        <v>1.4</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
@@ -701,34 +653,34 @@
         <v>25</v>
       </c>
       <c r="E6" t="n">
-        <v>-37.1</v>
+        <v>-5.3</v>
       </c>
       <c r="F6" t="n">
-        <v>-32.2</v>
+        <v>-12.7</v>
       </c>
       <c r="G6" t="n">
-        <v>-39.6</v>
+        <v>-4.4</v>
       </c>
       <c r="H6" t="n">
-        <v>171.6</v>
+        <v>166.8</v>
       </c>
       <c r="I6" t="s">
         <v>16</v>
       </c>
       <c r="J6" t="n">
-        <v>-32.5</v>
+        <v>-10.5</v>
       </c>
       <c r="K6"/>
       <c r="L6" t="s">
         <v>26</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
@@ -740,340 +692,28 @@
         <v>25</v>
       </c>
       <c r="E7" t="n">
-        <v>-37.1</v>
+        <v>-5.3</v>
       </c>
       <c r="F7" t="n">
-        <v>-32.2</v>
+        <v>-12.7</v>
       </c>
       <c r="G7" t="n">
-        <v>-39.6</v>
+        <v>-4.4</v>
       </c>
       <c r="H7" t="n">
-        <v>172.3</v>
+        <v>178.9</v>
       </c>
       <c r="I7" t="s">
         <v>18</v>
       </c>
       <c r="J7" t="n">
-        <v>-32.5</v>
+        <v>-10.5</v>
       </c>
       <c r="K7"/>
       <c r="L7" t="s">
         <v>26</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46242</v>
-      </c>
-      <c r="B8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-48.6</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-59.6</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-39.3</v>
-      </c>
-      <c r="H8" t="n">
-        <v>154.7</v>
-      </c>
-      <c r="I8" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8" t="n">
-        <v>-54.5</v>
-      </c>
-      <c r="K8"/>
-      <c r="L8" t="s">
-        <v>30</v>
-      </c>
-      <c r="M8" t="n">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46242</v>
-      </c>
-      <c r="B9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" t="n">
-        <v>-48.6</v>
-      </c>
-      <c r="F9" t="n">
-        <v>-59.6</v>
-      </c>
-      <c r="G9" t="n">
-        <v>-39.3</v>
-      </c>
-      <c r="H9" t="n">
-        <v>168.2</v>
-      </c>
-      <c r="I9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J9" t="n">
-        <v>-54.5</v>
-      </c>
-      <c r="K9"/>
-      <c r="L9" t="s">
-        <v>30</v>
-      </c>
-      <c r="M9" t="n">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="F10" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="G10" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="H10" t="n">
-        <v>170.6</v>
-      </c>
-      <c r="I10" t="s">
-        <v>16</v>
-      </c>
-      <c r="J10" t="n">
-        <v>-9.5</v>
-      </c>
-      <c r="K10"/>
-      <c r="L10" t="s">
-        <v>34</v>
-      </c>
-      <c r="M10" t="n">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="F11" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="G11" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="H11" t="n">
-        <v>170.6</v>
-      </c>
-      <c r="I11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J11" t="n">
-        <v>-9.5</v>
-      </c>
-      <c r="K11"/>
-      <c r="L11" t="s">
-        <v>34</v>
-      </c>
-      <c r="M11" t="n">
-        <v>3.1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" t="s">
-        <v>37</v>
-      </c>
-      <c r="E12" t="n">
-        <v>37.1</v>
-      </c>
-      <c r="F12" t="n">
-        <v>30.2</v>
-      </c>
-      <c r="G12" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="H12" t="n">
-        <v>159.8</v>
-      </c>
-      <c r="I12" t="s">
-        <v>16</v>
-      </c>
-      <c r="J12" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="K12"/>
-      <c r="L12" t="s">
-        <v>38</v>
-      </c>
-      <c r="M12" t="n">
-        <v>2.8</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B13" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" t="s">
-        <v>37</v>
-      </c>
-      <c r="E13" t="n">
-        <v>37.1</v>
-      </c>
-      <c r="F13" t="n">
-        <v>30.2</v>
-      </c>
-      <c r="G13" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="H13" t="n">
-        <v>165.6</v>
-      </c>
-      <c r="I13" t="s">
-        <v>18</v>
-      </c>
-      <c r="J13" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="K13"/>
-      <c r="L13" t="s">
-        <v>38</v>
-      </c>
-      <c r="M13" t="n">
-        <v>2.8</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B14" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D14" t="s">
-        <v>41</v>
-      </c>
-      <c r="E14" t="n">
-        <v>-5.3</v>
-      </c>
-      <c r="F14" t="n">
-        <v>-12.7</v>
-      </c>
-      <c r="G14" t="n">
-        <v>-4.4</v>
-      </c>
-      <c r="H14" t="n">
-        <v>166.8</v>
-      </c>
-      <c r="I14" t="s">
-        <v>16</v>
-      </c>
-      <c r="J14" t="n">
-        <v>-10.5</v>
-      </c>
-      <c r="K14"/>
-      <c r="L14" t="s">
-        <v>42</v>
-      </c>
-      <c r="M14" t="n">
-        <v>15.8</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>46243</v>
-      </c>
-      <c r="B15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" t="s">
-        <v>40</v>
-      </c>
-      <c r="D15" t="s">
-        <v>41</v>
-      </c>
-      <c r="E15" t="n">
-        <v>-5.3</v>
-      </c>
-      <c r="F15" t="n">
-        <v>-12.7</v>
-      </c>
-      <c r="G15" t="n">
-        <v>-4.4</v>
-      </c>
-      <c r="H15" t="n">
-        <v>178.9</v>
-      </c>
-      <c r="I15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J15" t="n">
-        <v>-10.5</v>
-      </c>
-      <c r="K15"/>
-      <c r="L15" t="s">
-        <v>42</v>
-      </c>
-      <c r="M15" t="n">
         <v>15.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-08-10 21:02:00
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -53,46 +53,85 @@
     <t xml:space="preserve">Forecast Rain mm</t>
   </si>
   <si>
-    <t xml:space="preserve">19:20</t>
+    <t xml:space="preserve">12:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weather Adjusted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Rain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gabba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marvel Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">western bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">greater western sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">west coast eagles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENGIE Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adelaide Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optus Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
   </si>
   <si>
     <t xml:space="preserve">st kilda</t>
   </si>
   <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weather Adjusted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marvel Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No Rain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">west coast eagles</t>
+    <t xml:space="preserve">hawthorn</t>
   </si>
   <si>
     <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optus Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13:10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corroboree Group Oval Manuka</t>
   </si>
 </sst>
 </file>
@@ -430,7 +469,7 @@
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="5.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="22.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="26.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="14.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
@@ -438,7 +477,7 @@
     <col min="9" max="9" width="16.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
     <col min="11" max="11" width="12.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="28.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="14.71" hidden="0" customWidth="1"/>
     <col min="13" max="13" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
@@ -485,7 +524,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46243</v>
+        <v>46248</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -497,34 +536,32 @@
         <v>15</v>
       </c>
       <c r="E2" t="n">
-        <v>5.9</v>
+        <v>47.9</v>
       </c>
       <c r="F2" t="n">
-        <v>-5.2</v>
+        <v>45.6</v>
       </c>
       <c r="G2" t="n">
-        <v>5.1</v>
+        <v>23.5</v>
       </c>
       <c r="H2" t="n">
-        <v>170.6</v>
+        <v>178</v>
       </c>
       <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="J2" t="n">
-        <v>-9.5</v>
-      </c>
+      <c r="J2"/>
       <c r="K2"/>
       <c r="L2" t="s">
         <v>17</v>
       </c>
       <c r="M2" t="n">
-        <v>3.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46243</v>
+        <v>46248</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -536,185 +573,627 @@
         <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>5.9</v>
+        <v>47.9</v>
       </c>
       <c r="F3" t="n">
-        <v>-5.2</v>
+        <v>45.6</v>
       </c>
       <c r="G3" t="n">
-        <v>5.1</v>
+        <v>23.5</v>
       </c>
       <c r="H3" t="n">
-        <v>170.6</v>
+        <v>181</v>
       </c>
       <c r="I3" t="s">
         <v>18</v>
       </c>
-      <c r="J3" t="n">
-        <v>-9.5</v>
-      </c>
+      <c r="J3"/>
       <c r="K3"/>
       <c r="L3" t="s">
         <v>17</v>
       </c>
       <c r="M3" t="n">
-        <v>3.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46243</v>
+        <v>46248</v>
       </c>
       <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
         <v>19</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>20</v>
       </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
       <c r="E4" t="n">
-        <v>37.1</v>
+        <v>-26.5</v>
       </c>
       <c r="F4" t="n">
-        <v>30.2</v>
+        <v>-25.2</v>
       </c>
       <c r="G4" t="n">
-        <v>31.6</v>
+        <v>-23.8</v>
       </c>
       <c r="H4" t="n">
-        <v>159.8</v>
+        <v>187.8</v>
       </c>
       <c r="I4" t="s">
         <v>16</v>
       </c>
-      <c r="J4" t="n">
-        <v>24.5</v>
-      </c>
+      <c r="J4"/>
       <c r="K4"/>
       <c r="L4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M4" t="n">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46243</v>
+        <v>46248</v>
       </c>
       <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>20</v>
       </c>
-      <c r="D5" t="s">
-        <v>21</v>
-      </c>
       <c r="E5" t="n">
-        <v>37.1</v>
+        <v>-26.5</v>
       </c>
       <c r="F5" t="n">
-        <v>30.2</v>
+        <v>-25.2</v>
       </c>
       <c r="G5" t="n">
-        <v>31.6</v>
+        <v>-23.8</v>
       </c>
       <c r="H5" t="n">
-        <v>165.6</v>
+        <v>187.8</v>
       </c>
       <c r="I5" t="s">
         <v>18</v>
       </c>
-      <c r="J5" t="n">
-        <v>24.5</v>
-      </c>
+      <c r="J5"/>
       <c r="K5"/>
       <c r="L5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M5" t="n">
-        <v>2.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46243</v>
+        <v>46248</v>
       </c>
       <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
         <v>23</v>
       </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" t="s">
-        <v>25</v>
-      </c>
       <c r="E6" t="n">
-        <v>-5.3</v>
+        <v>30.2</v>
       </c>
       <c r="F6" t="n">
-        <v>-12.7</v>
+        <v>29.2</v>
       </c>
       <c r="G6" t="n">
-        <v>-4.4</v>
+        <v>10.5</v>
       </c>
       <c r="H6" t="n">
-        <v>166.8</v>
+        <v>181.8</v>
       </c>
       <c r="I6" t="s">
         <v>16</v>
       </c>
-      <c r="J6" t="n">
-        <v>-10.5</v>
-      </c>
+      <c r="J6"/>
       <c r="K6"/>
       <c r="L6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M6" t="n">
-        <v>15.8</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46243</v>
+        <v>46248</v>
       </c>
       <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" t="s">
         <v>23</v>
       </c>
-      <c r="C7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" t="s">
-        <v>25</v>
-      </c>
       <c r="E7" t="n">
-        <v>-5.3</v>
+        <v>30.2</v>
       </c>
       <c r="F7" t="n">
-        <v>-12.7</v>
+        <v>29.2</v>
       </c>
       <c r="G7" t="n">
-        <v>-4.4</v>
+        <v>10.5</v>
       </c>
       <c r="H7" t="n">
-        <v>178.9</v>
+        <v>181.8</v>
       </c>
       <c r="I7" t="s">
         <v>18</v>
       </c>
-      <c r="J7" t="n">
-        <v>-10.5</v>
-      </c>
+      <c r="J7"/>
       <c r="K7"/>
       <c r="L7" t="s">
+        <v>24</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" t="s">
         <v>26</v>
       </c>
-      <c r="M7" t="n">
-        <v>15.8</v>
+      <c r="E8" t="n">
+        <v>9.3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-6.4</v>
+      </c>
+      <c r="G8" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>169.6</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8"/>
+      <c r="K8"/>
+      <c r="L8" t="s">
+        <v>24</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" t="n">
+        <v>9.3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-6.4</v>
+      </c>
+      <c r="G9" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>169.6</v>
+      </c>
+      <c r="I9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9"/>
+      <c r="K9"/>
+      <c r="L9" t="s">
+        <v>24</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-34.4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-40.4</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-30.4</v>
+      </c>
+      <c r="H10" t="n">
+        <v>174.9</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J10"/>
+      <c r="K10"/>
+      <c r="L10" t="s">
+        <v>29</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-34.4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-40.4</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-30.4</v>
+      </c>
+      <c r="H11" t="n">
+        <v>175.1</v>
+      </c>
+      <c r="I11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11"/>
+      <c r="K11"/>
+      <c r="L11" t="s">
+        <v>29</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="G12" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H12" t="n">
+        <v>175.3</v>
+      </c>
+      <c r="I12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J12"/>
+      <c r="K12"/>
+      <c r="L12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" t="n">
+        <v>15</v>
+      </c>
+      <c r="F13" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="G13" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H13" t="n">
+        <v>177.5</v>
+      </c>
+      <c r="I13" t="s">
+        <v>18</v>
+      </c>
+      <c r="J13"/>
+      <c r="K13"/>
+      <c r="L13" t="s">
+        <v>32</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-10.1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-17.5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>168.1</v>
+      </c>
+      <c r="I14" t="s">
+        <v>16</v>
+      </c>
+      <c r="J14" t="n">
+        <v>-22.5</v>
+      </c>
+      <c r="K14" t="n">
+        <v>169.5</v>
+      </c>
+      <c r="L14" t="s">
+        <v>35</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-10.1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-17.5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H15" t="n">
+        <v>168.1</v>
+      </c>
+      <c r="I15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-22.5</v>
+      </c>
+      <c r="K15" t="n">
+        <v>169.5</v>
+      </c>
+      <c r="L15" t="s">
+        <v>35</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="H16" t="n">
+        <v>164.1</v>
+      </c>
+      <c r="I16" t="s">
+        <v>16</v>
+      </c>
+      <c r="J16"/>
+      <c r="K16"/>
+      <c r="L16" t="s">
+        <v>17</v>
+      </c>
+      <c r="M16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B17" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="H17" t="n">
+        <v>167</v>
+      </c>
+      <c r="I17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17"/>
+      <c r="K17"/>
+      <c r="L17" t="s">
+        <v>17</v>
+      </c>
+      <c r="M17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" t="s">
+        <v>39</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-11.4</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="H18" t="n">
+        <v>169.3</v>
+      </c>
+      <c r="I18" t="s">
+        <v>16</v>
+      </c>
+      <c r="J18"/>
+      <c r="K18"/>
+      <c r="L18" t="s">
+        <v>17</v>
+      </c>
+      <c r="M18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-11.4</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="H19" t="n">
+        <v>172.3</v>
+      </c>
+      <c r="I19" t="s">
+        <v>18</v>
+      </c>
+      <c r="J19"/>
+      <c r="K19"/>
+      <c r="L19" t="s">
+        <v>17</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-08-13 16:01:33
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -6,13 +6,13 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="AFL JOINT Projections" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -26,6 +26,12 @@
     <t xml:space="preserve">Away Team</t>
   </si>
   <si>
+    <t xml:space="preserve">Home Team List</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away Team List</t>
+  </si>
+  <si>
     <t xml:space="preserve">Selected / JOINT Home Line</t>
   </si>
   <si>
@@ -53,13 +59,16 @@
     <t xml:space="preserve">Forecast Rain mm</t>
   </si>
   <si>
-    <t xml:space="preserve">12:00</t>
+    <t xml:space="preserve"/>
   </si>
   <si>
     <t xml:space="preserve">essendon</t>
   </si>
   <si>
     <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Previous</t>
   </si>
   <si>
     <t xml:space="preserve">Weather Adjusted</t>
@@ -467,18 +476,20 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="5.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="4.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="22.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="26.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="14.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="15.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="26.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="14.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="16.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="12.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="14.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="16.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="15.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="16.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="12.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="14.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -521,41 +532,53 @@
       <c r="M1" t="s">
         <v>12</v>
       </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
         <v>46248</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" t="n">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="n">
         <v>47.8</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>45.6</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>23.5</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>177.4</v>
       </c>
-      <c r="I2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2"/>
-      <c r="K2"/>
-      <c r="L2" t="s">
-        <v>17</v>
-      </c>
-      <c r="M2" t="n">
+      <c r="K2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2"/>
+      <c r="M2"/>
+      <c r="N2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O2" t="n">
         <v>1.3</v>
       </c>
     </row>
@@ -564,35 +587,41 @@
         <v>46248</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="n">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="n">
         <v>47.8</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>45.6</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>23.5</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
         <v>181</v>
       </c>
-      <c r="I3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J3"/>
-      <c r="K3"/>
-      <c r="L3" t="s">
-        <v>17</v>
-      </c>
-      <c r="M3" t="n">
+      <c r="K3" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3"/>
+      <c r="M3"/>
+      <c r="N3" t="s">
+        <v>20</v>
+      </c>
+      <c r="O3" t="n">
         <v>1.3</v>
       </c>
     </row>
@@ -601,35 +630,41 @@
         <v>46248</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-26.5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-25.2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-23.8</v>
+      </c>
+      <c r="J4" t="n">
+        <v>187.8</v>
+      </c>
+      <c r="K4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" t="n">
-        <v>-26.5</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-25.2</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-23.8</v>
-      </c>
-      <c r="H4" t="n">
-        <v>187.8</v>
-      </c>
-      <c r="I4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J4"/>
-      <c r="K4"/>
-      <c r="L4" t="s">
-        <v>21</v>
-      </c>
-      <c r="M4" t="n">
+      <c r="L4"/>
+      <c r="M4"/>
+      <c r="N4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -638,35 +673,41 @@
         <v>46248</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" t="n">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" t="n">
         <v>-26.5</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>-25.2</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>-23.8</v>
       </c>
-      <c r="H5" t="n">
+      <c r="J5" t="n">
         <v>187.8</v>
       </c>
-      <c r="I5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J5"/>
-      <c r="K5"/>
-      <c r="L5" t="s">
+      <c r="K5" t="s">
         <v>21</v>
       </c>
-      <c r="M5" t="n">
+      <c r="L5"/>
+      <c r="M5"/>
+      <c r="N5" t="s">
+        <v>24</v>
+      </c>
+      <c r="O5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -675,35 +716,41 @@
         <v>46248</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="n">
         <v>30.2</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>29.2</v>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>10.5</v>
       </c>
-      <c r="H6" t="n">
+      <c r="J6" t="n">
         <v>181.8</v>
       </c>
-      <c r="I6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J6"/>
-      <c r="K6"/>
-      <c r="L6" t="s">
-        <v>24</v>
-      </c>
-      <c r="M6" t="n">
+      <c r="K6" t="s">
+        <v>19</v>
+      </c>
+      <c r="L6"/>
+      <c r="M6"/>
+      <c r="N6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" t="n">
         <v>1.3</v>
       </c>
     </row>
@@ -712,35 +759,41 @@
         <v>46248</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" t="n">
+        <v>26</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="n">
         <v>30.2</v>
       </c>
-      <c r="F7" t="n">
+      <c r="H7" t="n">
         <v>29.2</v>
       </c>
-      <c r="G7" t="n">
+      <c r="I7" t="n">
         <v>10.5</v>
       </c>
-      <c r="H7" t="n">
+      <c r="J7" t="n">
         <v>181.8</v>
       </c>
-      <c r="I7" t="s">
-        <v>18</v>
-      </c>
-      <c r="J7"/>
-      <c r="K7"/>
-      <c r="L7" t="s">
-        <v>24</v>
-      </c>
-      <c r="M7" t="n">
+      <c r="K7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L7"/>
+      <c r="M7"/>
+      <c r="N7" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" t="n">
         <v>1.3</v>
       </c>
     </row>
@@ -749,35 +802,41 @@
         <v>46248</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" t="n">
+        <v>29</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" t="n">
         <v>9.3</v>
       </c>
-      <c r="F8" t="n">
+      <c r="H8" t="n">
         <v>-6.4</v>
       </c>
-      <c r="G8" t="n">
+      <c r="I8" t="n">
         <v>19.5</v>
       </c>
-      <c r="H8" t="n">
+      <c r="J8" t="n">
         <v>169.6</v>
       </c>
-      <c r="I8" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8"/>
-      <c r="K8"/>
-      <c r="L8" t="s">
-        <v>24</v>
-      </c>
-      <c r="M8" t="n">
+      <c r="K8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L8"/>
+      <c r="M8"/>
+      <c r="N8" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" t="n">
         <v>1.3</v>
       </c>
     </row>
@@ -786,35 +845,41 @@
         <v>46248</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" t="n">
+        <v>29</v>
+      </c>
+      <c r="E9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" t="n">
         <v>9.3</v>
       </c>
-      <c r="F9" t="n">
+      <c r="H9" t="n">
         <v>-6.4</v>
       </c>
-      <c r="G9" t="n">
+      <c r="I9" t="n">
         <v>19.5</v>
       </c>
-      <c r="H9" t="n">
+      <c r="J9" t="n">
         <v>169.6</v>
       </c>
-      <c r="I9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J9"/>
-      <c r="K9"/>
-      <c r="L9" t="s">
-        <v>24</v>
-      </c>
-      <c r="M9" t="n">
+      <c r="K9" t="s">
+        <v>21</v>
+      </c>
+      <c r="L9"/>
+      <c r="M9"/>
+      <c r="N9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O9" t="n">
         <v>1.3</v>
       </c>
     </row>
@@ -823,35 +888,41 @@
         <v>46248</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" t="n">
+        <v>31</v>
+      </c>
+      <c r="E10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" t="n">
         <v>-34.4</v>
       </c>
-      <c r="F10" t="n">
+      <c r="H10" t="n">
         <v>-40.4</v>
       </c>
-      <c r="G10" t="n">
+      <c r="I10" t="n">
         <v>-30.4</v>
       </c>
-      <c r="H10" t="n">
+      <c r="J10" t="n">
         <v>175.1</v>
       </c>
-      <c r="I10" t="s">
-        <v>16</v>
-      </c>
-      <c r="J10"/>
-      <c r="K10"/>
-      <c r="L10" t="s">
-        <v>29</v>
-      </c>
-      <c r="M10" t="n">
+      <c r="K10" t="s">
+        <v>19</v>
+      </c>
+      <c r="L10"/>
+      <c r="M10"/>
+      <c r="N10" t="s">
+        <v>32</v>
+      </c>
+      <c r="O10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -860,35 +931,41 @@
         <v>46248</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
-      </c>
-      <c r="E11" t="n">
+        <v>31</v>
+      </c>
+      <c r="E11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" t="n">
         <v>-34.4</v>
       </c>
-      <c r="F11" t="n">
+      <c r="H11" t="n">
         <v>-40.4</v>
       </c>
-      <c r="G11" t="n">
+      <c r="I11" t="n">
         <v>-30.4</v>
       </c>
-      <c r="H11" t="n">
+      <c r="J11" t="n">
         <v>175.1</v>
       </c>
-      <c r="I11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J11"/>
-      <c r="K11"/>
-      <c r="L11" t="s">
-        <v>29</v>
-      </c>
-      <c r="M11" t="n">
+      <c r="K11" t="s">
+        <v>21</v>
+      </c>
+      <c r="L11"/>
+      <c r="M11"/>
+      <c r="N11" t="s">
+        <v>32</v>
+      </c>
+      <c r="O11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -897,35 +974,41 @@
         <v>46248</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
-      </c>
-      <c r="E12" t="n">
-        <v>15</v>
-      </c>
-      <c r="F12" t="n">
+        <v>34</v>
+      </c>
+      <c r="E12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" t="n">
+        <v>15</v>
+      </c>
+      <c r="H12" t="n">
         <v>6.7</v>
       </c>
-      <c r="G12" t="n">
+      <c r="I12" t="n">
         <v>10.7</v>
       </c>
-      <c r="H12" t="n">
+      <c r="J12" t="n">
         <v>175.5</v>
       </c>
-      <c r="I12" t="s">
-        <v>16</v>
-      </c>
-      <c r="J12"/>
-      <c r="K12"/>
-      <c r="L12" t="s">
-        <v>32</v>
-      </c>
-      <c r="M12" t="n">
+      <c r="K12" t="s">
+        <v>19</v>
+      </c>
+      <c r="L12"/>
+      <c r="M12"/>
+      <c r="N12" t="s">
+        <v>35</v>
+      </c>
+      <c r="O12" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -934,35 +1017,41 @@
         <v>46248</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C13" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E13" t="n">
-        <v>15</v>
-      </c>
-      <c r="F13" t="n">
+        <v>34</v>
+      </c>
+      <c r="E13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" t="n">
+        <v>15</v>
+      </c>
+      <c r="H13" t="n">
         <v>6.7</v>
       </c>
-      <c r="G13" t="n">
+      <c r="I13" t="n">
         <v>10.7</v>
       </c>
-      <c r="H13" t="n">
+      <c r="J13" t="n">
         <v>177.5</v>
       </c>
-      <c r="I13" t="s">
-        <v>18</v>
-      </c>
-      <c r="J13"/>
-      <c r="K13"/>
-      <c r="L13" t="s">
-        <v>32</v>
-      </c>
-      <c r="M13" t="n">
+      <c r="K13" t="s">
+        <v>21</v>
+      </c>
+      <c r="L13"/>
+      <c r="M13"/>
+      <c r="N13" t="s">
+        <v>35</v>
+      </c>
+      <c r="O13" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -971,39 +1060,45 @@
         <v>46248</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" t="n">
+        <v>37</v>
+      </c>
+      <c r="E14" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" t="n">
         <v>-10.1</v>
       </c>
-      <c r="F14" t="n">
+      <c r="H14" t="n">
         <v>-17.5</v>
       </c>
-      <c r="G14" t="n">
+      <c r="I14" t="n">
         <v>2.6</v>
       </c>
-      <c r="H14" t="n">
+      <c r="J14" t="n">
         <v>168.1</v>
       </c>
-      <c r="I14" t="s">
-        <v>16</v>
-      </c>
-      <c r="J14" t="n">
+      <c r="K14" t="s">
+        <v>19</v>
+      </c>
+      <c r="L14" t="n">
         <v>-17.5</v>
       </c>
-      <c r="K14" t="n">
+      <c r="M14" t="n">
         <v>170.5</v>
       </c>
-      <c r="L14" t="s">
-        <v>35</v>
-      </c>
-      <c r="M14" t="n">
+      <c r="N14" t="s">
+        <v>38</v>
+      </c>
+      <c r="O14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1012,39 +1107,45 @@
         <v>46248</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D15" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" t="n">
+        <v>37</v>
+      </c>
+      <c r="E15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" t="n">
         <v>-10.1</v>
       </c>
-      <c r="F15" t="n">
+      <c r="H15" t="n">
         <v>-17.5</v>
       </c>
-      <c r="G15" t="n">
+      <c r="I15" t="n">
         <v>2.6</v>
       </c>
-      <c r="H15" t="n">
+      <c r="J15" t="n">
         <v>168.1</v>
       </c>
-      <c r="I15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J15" t="n">
+      <c r="K15" t="s">
+        <v>21</v>
+      </c>
+      <c r="L15" t="n">
         <v>-17.5</v>
       </c>
-      <c r="K15" t="n">
+      <c r="M15" t="n">
         <v>170.5</v>
       </c>
-      <c r="L15" t="s">
-        <v>35</v>
-      </c>
-      <c r="M15" t="n">
+      <c r="N15" t="s">
+        <v>38</v>
+      </c>
+      <c r="O15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1053,35 +1154,41 @@
         <v>46248</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D16" t="s">
-        <v>37</v>
-      </c>
-      <c r="E16" t="n">
+        <v>40</v>
+      </c>
+      <c r="E16" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" t="n">
         <v>23.1</v>
       </c>
-      <c r="F16" t="n">
+      <c r="H16" t="n">
         <v>28.6</v>
       </c>
-      <c r="G16" t="n">
+      <c r="I16" t="n">
         <v>16.3</v>
       </c>
-      <c r="H16" t="n">
+      <c r="J16" t="n">
         <v>163.5</v>
       </c>
-      <c r="I16" t="s">
-        <v>16</v>
-      </c>
-      <c r="J16"/>
-      <c r="K16"/>
-      <c r="L16" t="s">
-        <v>17</v>
-      </c>
-      <c r="M16" t="n">
+      <c r="K16" t="s">
+        <v>19</v>
+      </c>
+      <c r="L16"/>
+      <c r="M16"/>
+      <c r="N16" t="s">
+        <v>20</v>
+      </c>
+      <c r="O16" t="n">
         <v>1.3</v>
       </c>
     </row>
@@ -1090,35 +1197,41 @@
         <v>46248</v>
       </c>
       <c r="B17" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C17" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" t="n">
+        <v>40</v>
+      </c>
+      <c r="E17" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" t="s">
+        <v>18</v>
+      </c>
+      <c r="G17" t="n">
         <v>23.1</v>
       </c>
-      <c r="F17" t="n">
+      <c r="H17" t="n">
         <v>28.6</v>
       </c>
-      <c r="G17" t="n">
+      <c r="I17" t="n">
         <v>16.3</v>
       </c>
-      <c r="H17" t="n">
+      <c r="J17" t="n">
         <v>167</v>
       </c>
-      <c r="I17" t="s">
-        <v>18</v>
-      </c>
-      <c r="J17"/>
-      <c r="K17"/>
-      <c r="L17" t="s">
-        <v>17</v>
-      </c>
-      <c r="M17" t="n">
+      <c r="K17" t="s">
+        <v>21</v>
+      </c>
+      <c r="L17"/>
+      <c r="M17"/>
+      <c r="N17" t="s">
+        <v>20</v>
+      </c>
+      <c r="O17" t="n">
         <v>1.3</v>
       </c>
     </row>
@@ -1127,35 +1240,41 @@
         <v>46248</v>
       </c>
       <c r="B18" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D18" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" t="n">
+        <v>42</v>
+      </c>
+      <c r="E18" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" t="n">
         <v>-5.6</v>
       </c>
-      <c r="F18" t="n">
+      <c r="H18" t="n">
         <v>-11.4</v>
       </c>
-      <c r="G18" t="n">
+      <c r="I18" t="n">
         <v>-4.8</v>
       </c>
-      <c r="H18" t="n">
+      <c r="J18" t="n">
         <v>168.7</v>
       </c>
-      <c r="I18" t="s">
-        <v>16</v>
-      </c>
-      <c r="J18"/>
-      <c r="K18"/>
-      <c r="L18" t="s">
-        <v>17</v>
-      </c>
-      <c r="M18" t="n">
+      <c r="K18" t="s">
+        <v>19</v>
+      </c>
+      <c r="L18"/>
+      <c r="M18"/>
+      <c r="N18" t="s">
+        <v>20</v>
+      </c>
+      <c r="O18" t="n">
         <v>1.3</v>
       </c>
     </row>
@@ -1164,35 +1283,41 @@
         <v>46248</v>
       </c>
       <c r="B19" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D19" t="s">
-        <v>39</v>
-      </c>
-      <c r="E19" t="n">
+        <v>42</v>
+      </c>
+      <c r="E19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" t="n">
         <v>-5.6</v>
       </c>
-      <c r="F19" t="n">
+      <c r="H19" t="n">
         <v>-11.4</v>
       </c>
-      <c r="G19" t="n">
+      <c r="I19" t="n">
         <v>-4.8</v>
       </c>
-      <c r="H19" t="n">
+      <c r="J19" t="n">
         <v>172.3</v>
       </c>
-      <c r="I19" t="s">
-        <v>18</v>
-      </c>
-      <c r="J19"/>
-      <c r="K19"/>
-      <c r="L19" t="s">
-        <v>17</v>
-      </c>
-      <c r="M19" t="n">
+      <c r="K19" t="s">
+        <v>21</v>
+      </c>
+      <c r="L19"/>
+      <c r="M19"/>
+      <c r="N19" t="s">
+        <v>20</v>
+      </c>
+      <c r="O19" t="n">
         <v>1.3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update model outputs 2026-08-13 16:11:36
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -573,8 +573,12 @@
       <c r="K2" t="s">
         <v>19</v>
       </c>
-      <c r="L2"/>
-      <c r="M2"/>
+      <c r="L2" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="M2" t="n">
+        <v>184.5</v>
+      </c>
       <c r="N2" t="s">
         <v>20</v>
       </c>
@@ -616,8 +620,12 @@
       <c r="K3" t="s">
         <v>21</v>
       </c>
-      <c r="L3"/>
-      <c r="M3"/>
+      <c r="L3" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="M3" t="n">
+        <v>184.5</v>
+      </c>
       <c r="N3" t="s">
         <v>20</v>
       </c>
@@ -659,8 +667,12 @@
       <c r="K4" t="s">
         <v>19</v>
       </c>
-      <c r="L4"/>
-      <c r="M4"/>
+      <c r="L4" t="n">
+        <v>-32.5</v>
+      </c>
+      <c r="M4" t="n">
+        <v>188.5</v>
+      </c>
       <c r="N4" t="s">
         <v>24</v>
       </c>
@@ -702,8 +714,12 @@
       <c r="K5" t="s">
         <v>21</v>
       </c>
-      <c r="L5"/>
-      <c r="M5"/>
+      <c r="L5" t="n">
+        <v>-32.5</v>
+      </c>
+      <c r="M5" t="n">
+        <v>188.5</v>
+      </c>
       <c r="N5" t="s">
         <v>24</v>
       </c>
@@ -745,8 +761,12 @@
       <c r="K6" t="s">
         <v>19</v>
       </c>
-      <c r="L6"/>
-      <c r="M6"/>
+      <c r="L6" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="M6" t="n">
+        <v>183.5</v>
+      </c>
       <c r="N6" t="s">
         <v>27</v>
       </c>
@@ -788,8 +808,12 @@
       <c r="K7" t="s">
         <v>21</v>
       </c>
-      <c r="L7"/>
-      <c r="M7"/>
+      <c r="L7" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="M7" t="n">
+        <v>183.5</v>
+      </c>
       <c r="N7" t="s">
         <v>27</v>
       </c>
@@ -831,8 +855,12 @@
       <c r="K8" t="s">
         <v>19</v>
       </c>
-      <c r="L8"/>
-      <c r="M8"/>
+      <c r="L8" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="M8" t="n">
+        <v>175.5</v>
+      </c>
       <c r="N8" t="s">
         <v>27</v>
       </c>
@@ -874,8 +902,12 @@
       <c r="K9" t="s">
         <v>21</v>
       </c>
-      <c r="L9"/>
-      <c r="M9"/>
+      <c r="L9" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="M9" t="n">
+        <v>175.5</v>
+      </c>
       <c r="N9" t="s">
         <v>27</v>
       </c>
@@ -917,8 +949,12 @@
       <c r="K10" t="s">
         <v>19</v>
       </c>
-      <c r="L10"/>
-      <c r="M10"/>
+      <c r="L10" t="n">
+        <v>-32.5</v>
+      </c>
+      <c r="M10" t="n">
+        <v>168.5</v>
+      </c>
       <c r="N10" t="s">
         <v>32</v>
       </c>
@@ -960,8 +996,12 @@
       <c r="K11" t="s">
         <v>21</v>
       </c>
-      <c r="L11"/>
-      <c r="M11"/>
+      <c r="L11" t="n">
+        <v>-32.5</v>
+      </c>
+      <c r="M11" t="n">
+        <v>168.5</v>
+      </c>
       <c r="N11" t="s">
         <v>32</v>
       </c>
@@ -1003,8 +1043,12 @@
       <c r="K12" t="s">
         <v>19</v>
       </c>
-      <c r="L12"/>
-      <c r="M12"/>
+      <c r="L12" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="M12" t="n">
+        <v>182.5</v>
+      </c>
       <c r="N12" t="s">
         <v>35</v>
       </c>
@@ -1046,8 +1090,12 @@
       <c r="K13" t="s">
         <v>21</v>
       </c>
-      <c r="L13"/>
-      <c r="M13"/>
+      <c r="L13" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="M13" t="n">
+        <v>182.5</v>
+      </c>
       <c r="N13" t="s">
         <v>35</v>
       </c>
@@ -1183,8 +1231,12 @@
       <c r="K16" t="s">
         <v>19</v>
       </c>
-      <c r="L16"/>
-      <c r="M16"/>
+      <c r="L16" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="M16" t="n">
+        <v>167.5</v>
+      </c>
       <c r="N16" t="s">
         <v>20</v>
       </c>
@@ -1226,8 +1278,12 @@
       <c r="K17" t="s">
         <v>21</v>
       </c>
-      <c r="L17"/>
-      <c r="M17"/>
+      <c r="L17" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="M17" t="n">
+        <v>167.5</v>
+      </c>
       <c r="N17" t="s">
         <v>20</v>
       </c>
@@ -1269,8 +1325,12 @@
       <c r="K18" t="s">
         <v>19</v>
       </c>
-      <c r="L18"/>
-      <c r="M18"/>
+      <c r="L18" t="n">
+        <v>-19.5</v>
+      </c>
+      <c r="M18" t="n">
+        <v>174.5</v>
+      </c>
       <c r="N18" t="s">
         <v>20</v>
       </c>
@@ -1312,8 +1372,12 @@
       <c r="K19" t="s">
         <v>21</v>
       </c>
-      <c r="L19"/>
-      <c r="M19"/>
+      <c r="L19" t="n">
+        <v>-19.5</v>
+      </c>
+      <c r="M19" t="n">
+        <v>174.5</v>
+      </c>
       <c r="N19" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
Update model outputs 2026-09-12 21:25:57
</commit_message>
<xml_diff>
--- a/files/AFL_upcoming_projections.xlsx
+++ b/files/AFL_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -62,10 +62,10 @@
     <t xml:space="preserve"/>
   </si>
   <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
   </si>
   <si>
     <t xml:space="preserve">Previous</t>
@@ -74,19 +74,10 @@
     <t xml:space="preserve">Weather Adjusted</t>
   </si>
   <si>
-    <t xml:space="preserve">Optus Stadium</t>
+    <t xml:space="preserve">Gabba</t>
   </si>
   <si>
     <t xml:space="preserve">No Rain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gabba</t>
   </si>
 </sst>
 </file>
@@ -434,7 +425,7 @@
     <col min="11" max="11" width="16.71" hidden="0" customWidth="1"/>
     <col min="12" max="12" width="11.71" hidden="0" customWidth="1"/>
     <col min="13" max="13" width="12.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="13.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="5.71" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
@@ -487,7 +478,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B2" t="s">
         <v>15</v>
@@ -505,36 +496,36 @@
         <v>18</v>
       </c>
       <c r="G2" t="n">
-        <v>-3.3</v>
+        <v>-14.4</v>
       </c>
       <c r="H2" t="n">
-        <v>-6.3</v>
+        <v>-12.5</v>
       </c>
       <c r="I2" t="n">
-        <v>2.7</v>
+        <v>-15.6</v>
       </c>
       <c r="J2" t="n">
-        <v>180.8</v>
+        <v>184.3</v>
       </c>
       <c r="K2" t="s">
         <v>19</v>
       </c>
       <c r="L2" t="n">
-        <v>-10.5</v>
+        <v>-21.5</v>
       </c>
       <c r="M2" t="n">
-        <v>173.5</v>
+        <v>179.5</v>
       </c>
       <c r="N2" t="s">
         <v>20</v>
       </c>
       <c r="O2" t="n">
-        <v>0.1</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
@@ -552,124 +543,30 @@
         <v>18</v>
       </c>
       <c r="G3" t="n">
-        <v>-3.3</v>
+        <v>-14.4</v>
       </c>
       <c r="H3" t="n">
-        <v>-6.3</v>
+        <v>-12.5</v>
       </c>
       <c r="I3" t="n">
-        <v>2.7</v>
+        <v>-15.6</v>
       </c>
       <c r="J3" t="n">
-        <v>181.1</v>
+        <v>189.9</v>
       </c>
       <c r="K3" t="s">
         <v>21</v>
       </c>
       <c r="L3" t="n">
-        <v>-10.5</v>
+        <v>-21.5</v>
       </c>
       <c r="M3" t="n">
-        <v>173.5</v>
+        <v>179.5</v>
       </c>
       <c r="N3" t="s">
         <v>20</v>
       </c>
       <c r="O3" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>46277</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-14.4</v>
-      </c>
-      <c r="H4" t="n">
-        <v>-12.5</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-15.6</v>
-      </c>
-      <c r="J4" t="n">
-        <v>184.3</v>
-      </c>
-      <c r="K4" t="s">
-        <v>19</v>
-      </c>
-      <c r="L4" t="n">
-        <v>-21.5</v>
-      </c>
-      <c r="M4" t="n">
-        <v>179.5</v>
-      </c>
-      <c r="N4" t="s">
-        <v>24</v>
-      </c>
-      <c r="O4" t="n">
-        <v>2.7</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>46277</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" t="n">
-        <v>-14.4</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-12.5</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-15.6</v>
-      </c>
-      <c r="J5" t="n">
-        <v>189.9</v>
-      </c>
-      <c r="K5" t="s">
-        <v>21</v>
-      </c>
-      <c r="L5" t="n">
-        <v>-21.5</v>
-      </c>
-      <c r="M5" t="n">
-        <v>179.5</v>
-      </c>
-      <c r="N5" t="s">
-        <v>24</v>
-      </c>
-      <c r="O5" t="n">
         <v>2.7</v>
       </c>
     </row>

</xml_diff>